<commit_message>
Update LDA analysis outputs and scripts
</commit_message>
<xml_diff>
--- a/result/Eng_cutted.xlsx
+++ b/result/Eng_cutted.xlsx
@@ -425,36 +425,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>filename</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>filename</t>
+          <t>content</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>content_cutted</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>伊利诺伊大学香槟分校 ‌ 信息科学职业资源.doc</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
-        <is>
-          <t>伊利诺伊大学香槟分校 ‌ 信息科学职业资源.doc</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
         <is>
           <t>Careers in Information Sciences: Job Searching and Beyond
 This page highlights resources for job seekers in the information sciences and information management and for those looking for professional development in their careers. Those looking for information on informational interviews, mentoring, or other career-related information beyond those listed here should consult the Careers page of the iSchool.
@@ -512,22 +509,19 @@
 You can use this list on Wikipedia to identify gaming conventions or conferences to attend in your location.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>career information science job highlight material job seeker information science information management growth career information interview information career ischool career information publishing job list survey trend statistic article book growth topic game job list job aggregator position announcement database job link information resume salary library association career material job posting association library member bank information residency diversity program chronicle education job database browse job tool resumescover letter job alert online submission account higheredjobs database list job education search category library association jobline job listing library inalj job job posting job material bank career community job feature job seeker career profile interview partnership job board job board job canada rail job board list job illinois listing state career ischool list job list option survey statistic profession people job market career path survey sense expectation job offer survey source data gender representation position survey report statistic survey career library data health law library survey workplace survey data library survey position master degree alaapa survey position master print library statistic version position version bureau labor statistic outlook guide government publication profile path income requirement information section computer information technology education training occupation journal placement salary survey journal report table placement survey articleoften article title survey report example october issue report title report information job title distribution placement job type salary book article growth topic database catalog date field specialty material growth term article liss body trade magazine database search term job description job qualification topic trend job requirement position job market field print ebooks catalog topic information date publication library congress guidance field term try information science guidance game list material career game game developer site art business game industry news job posting link company business institution gdc game developer conference game design portfolio article portfolio advice career portfolio industry reputation employer game developer igda membership institution individual video game site element material library career center list convention list wikipedia convention conference location</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>career science job_searching highlight resource job seeker science professional career informational interview mentor career relate list consult career ischool related career researching publishing job post list salary survey related professional trend statistic article book professional topic game job post list find job aggregator position announcement ala joblist searchable database job resume salary interview sponsor american library association career resource job posting association library member libraries resume bank residency diversity chronicle higher_education job database browse category job tool save resume resume resume job alert application free account higheredjobs database contain comprehensive list library job higher_education category administrative library illinois library association jobline job listing library illinois inalj library job comprehensive international job posting update weekly job hunt resource resume bank career community list job extra feature job seeker career resume interview tip partnership job board comprehensive job board library job canada rail job board rail host list library job illinois occasional listing surround state ischool career ischool expansive list job list option salary survey related statistic profession job_market interested particular career path salary survey sense realistic expectation negotiate job survey best data gender ethnic representation professional position arl annual salary survey report statistic base survey professional library report separate data health law library sla annual salary survey workplace salary survey data special library ala salary survey position require master degree ala apa salary survey position require ala accredit master degree print include academic library statistic version position require run last version bureau labor statistic occupational outlook handbook government article resume career path tell median income educational requirement related section computer technology education training library job library article annual placement salary survey october library article include report basic statistical table annual placement salary survey graduate browse little find article article thematic title indicate survey report october issue report title emerge databrarian report full unique emerge job title distribution placement job start salary book article professional topic database library catalog stay field specialty resource focus professional assign specific subject term article liss significant body trade magazine include database try term job description job qualification librarians employment article topic trend job requirement particular position want consult job_market want know skills develop particular field print ebooks library catalog topic want recent sure sort article attach library congress sub head vocational guidance different field main subject term try science vocational guidance game brief list resource career game design game developer dedicate art business game contain late industry job posting top company business organization host annual gdc game developer conference build game design portfolio article portfolio advice game professional portfolio allow build industry reputation promote prospective employer international game developer association igda large non profit membership organization serve video game useful element include resource library career list game related convention list wikipedia identify game convention conference attend</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>伊利诺伊大学香槟分校 ‌ 职业角.doc</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
-        <is>
-          <t>伊利诺伊大学香槟分校 ‌ 职业角.doc</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
         <is>
           <t>Career Corner
 Information about getting started with your career. For current and former undergraduate and graduate students.
@@ -681,22 +675,19 @@
 Free Job Boards and Databases</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>career corner information career undergraduate graduate student welcome career corner regardless area job task guide importance understanding information company industry employer job candidate understanding curiosity work company industry guide company industry question job interview thing webpage database guide student staff faculty student staff faculty access university netid password description highlight material effort information material company career reason time company representative youre position youll company interview company question job helpful company history stability product service personnel information company culture youre candidate position specific company goal mission product policy company culture hiring manager interest position ability role company sense industry example job mortgage company instance helpful homeownership trend feel company competitor success flaw company industry rival interviewer company company source information company axle company company data video privco article business business source nexis company chart challenging database search material feature database chart database feature database database netid password youre trouble database error code try link incognito window assistance contact company database overview business source text content indexing abstract business journal text journal article discipline business marketing management pom accounting finance database text content data book reference work book conference proceeding investment report industry report market report country report company analysis data company batch material user business record consumer record business record variety factor custom list chart heat map database market mapping project activity trend emis material information market content news article statement company information industry equity quote statistic marketspecific information publication feature news business source court decision news business information company state law regulation privco business data nonpublicly corporation family equity venture company data company market deal venture capital funding market market investor keyword industry access university illinois user account sign university email address search company top click company menu search right screen business database data privatelyheld company financials revenue deal multiple valuation equity deal history family ownership data user account university email address access database statista access statistic market researcher institution publication government source industry information glassdoor insider information salary employee interview interview question image source httpsmediaglassdoorcombrandlogogreenstackedlogoglassdoorlogopng vault company information culture reputation subscription access engineering career service industry industry information chart challenging database search material feature database chart database feature database database netid password internship material student profile search internship job position location incl campus company host event career fair student platform view employer image source httpsacesillinoisedusitesacesillinoisedufileslegacy_bloghandshakelogocroppedjpg summer chance office database summer chance student chance student database business chance business economics area menu keyword search database posting thousand job board career site internet handshake link website profile internlist repository material seeker profile resume interview sponsor information october note lapse funding government work stoppage labor certification program website update office labor certification department labor labor submission material time alert date change program proclamation visa quota update government work stoppage program site funding information visa specialty operation job program status citizenship immigration service specialty occupation site site eligibility criterion information visa apply visa department labor program site news guidance form link program department labor onestop shop visa material metric immigration council fact sheet overview visa category petition myth impact visa worker immigration council advocate advocacy agency program contains material immigrant visa sponsor database visa sponsor employer data hub map employer citizenship immigration service year data company petition worker city state zip code employer year naics code data excel csv instruction data center job list company labor condition submission evidence visa petition downloadable access format site lapse funding myvisajobscom list company institution people card visa metric people information worker protection information job board visa job posting employer employee job posting candidate letter resume letter cover letter book james innes letter louise element style scott bennett job search experience job search kat mckay writing book element style strunk book royal place resume cover letter note graduate student work student hour appointment people question video tip answer question interview information skill question interviewer question industry question question interviewer material student strategy company industry turn question knowledge industry company interest ibisworld industry top industry information salarycost allowance salarycom bell curve distribution income job title zip code data cover bonus benefit people company bureau labor statistic branch department labor job wage estimate occupation state metropolitan job wage university guide list faculty staff salary illini cupahrs data data finding faculty survey cupa member education material department instituions institution master institution bachelor institution institution company company database location company information company company country industry geolocation coordinate parent subsidiary location company location user guide instruction database export result form job posting student alumnus material job board office student aid job board student work university department designation job search preference notification posting work position login job board job student job library job position undergraduate graduate student box position student status student career faculty service position student position student clearinghouse graduate student experience illinois assistantship clearinghouse graduate assistantships stipend tuition waiver housing chance position basis note student assistantships assistantships department exploration college business compiles material business student job posting posting career growth tool student login material graduation coursework growth job posting material nonstudents job illinois material job seeker staff faculty job posting employee access job posting material job seeker user illinois career site user profile job city date job category type position city champaign job job board city view position job interest form opening preference user government job city job chance job board city view position service position government user email account news gazette classified classified job posting news gazette job champaign danville illinois submission news gazette job board database</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>career corner start career former undergraduate graduate student welcome career corner regardless academic area job entail task common guide emphasize importance gain understanding company apply industry operate interview employer expect job candidate demonstrate understanding curiosity job company broad industry guide equip company industry assist formulate take job interview begin mention database guide student staff faculty student staff faculty try university databases netid password require description contain elementary highlight material effort take try include material accessible company accord balance career various reason spend little company interview representative apply position want find company sit interview know company feel comfortable able ask show interested job helpful company history financial stability product personnel company culture fit hire prepared candidate position know specific company goal mission product policy company culture impress hiring manager keen interest position ability assimilate productive work company sense examine overall industry interview job mortgage company instance helpful inform homeownership trend feel company big competitor identify success flaw company industry rival bind impress interviewer company company consult company data axle company company list data tutorial video privco check article databases proquest business business ultimate nexis university company chart sometimes challenge right database start resource hard remember feature various database chart include subscribed key database various feature database database netid password trouble database error code try incognito assistance contact library illinois company database overview business ultimate bibliographic full text content include indexing abstract scholarly business article full text article article discipline business include marketing pom accounting finance economics database full text content include financial data book monographs major job book digest conference proceeding investment report industry report report country report company resume swot analysis data company batch resource connect business record record historical business record demographic factor custom list excel render graphs chart heat map database ideal entrepreneurial plan mapping project job seek activity gauge economic trend emis resource deliver hard emerge aggregate produce unique content include full text article financial statement company industry analyse equity quote macroeconomic statistic specific derive local global article nexus university feature business legal include supreme court decision include business company directories federal state law regulation legal privco business financial data major non trade corporation include family equity venture back international unlisted company contain data company deal venture finance funding investor keyword industry free university illinois urbana champaign account sign university mail address main company top company dropdown right screen proquest business database financial data major hold company include finance revenue deal deal multiple firm valuation fund equity deal history family ownership data note account university illinois address database statista statistic gather researcher trade organization scientific article government industry insider glassdoor free great insider include salary employee interview real interview image medium glassdoor brand logo green stack logo glassdoor logo png firsthand vault company insider company culture reputation subscription require engineering career_services industry industry chart sometimes challenge right database start resource hard remember feature various database chart include subscribed key database various feature database database netid password internship free job salary resource handshake similar linkedin uiuc student complete resume internship full job position incl company handshake host event include virtual career fair allow student sign platform employer attendance image ace illinois ace illinois file legacy_blog handshake logo crop jpg summer undergraduate database maintain illinois office undergraduate database summer undergraduate student domestic international international student database business business economics area keyword recommend intern list database aggregate internship posting job board career internet include linkedin handshake glassdoor external resume apply intern list wide repository resource internship seeker build resume resume prepare interview visa sponsor visa october note due lapse funding government job stoppage foreign labor certification federal update suspend include office foreign labor certification uscis department labor foreign labor application resource include describe disable federal remain active include alert last update change recent federal proclamation include visa quota federal update resume government job stoppage cease reactivate federal funding restore visa specialty operation employment federal status citizenship immigration specialty job federal uscis contain eligibility criterion relate obtain visa apply visa uscis department labor guidance related department labor stop shop visa material metric american immigration council visa fact sheet overview visa category petition myth impact visa worker american immigration council non profit advocate immigrant advocacy federal agency visa contain helpful resource immigrant find visa sponsor free database visa sponsor employer data hub interactive map employer citizenship immigration include data company submit petition employ worker filter city state zip code employer fiscal naics code data downloadable excel csv include instruction flc data job long list company file labor application evidence visa petition downloadable format disabled due lapse federal funding myvisajobs list company institution hire green card visa relevant metric include rank hire salary include worker protection legal bvisajobs specific job board visa job posting employer sponsor employee submit job posting browse candidate resume resume resume resume resume resume write resume resume book james innes resume resume magic wendy enelow louise kursmark element resume style scott bennett job_search steven experience job_search kat mckay writing book element style william strunk white little red write book brandon royal write write excellent resume resume resume note graduate student job graduate student appointment interview answer watch video tip best answer interview continue scroll skill develop ask interviewer ask ask industry specific prepare ask interviewer resource uiuc student outline strategy company industry turn assist craft broaden knowledge industry company professional interest ibisworld industry top industry salary salary cost live allowance salary display bell curve distribution income job title particular zip code data resume base salary bonus benefit job company bureau labor statistic branch department labor employment wage estimate job include national state metropolitan nonmetropolitan employment wage estimate university illinois salary guide list faculty staff salary daily illini cupa salary data salary data base finding cupa annual national faculty salary survey cupa member higher_education human resource department large academic instituions doctoral institution master institution bachelor institution specialized institution best company list best company list uniworld database contain company multinational company represent company country industry geolocation coordinate parent subsidiary find large profitable relevant company desired uniworld guide instruction database export result different job posting student alumni student resource virtual job board office student financial aid virtual job board student find job university department designation save job_search preference sign notification posting find job eligible position valid require virtual job board library employment student interested employment uiuc library visit library employment find position undergraduate graduate student label graduate undergraduate extra find position respective student status student active apply note academic academic professional faculty civil position enrolled student graduate assistant position mslis student assistantship clearinghouse graduate student pre professional experience illinois check assistantship clearinghouse least semi graduate assistantships come stipend tuition waiver come housing assistantship position post rolling basis note graduate student eligible assistantships assistantships distribute academic department career exploration university business compiles career resource business student include job posting internship posting career_development tool limit student active resource helpful graduation shape coursework pre professional local job posting human_resources alumni non student job illinois explore human resource job seeker find staff faculty temporary job posting employee job posting human_resources job seeker take illinois career resume apply job city post job category position city champaign job job post board city champaign position fill job interest notify opening fit preference government job apply city urbana job_opportunities job post board city urbana position include civil position urbana government active account apply gazette classified check classified job posting gazette find local job champaign urbana danville east central illinois application external gazette free job board database</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>俄亥俄州立大学 通用型.doc</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
-        <is>
-          <t>俄亥俄州立大学 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
         <is>
           <t>Career Development Success
 Home
@@ -745,22 +736,19 @@
 Succeeding in Practice</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>career growth success home introduction guide overview career material moritz law library material stage job search experience area position material student career growth intranet career growth office student career advice career growth office student job fit assessment career option training job search skill source job chance employer directory directory leadership book database information law firm office government agency level contact information content varies community martindalehubbell directory attorney law firm experience area location alma mater content varies profile directory employer association law placement information law firm government agency interest institution corporation lawyer demographic experience area compensation benefit search location firm size experience area account email address directory judiciary almanac judiciary allows judge district court address profile sketch ruling evaluation lawyer disclosure report ballotpedia ballotpedia state judge court state profile information judge career election nomination state county judge directory article judge directory background judge courtlistener database courtlisteners database information onthousands judge state court biographical background position affiliation bar association rating campaign finance data opinion profile analytics litigation analyticsmoritz law user litigation analytics attorney law firm company addition analytics docket link individual institution information profile career history link court opinion news analytics motion outcome length solutionsmoritz law user solution intelligence provider career tool business strategy chance industry access user reference team lexis contextmoritz law user allows attorney judge court company expert area expertise profile information select contact information analytics litigation analyticsmoritz law user litigation analytics insight attorney law firm judge court company area expertise industry profile insight experience ruling tendency westlaw profilermoritz law user profiler attorney judge arbitrator career institution court area profile information contact information analytics profile reference source state county judge search alumnus college law search term tutorial howto guide law guidance litigation analytics employer video lexis support training westlaw reference guide litigation analytics job search tip summer job success experience area experience</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>career_development success introduction guide selective overview career resource moritz law library find resource job_search practice area interview settle position resource specific moritz student consult career_development intranet career_development office encourage moritz student seek career advice contact career_development office commit student find best job fit possible individualize self assessment identify appropriate legal career option training job_search skill employment employer leadership connect know yellow book database law firm judicial office government agency include contact biographical content varies community martindale hubbell martindale hubbell legal allow attorney law firm practice area alma mater content varies resume legal employer national association law placement specific law firm government agency interest organization corporation include lawyer demographic practice area compensation benefit firm practice area free account enter address judicial federal judiciary almanac federal judiciary allows federal judge district court address resume biographical sketch noteworthy ruling anonymous evaluation lawyer financial disclosure report ballotpedia ballotpedia allow federal state judge court state resume include judge education career election nomination state county judge include biographical article iii federal judge present searchable contain educational professional background federal judge present courtlistener judicial database courtlistener database onthousands judge federal state court include biographical educational background judicial non judicial position hold political affiliation american bar association rating campaign finance data opinion author resume analytics bloomberg litigation analyticsmoritz law bloomberg litigation analytics allow attorney law firm company addition analytics docket bloomberg organization contain biographical contact judicial resume include career history cited court opinion recent analytics motion outcome appeal length leopard solutionsmoritz law leopard solution leading legal intelligence provider professional seek sophisticated tool business strategy recruit legal industry restrict moritz contact username password lexis contextmoritz law lexis context allows attorney judge court company expert area expertise resume include biographical contact analytics westlaw litigation analyticsmoritz law westlaw litigation analytics data insight attorney law firm judge court company area expertise industry resume include insight experience ruling tendency westlaw profilermoritz law westlaw profiler allow attorney judge arbitrator professional organization court geographic area resume include biographical contact analytics judicial resume include list secondary state county judge include narrow moritz alumnus include moritz university law key term tutorial guide bloomberg law practical guidance litigation analytics lexis potential employer youtube video lexis context support training westlaw quick guide understand litigation analytics job_search tip summer job success practice area succeed practice</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>利亚桑那州立大学 通用型.doc</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>利亚桑那州立大学 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
         <is>
           <t>Career Resources for Students
 Campus Career Resources
@@ -820,22 +808,19 @@
 The Consumer Price Index (CPI) is a measure of the average change over time in the prices paid by urban consumers for a market basket of consumer goods and services. Indexes are available for the U.S. and various geographic areas. Average price data for select utility, automotive fuel, and food items are also available.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>career material student career material student career growth student career growth secd campus graduate life chance purpose value student material support student job fulltime job search job internship connection careerreadiness skill place way employer career onestop department labor career tool job seeker student business career career site salary compensation data company culture rating comparison industry career community woman job advice support membership glassdoor student employer company information interview experience workplace insight employee networking site student company job posting employee career path outlook career outlook material outlook material website publication information future job career field thing growth demand salary skill industry student job seeker people career change onet database information skill work activity job outlook department labor offer exploration industry data training material move tool student search career keyword industry interest link data job wage statistic bls material wage job trend occupation bureau labor statistic outlook guide career material information job duty education requirement range job outlook hundred occupation interview boundforcareer boundforcareer guidebook adolescent adult career growth guidance exploration decisionmaking workplace transition myth question reader control career journey interview secret interview secret instruction job interview worldthe interview victor mckinsey management consultant insider interview confidence intelligence series work intelligence selfdoubt manage imposter syndrome guidance insight expert harvard business intelligence series job job student graduate job search confidence guidance strength interview offer job interview identity book job seeker interview success interview confidence employer strategy competency bias confidence job offer cost cost living mylifeelsewhere country area grocery transportation wallet cost calculator cost city cost salaryexperts cost data expenditure component housing consumables transportation health care income payroll tax bureau labor statistic consumer price index consumer price index cpi measure change time price consumer market basket consumer good service index area price data utility fuel food item</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>career resource student career resource student engagement career_development student engagement career_development secd inspire prepare graduate life align purpose value undergraduate student find resource support prepare internships student employment full job apply employment internship experiential connection build career readiness skill job potential employer career onestop sponsor department labor career tool job seeker student business career professional highlight salary compensation data company culture rating comparison industry fairygodboss join large career community woman find job advice support membership free glassdoor glassdoor student employer company salary interview experience workplace insight former employee linkedin professional networking student explore company job posting employee career path career outlook career outlook resource career outlook resource tools article give future job career field project growth demand typical salary skill industry hire useful student job seeker consider career change net comprehensive database occupational include skill job activity job outlook careeronestop department labor career exploration industry outlooks salary data training resource next move interactive tool student career keyword industry personal interest net data occupational employment wage statistic bls resource focus wage employment trend job bureau labor statistic occupational outlook handbook comprehensive career resource detailed job duty education requirement salary_ranges employment outlook job prepare interview bound career guidebook bound career guidebook adolescent young adult navigate career_development guidance exploration decision making workplace transition dispel myth answer common empower take control career journey interview secret interview secret discover instruction dominate consider complex difficult intimidating corporate job interview infamous interview victor cheng former mckinsey consultant reveal proven insider method ace interview confidence hbr emotional intelligence confident job emotional intelligence overcome doubt manage imposter syndrome communicate practical guidance insight lead expert harvard business hbr emotional intelligence job job student recent graduate navigate job_search confidence guidance identify strength network interviewing evaluate land job interview identity book job seeker improve interview success identify interview identity base confidence experience teach employer perceive strategy communicate competency reduce bias build confidence increase job regional cost live cost living mylifeelsewhere allow compare cost live country resume area din grocery transportation nerd wallet cost live calculator compare cost live city salaryexpert cost live eri salaryexpert cost live data calculate main expenditure component housing consumables transportation health care income payroll tax bureau labor statistic price price cpi measure average change price pay urban basket good various geographic area average price data utility automotive fuel food item</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>加州大学圣地亚哥分校  职业指南.docx</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
-        <is>
-          <t>加州大学圣地亚哥分校  职业指南.docx</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
         <is>
           <t>Career Choice &amp; Change: Job Hunting, Internship Seeking &amp; Discovering Your Career Path: Home
 New Resources
@@ -870,22 +855,19 @@
 .......</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>career choice change job internship career path home material market atlas platform online information mergent market atlas access company ratio business segment description sustainability officer director esg data content company industry index filing report interface database business interface upgrade business source interface bsc searching magazine journal upgrade business news openathensrollout openathens access library openathens access material service quicker access diegos signon sso identity management login credential access material news release vpn method option offcampus access tab info option business journal bizjournalscom business news silicon valley francisco boston pittsburgh access geography city business journal book list ranking institution business category city business news job hunter market company growth library school management account email link right corner content career workplace feed article profile publication job news feed industry article diego business journal publisher vendor california title link business news feed book list material area guide vault material company ranking industry profession profile career advice career guide template sample cover letter job internship program email address job career growth content business source bsc industry coverage industry analyst report book chapter industry news article industry nonprofit education field topic factivacom access source newspaper journal magazine company factivacom delivers language background information job seeker nexis thousand source newspaper wire newsletter magazine trade journal industry news company information information coverage source background information job seeker outlook guide ooh overview job information job environment demand salary bureau labor statistic information career explorer job searcher onet online job title career skill growth education requirement</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>career choice change job hunt internship seek discover career path resource mergent atlas arrive platform replace mergent mergent atlas easy historical company finance ratio business segment description sustainability officer director added esg economic data content useful company industry sec filing report ebscohost interface ebsco database special business interface upgrade business complete interface bsc fresh arrange good efficient searching find requested magazine article upgrade regional business openathens rollout openathens improved start library enable openathens licensed resource allow quicker easy stable integrate san diego single sign sso identity credential resource release understand vpn method continue option full option business article bizjournals business silicon valley san francisco seattle boston pittsburgh geography publish american city business article come associate book list ranking top organization business category respective city regional business useful job hunter company economic fund library rady university prompt account ucsd upper right corner featured content career workplace feed article resume feature regional article keep grow job feed industry article note san diego business article different publisher vendor southern title dedicated socal business feed book list resource professional area include guide contact know vault resource company resume ranking industry profession resume find career advice career guide template sample resume resume job internship find graduate ucsd address career relate content wide job seek career_development content business complete bsc great industry coverage include industry analyst report book chapter industry academic article industry include non profit education field typical business relate topic factiva factiva include global local report article magazine company report factiva delivers content language great background job seeker nexis university nexis university contain full text include report wire transcripts newsletter magazine trade article industry company legal coverage vary international great background job seeker job outlook handbook ooh overview job include job environment demand salary organize bureau labor statistic recent relevant career explorer job_searchers net net allow job title career relevant skill project growth education requirement</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>加州大学戴维斯分校 教师就业资源指南.docx</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
-        <is>
-          <t>加州大学戴维斯分校 教师就业资源指南.docx</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
         <is>
           <t>Getting Started
 /
@@ -1079,22 +1061,19 @@
 Connect to the Library VPN</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>guide share information material davis employee interest access news film learning growth chance support endeavor material community material davis library davis campus access staff vpn davis health vpn question news source davis enterprise search text davis enterprise forward advertisement graphic coverage present sacramento beethis link window search text sacramento bee day advertisement graphic coverage california los angeles time link open window content los time coverage francisco chronicle editionthis link window edition chronicle newspaper california newspaper california newspaper newsbanks newspaper search california title set california california newspaper enterprise fresno bee modesto bee orange county register sacramento bee francisco chronicle san mercury news diego nytimescomthis link window access apps edition variety topic news article blog video feature archive article day user access archive newspaper time user account access account basis access step visit accessnytcom davis network step search listing university california davis davis create account registration field address york time site step account log create account button step login setup download app app store login credential access login location coverage post content washington post coverage daily link window fulltext chicago tribune los angeles york time york time magazine york time book street journal washington post link los angeles time york time street journal washington post economist currentthis link window subscription magazine access feature report economist app android economist version podcasts economist newsletter access davis patron email domain user economistcom account email address chronicle educationthis link window chronicle education source news information job college university faculty researcher staff administrator coverage access world newsthis link window newspaper enterprise selection california selection language newspaper link enterprise check search coverage book web google book book search fulltext book book copyright preview title book search chapter document delivery worldcat catalog catalog million record book title material format library coverage hathitrustthis link window repository book institution state campus google internet archive book copyright text scan online copyright google book site search interface detail hathitrust book davis collection search print search sign right corner davis login access feature loan period book renewal ability item storage borrower locate book person call library congress call loan request journal book loan ill request book article library book article community book project year davis campus community book project ccbp dialogue community member campus community book event stress life society geronimus publication date fusing science justice health researcher arline geronimus book way injustice health people homeland cynthia publication date place hate group people fear zach publication date vision safety year discrimination othering punishment antiracist kendi publication date antiracism concept reorients conversation racismand way day death america younge publication date work facea child damage death country book gun control country book joy lama desmond tutu douglas publication date peace prize holiness dalai lama archbishop desmond tutu year exile violence oppression hardshipsor themthey people planet marble forney publication date cartoonist forney relationship crazy memoir disorder story artist writer documentary film film link window ondemand service filmmaker film distribution company thousand documentary film release cover subject discipline collection title defa film artmattan film ruscico pragda bbc flicker film board canada run feature studio day film criterion collectionjanus film coverage link window documentary film producer distributor bullfrog film film bbc film board canada cbc television trust environment mediastorm terra film kimstim scorpion filmmaker world collection title link window swank access movie show home theater licensing distributing content market college university school library swank distributor movie show library film note license title account film period year link window contains news feature story graphic clip network journalist location coverage file contains screening roomthis link window image collection movie domain viewer topic history film advertising newsreel century material attack selection part record past document attitude perspective belief time wildlife service online medium library assortment image publication document history video clip map domain photo librarythis link window photo collection work observation scientist engineer officer personnel collection century time world center earth surface sun thousand weather space image hundred image shore sea thousand specie image whale range work region region world ocean image art imagesthis link window contains work art collection museum culture time period art art roman work work type work painting sculpture drawing print photograph textile costume art book manuscript link open window library image time period culture document field architecture painting sculpture photography art design form culture music music library classicalthis link window recording music content reference source news text access apps medium music library jazzthis link window music jazz offer track jazz album jazz artist music jazz comprises jazz label jazz content music library worldthis link window music world range content performance world music recording artist catalogue world music label arc folkways platform thousand title label title nml world music country group archive cylinder audio library funding institute museum service foundation donor collection recording library recording wider audience online database type recording song act music comedic recording speech website collection cylinder recording part library registry recording home wax recording people home record company field researcher spirit public interaction technology ethnomusicology field recordingsthis link window collection hundred field recording photograph field note collection material tradition yoruba africa hop brooklyn guatemala people javanese format field recording interview recording film footage field slide correspondence ephemera instrument map feature identity norm religion gender role theme feature ethnomusicology archive university washington music music online link window oxford music online material music grove dictionary music oxford dictionary music oxford companion music growth information onet onet program nation source information data nature work workforce economy outlook bureau labor statistic outlook guide information worker work environment education training qualification job outlook occupation source information profile percent job economy ooh cluster occupation occupation occupation group side homepage index occupation search occupation selector menu homepage select pay range education job growth rate occupation job title search guide box ooh faq education education link window contains title ebooks tutorial path book title publisher mcgrawhill pearson technology group time press rider press prentice hall ptr que sam harpercollins publisher management astd apress amacom provider coverage business desktop web submission science management medium engineering information technology software growth architecture math science career growth database hour video presentation education information result reading list notetaking bookmarking libguide ohe coverage material information centerthis link window education material information center database education information department education platform citation journal article book conference report policy dissertation thesis material field education majority journal document institution association center policy institution university department education agency state agency agency contributor conference dissertation thesis coverage jove science education link window library video teach concept technique demonstration interface jove core video textbook area biochemistry biology cancer chemistry biology engineering environment genetics immunology infection medicine neuroscience davis access jove platform jove overview introduction education support jove faculty jove video class syllabus lab education requirement link canvas course jove faculty material interest habitat world field guide birder naturalist ecologist campbell author field guide world land habitat format history field guide compact book feature identification description color photograph habitat wildlife distribution map diagram silhouette habitat figure grasp scale habitat climate box comparison habitat box explanation phenomenon habitatsfrom plate tectonics mountain formation regime climate change field guide author diane database field guide listing title field researcher guide region andor type specie history topic note field guide davis library ruth gustafson biodiversity heritage link window biodiversity heritage bhl consortium history library cooperate legacy literature biodiversity collection literature access part biodiversity common bhl literature component encyclopedia life eol access information specie language spectacle world historythis link window material hundred account woman travel globe century century student researcher source variety topic empire climate custom exploration family life housing industry language monument history politics diplomacy race religion science shopping war variety form travel writing manuscript diary correspondence guidebook material slideshow hundred item material postcard sketch access world newsthis link window newspaper enterprise selection california selection language newspaper link enterprise check search coverage bibliographythis link window language association bibliography mlaib material language linguistics folklore world citation item journal series book collection proceeding dissertation bibliography mlaib index book coverage politics press reference suitethis link press search environment analysis issue news coverage status bill vote amendment floor committee activity backroom maneuvering database fulltext magazine researcher document variety reference book datasets issue politics area policy health care education economics bioethics environment society content capitol hill reporter editor researcher coverage analysis issue congress way davis material university network journal newspaper subscription database medium service apps way access material campus signon vendor signon access journal video material davis kerberos material signon vpn connection network access material campus connect vpn</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>start guide design introduce share library resource davis employee interest include late watch documentary film lifelong learning seek professional davis library support endeavor resource entire community resource license davis library davis staff library vpn davis health vpn find feel free ask librarian local davis enterprise retrieve full text davis enterprise august forward exclude advertisement graphic coverage august present sacramento beethis retrieve full text sacramento bee previous exclude advertisement graphic coverage present los angeles full text content los angeles coverage present san francisco chronicle digital editionthis digital edition san francisco chronicle daily report report report newsbank america report database title small set northern local report include davis enterprise fresno bee modesto bee orange county sacramento bee san francisco chronicle san jose mercury san diego union tribune national nytimes comthis unlimited nytimes nyt mobile include spanish chinese edition resume topic break article blog video interactive feature include archive present article limit unlimited archive proquest historical report note nyt account gain account reactivate annual basis activate visit accessnyt connect davis network include vpn listing university davis davis account complete registration field address account log account mobile setup nyt app app store credential unlimited nytimes coverage present post full text content post coverage present major daily full text chicago tribune los angeles include magazine book wall article post direct uclibs pid chicago tribune uclibs pid los angeles uclibs pid uclibs wall article uclibs pid post economist subscription weekly magazine full interactive feature special report economist app android ios economist audio version podcasts economist digital newsletter davis patron ucdavis domain mean visit economist account xxx address chronicle higher_educationthis chronicle higher_education job university university faculty researcher staff administrator coverage present international newsthis international report include davis enterprise selection include selection spanish language report direct davis enterprise check library early coverage find book book google book google book full text book book copyright able preview title book library chapter report delivery worldcat catalog catalog million record book article title material format library worldwide coverage present hathitrustthis repository scan book contribute academic institution united state include digitize google internet archive book copyright scan searchable full text scan copyright expire significant google book effective sophisticated interface additional detail hathitrust find book davis library collection print ebooks library sign top right corner davis full feature include loan period book renewal ability item storage check borrower locate book person understand call explain library congress call interlibrary loan article book submit interlibrary loan ill book article mail free library book article community book project davis community book project ccbp promote dialogue build community encourage diverse member surround community book attend related event weather extraordinary stress ordinary life unjust society arline geronimus article fusing science social justice renowned health researcher arline geronimus urgent monumental book explore systemic injustice erode health marginalized hate homeland cynthia miller idriss article startling unexpected violent hate recruit young fear zach norris article groundbreaking vision safety overturn fear base discrimination othering punishment antiracist ibram kendi article antiracism transformative concept reorients reenergizes conversation racism liberate think death america gary younge article powerful move job put human face child face collateral damage gun death country book gun control happen country exist book joy dalai lama desmond tutu douglas abrams article nobel peace prize laureates holiness dalai lama archbishop desmond tutu survive fifty exile soul crush violence oppression hardship say joyful planet marble ellen forney article cartoonist forney explore relationship crazy creative graphic memoir bipolar disorder weave story famous bipolar writer documentary film kanopy film stream servicethis demand stream video job filmmaker film distribution company award win documentary train film theatrical release resume diverse subject discipline collection include title defa film library artmattan film hbo frameline ruscico pragda bbc flicker alley national film board canada run feature cinema libre studio film criterion collection janus film coverage present docuseek documentary lead film producer distributor include bullfrog film icarus film bbc national film board canada cbc television trust environment mediastorm terra nova film kimstim scorpion independent filmmaker full collection title anticipate complete swankthis swank movie show theater licensing distributing content non theatrical include university university university library swank old distributor movie show operate ucd library license film swank note additional license title license require account film license period image photography newsroomthis contains break feature story photograph graphic audio clip produce network award win journalist operate worldwide coverage present file contains present national screening roomthis showcases vast moving image collection design unavailable movie copyright domain accessible viewer worldwide topic include history film advertising newsreel span twentieth century end material relate september attack selection present record past historical report reflect attitude perspective belief different national digital library fish wildlife free digital medium library wide assortment image article include historic report oral history video audio clip map domain noaa photo librarythis digital photo collection include job observation carry scientist commission officer administrative personnel collection span century natural earth surface sun include weather image image shore coastal sea marine specie image great whale minute plankton geographic noaa job encompass polar polar ocean art image amica library art image contains job art collection contribute museum worldwide culture period contemporary art native american inuit art ancient greek roman egyptian job japanese chinese job job include painting sculpture drawing print photograph textile costume jewelry decorative art book manuscript artstorthis contain library digital image resume period culture report field architecture painting sculpture photography decorative art design visual culture music stream audio naxos music library classicalthis stream recording classical music content add include biographical text include apps social medium present naxos music library jazzthis naxos music library jazz track jazz album jazz represent naxos music library jazz comprises naxos jazz label fantasy jazz content add naxos music library worldthis naxos music library wide content legendary historical performance contemporary music feature recording complete catalogue important music label arc smithsonian folkways platform title label title added weekly nml resume music country cultural audio archive ucsb cylinder audio archive ucsb library funding institute museum library grammy foundation donor digital collection cylinder recording hold ucsb library bring recording wider audience library stream free searchable database feature recording late early include popular song act classical operatic music comedic monologues ethnic foreign recording speech readings include library collection vernacular wax cylinder recording library congress national record registry personal recording know wax recording everyday record company field researcher capture early spirit interaction record technology ethnomusicology global field recordingsthis global collection audio field recording videos photograph field note ethnomusicological collection material report musical tradition worldwide yoruba africa hip hop brooklyn guatemala indigenous javanese indonesia format include audio field recording interview educational recording film footage field notebooks slide correspondence ephemera unique musical instrument map feature support cultural identity social norm religion ritual gender work theme feature content ucla ethnomusicology archive university music dictionaries oxford music oxford music consist resource music grove dictionary music musicians oxford dictionary music oxford companion music professional occupational net net nation primary occupational valid data essential understand changing nature job impact workforce economy occupational outlook handbook bureau labor statistic occupational outlook handbook ooh worker job environment education training qualification pay job outlook similar job additional occupational resume resume percent job economy ooh break cluster similar job find job browse job left hand side homepage know specific job job selector drop ooh homepage pay entry education job training project job project growth rate specific job interested enter job title handbook top ooh faq bls ooh ooh faq htm education higher_education contains title technical ebooks videos interactive tutorial path audio book associate include selective title global publisher include mcgraw hill pearson technology addison alpha financial hall cisco press rider peachpit press prentice hall ptr que sam harpercollins pakt publisher mit sloan astd apress amacom provider subject coverage business desktop application data science digital medium engineering technology software architecture math science personal professional database contain video include presentation higher_education additional customize result develop personalized reading list engage notetaking bookmarking find proquest libguide ohe proquest libguides coverage present eric educational resource eric education resource database education sponsor department education proquest platform eric include citation article article book conference technical report policy dissertation thesis material field education majority article peer report eric produce scholarly organization professional association policy organization university press department education federal agency state agency local agency contributor submit conference dissertation thesis coverage present jove science education library scientific video teach key concept fundamental technique visual demonstration platform interface include jove core video textbook jove lab manual subject area include behavior biochemistry bioengineering biology cancer chemistry developmental biology engineering environment genetics immunology infection medicine neuroscience davis full entire jove platform jove overview introduction start train education faculty support jove job faculty identify jove video appropriate training syllabus lab education requirement integrate video canvas training jove faculty resource special interest nature habitat field guide birder naturalist ecologist iain campbell author field guide major land habitat format natural history field guide compact accessible comprehensive book feature concise identification description illustrated include color photograph habitat wildlife distribution map diagram silhouette depict habitat human figure immediate grasp scale major habitat illustrated climate allow easy comparison habitat thirty illustrated present clear explanation complex phenomenon affect habitat plate tectonics mountain formation fire regime climate change international field guide database author diane schmidt database field guide assess listing title useful field researcher wish determine publish portable guide exist resume geographic specie natural history topic note field guide davis library contact ruth gustafson ragustafson ucdavis biodiversity heritage librarythis biodiversity heritage library bhl consortium natural history botanical library worldwide cooperate digitize accessible legacy literature biodiversity hold collection literature responsible global biodiversity common bhl serve foundational literature component encyclopedia life eol texts specie travel foreign language travel write spectacle historythis resource bring account woman travel globe early century late century student researcher find resume topic include architecture art british empire climate custom exploration family life housing industry language monument mountains natural history politics diplomacy race religion science shopping war wide travel writing include unique manuscript diary correspondence drawings guidebook photograph resource include slideshow item visual material include postcard sketch photographs newsthis international report include davis enterprise selection include selection spanish language report direct davis enterprise check library early coverage mla international bibliographythis modern language association international bibliography mlaib resume international scholarly material language literatures linguistics folklore include citation item article book essay collection job proceeding dissertation bibliography mlaib book coverage present politics press library political suitethis congressional quarterly press integrate environment obtain analysis congressional issue coverage status bill vote amendment committee activity backroom maneuvering database full text magazine researcher historic report contact directories book datasets focus issue politics area policy health care education economics bioethics environment society content capitol hill reporter editor researcher non partisan coverage detailed analysis issue face congress connect davis library resource limit university network pay article report subscription library database stream medium educational clinical apps possible license resource single sign vendor support single sign allow article video resource davis kerberos cas password resource single sign library vpn library vpn allow secure connection university network direct library material connect library vpn</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>6</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>加州大学洛杉矶分校  资源链接.docx</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
-        <is>
-          <t>加州大学洛杉矶分校  资源链接.docx</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
         <is>
           <t>Career Research in the Rosenfeld Library
 The Rosenfeld Library partners with the Parker Career Management Center (PCMC) and the Professional MBA Programs Career Management Center, who along with the UCLA Career Center, have the primary responsibility for career planning and job search. Parker CMC provides research resources (including Vault and WetFeet) and appointments (Anderson student login required) with professional counselors. FEMBA and EMBA students have access to the ProMBA Career Management Center and their Career Tools.
@@ -1203,22 +1182,19 @@
 Career Management - Research Using the Rosenfeld Library</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>career rosenfeld rosenfeld partner parker career management center pcmc master of business administration program management center career center responsibility career planning job search parker cmc material vault wetfeet appointment student login counselor student access promba career management center career tool material career need career center job search job search link job search link graduate student center career acquires material curriculum source company industry information career planning evident strategy guide career management rosenfeld note online source contract access faculty student anderson information employer company stock company company disclosure information edgar company search company security exchange commission company search bloombergbusiness week company search mergent index company mergent online index reference quotecom symbol company stock company subsidiary company business topic company ownership subsidiary source rosenfeld family affiliation reference mouseover business tab custom search menu ownership headquarterbranch strategy background company company word disclosure report company source company report mergent online report online type company identifier box company match result report tab database report filing security exchange commission click strategy background company party analysis thomson reuters fulltext street analyst report capital mergent standard poor description reference yahoofinance profile data news zacks analysis stock performance click strategy company growth year business source ebsco type company box select field company entity select tab business proquest newspaper company box select field companyorg company menu search box click strategy company event day change news wire service newspaper company box select field companyorg company menu search box abcnewscom business news cnnmoney marketwatch click strategy target company size specific company business topic ranking source rosenfeld business ranking reference angeles business journal reference list company company reference business sale employee strategy iib company industry index code company industry forbes industry industry week manufacturer industry dollar directory reference reference business naics industry keyword register corporation reference click strategy iic company area california company state directory reference business custom search geography register manufacturer thomasnet search state california manufacturer reference affiliation list angeles business journal reference california business directory buyer reference click strategy company world company business reference click strategy target industry standard industry grouping classification sic reference industry classification system naics reference hfa click strategy iiib industry profile guide industry labor freedonia focus industry market world industry market mergent industry report online manufacturing service industry trade administration service market search industry click strategy iiic industry news business source ebsco select publication type industry profile factiva industry menu search box click strategy iiid industry performance measure ratio company source ratio industry ratio source ratio industry norm business ratio reference statement business topic ratio source strategy association trade source contact information association institution gateway association society association executive manufacturing service analyst trade administration reuters street analyst industry focus strategy rosenfeld library guide cmc listing career management rosenfeld library</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>career rosenfeld library rosenfeld library partner parker career pcmc professional master of business administration career ucla career primary responsibility career planning job_search parker cmc resource include vault wetfeet appointment anderson student require professional counselor femba emba student promba career career tool internet resource career ucla career job_search websites academic job_search non academic job_search graduate student library specialize career rosenfeld library acquires material curriculum company industry career planning evident strategy guide list career rosenfeld library note resume contract limit curriculum ucla faculty ucla student limit ucla anderson prospective employer determine company stock company company require disclosure jump know edgar company company require file security exchange commission company bloomberg business week company mergent complete corporate company include mergent hardcopy mergent complete corporate quote locate ticker symbol company stock company check subsidiary company business topic company ownership structure subsidiary compile rosenfeld library include america corporate family lexisnexis corporate affiliation usa mouseover business custom ownership headquarter branch strategy background company company word disclosure report company jump company annual report mergent annual report enter mergent company identifier company match result annual report edgar database company file annual report filing security exchange commission strategy background company third party analysis investext thomson reuters full text wall analyst report finance mergent standard poor corporation description yahoo finance resume data zacks analysis company stock performance strategy company late business complete ebsco company field company entity lexisnexis academic red business proquest report company field company factiva expand company strategy late company event late lexisnexis academic change check wire proquest report company field company factiva expand company abcnews business bloomberg cnn money marketwatch strategy seek target company large specific company business topic ranking compile rosenfeld library include business ranking annual list los angeles business article forbes list include forbes big company large company fortune usa business sale employee strategy company specific industry sic code forbes best company sort industry forbes global sort industry industry week large manufacturer sort industry dollar usa business sic naics industry keyword corporation strategy company specific geographical area company state national list usa business custom geography thomas american manufacturer thomasnet state manufacturer lexisnexis corporate affiliation list los angeles business article southern business buyer guide strategy international company forbes forbes global big company fortune fortune global principal international business strategy iii seek target industry iii standard industry grouping standard industrial classification manual sic hardcopy north american industry classification naics hardcopy strategy iii industry resume career guide industry department labor freedonia focus industry portal ibis industry mergent webreports include industry report manufacturing industry international trade administration commercial international industry strategy iii industry trend title business complete ebsco article industry resume factiva expand industry lexisnexis academic strategy iii industry performance measure benchmarks ratio company ratios ratio industry ratio ratio industry norm key business ratio rma annual statement business topic financial ratio additional strategy iii association trade contact unpublished association organization compile internet library gateway association american society association executive manufacturing analyst international trade administration thomson reuters identify wall analyst industry focus strategy additional rosenfeld library guide cmc listing career rosenfeld library</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>华盛顿大学 3个链接.docx</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
-        <is>
-          <t>华盛顿大学 3个链接.docx</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
         <is>
           <t>Career Tools: Print, E-Book, &amp; Audiobook
 Links to continually updated lists of e-books, print books, and audiobooks that you can browse or search -- all focused on helping you with your job and career search.
@@ -1266,22 +1242,19 @@
 What's in this guide</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>career tool ebook audiobook link list ebooks book job career search title youd book ebooks database career company job advice guidance career intelligence vaultcom material vault guide ranking article career strategy job posting vaultcom student onestopshop student alumnus job information career chance visa immigration support screen company capital contains company analysis pitchbook search thousand equity venture capital deal hundred criterion pitchbook benchmark time data deal identify comparables search investor detail data reference usa information address phone business resident health care provider consumer orbis company emphasis company information information bvdeps company information product range report format information company financials news market rating country report report ownership data college career find information career career information system tool career chance school campus access account wois offcampus site key access service account hour campus library access unique bothell college career center support washington state job state washington site job service job job search workforce service area access career information outlook guide state department labor reference source hundred type job training education earnings job prospect worker job condition information center multivolume reference information job seeker career area profile job chart job description information department web site career material workforce information job seeker student business workforce career talent growth economy career home guide material career choice school occupation information material career outlook salary job search strategy material career option information employer responsibility job search material job chance interview cover letter material resume building interview skill school material school chance test preparation networking material career association skill job career whats guide</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>career tool print book audiobook updated list book print book audiobooks browse focus job career know title add know book print book audiobooks overdrive database career company job advice guidance vault career intelligence vault primary resource vault guide vault ranking article career job seek strategy job posting due cost vault fuqua student interstride stop shop empowers duke student alumnus seek international employment career network mentorship visa immigration support screen company finance contains comprehensive fundamental quantitative company analysis pitchbook equity venture finance deal criterion pitchbook establish benchmark find real data deal identify analyze comparables investor detail data fka usa contain detailed include address phone business resident health care provider orbis orbis resume company worldwide emphasis company integrate hold bvdep company product orbis global standard report format descriptive company finance rating country report scan report ownership data university career find career wois career tool explore career educational university wois account wois key personal account contact library key unique bothell cascadia university contact career support state job train state official employment find job job_search locate workforce area career occupational outlook handbook put united state department labor describe different job describe training education earnings expect job prospect worker job career multi volume set job seeker various career area resume include job summary chart job description salary careeronestop department labor sponsor career resource workforce job seeker student business workforce professional foster talent global economy career guide guide resource career choice include graduate_school job resource describe different career outlook salary job_search strategy resource explore career option company industry employer social responsibility job_search engines specialized resource locate job_opportunities resume interview resume resume resource resume write resume interview skill graduate_school test resource graduate_school international test preparation networking resource career alumni association network skill job career welcome guide</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>8</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>华盛顿大学盛路易斯 通用型.doc</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
-        <is>
-          <t>华盛顿大学盛路易斯 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
         <is>
           <t>Finding a Job: Job Postings
 Job Postings
@@ -1611,22 +1584,19 @@
 Administered by the Open Society Foundations, this fellowship funds individuals working to reform the criminal justice system. Fellowships are available for advocacy, media, or scholarly work, and last 12–18 months.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>job job posting job posting job board bar association career center bar association career job job enhance career association counsel job board listing fellowship role law student graduate inhouse position attorney job usa job board position keyword location filter update experience area region postgrad position job search engine job website prospect wustledu email address login law job search platform firm data trend job posting helpful law firm activity employer recruit forward wustledu email address login platform recruiting event oncampus program student interview session fair law school employer biglaw law student summer associate position firm profile interview tip insight law firm handshake log washu job internship platform university law school listing student access event interview llm nonjd job china job board job seeker job chance job board job seeker job chance filter experience level search networking platform law student job alumnus law firm career path job directory employer material association law placement information law firm government agency interest institution corporation profile experience area office location criterion data hour expectation diversity statistic nalp job material association law placement information law firm government agency interest institution corporation profile experience area office location criterion data hour expectation diversity statistic symplicity log washu key feature posting internship externships postgraduate job program book appointment event house representative job house representative job posting counsel role committee staff job job posting chance system submission online portal clerkship applicant law school official judge clerkship submission platform judge staff oscar submission material profile letter transcript sample letter recommendation cora center state court court chance recruitment cora online portal court internship externship chance student graduate court jersey court jersey court law clerkship court tax court experience salary career prospect chance center state court material court job posting cles update state court state court job posting position court probation service institution branch agency search term career law law clerk staff attorney supervisory staff attorney interest capital defense internship job website internship job country capital defense berkeley law school justice work institution interest career fellowship law student program career growth material law student lawyer chance community advance access idealist link institution job publication support service networking information aid job posting volunteer chance internship dropdown career district attorney career center aid defender association job board position justice community posting position aid service institution interest institution interest law firm york state defender association york defense community defense job job listing job type title skill location psjdorg account job law firm employer interest law initiative pili illinois institution interest law work internship fellowship law student graduate career lowincome client society nonprofit job listing type location work institution classified search keyword institution type position type statecountry europe lawyer group ealg association law firm member country service site directory member firm country euro job posting board euro affair kingdom allaboutlaw job posting law career society law asil job posting institution career law student member institution institution washington law relation member country attorney academic judge student nation career job nation job network state state bar alaska bar association attorney magazine arkansas bar association account california california lawyer colorado colorado bar association bar association delaware delaware state bar association job board bar georgia state bar georgia state bar georgia list vacancy government attorney position hawaii state bar association idaho state bar illinois illinois state bar association indiana indiana state bar association iowa iowa state bar association bar association bar association state bar association maine maine bar association maryland maryland state bar association massbar association michigan state bar minnesota minnesota state bar association job board bar missouri bar montana state bar montana nebraska nebraska state bar association state bar hampshire hampshire bar association jersey jersey state bar association mexico state bar york york state bar association north bar association dakota state bar association ohio ohio bar oklahoma oklahoma bar association oregon oregon state bar pennsylvania pennsylvania bar association rhode island rhode island bar association carolina south bar south state bar tennessee tennessee bar association texas state bar island island bar association state bar vermont vermont bar association virginia state bar washington washington state bar association washington district bar virginia virginia state bar wisconsin state bar wisconsin state bar interest lcc aflcio lawyer committee institution lawyer firm union department hall list law position state immigration lawyer immigration job posting defense fund aldf list job chance law firm institution career law trademark association intas job bank feature attorney job chance internship tax talent position tax world position job government job interest law association counsel job board material law student career law counsel role listing attorney company internship externships entrylevel chance compliance privacy environment governance interest law environmentalcareercom search job region keyword ecojobs subscription week advocacy job dream job sustainablebusinesscom search job type skill level state interest group listing opening state interest group interest immigration refugee law immigration lawyer offer law student mentorship career material immigration law access job listing training chapter event immigration chance bar association student volunteer internship role institution service detainee experience interest immigration law interest growth growth bank offer internship program law student graduate growth finance policy role contract project finance procurement governance growth bank internship earlycareer chance law student growth law finance partnership asia intern lending compliance policy center growth engagement growth issue policy community focusing policy country growth prospect country cgd partnership participant work bank reconstruction growth offer internship earlycareer chance law student graduate finance growth reform intern banking law investment agreement framework market policy policy forum information globalization growth growth bank internship fellowship law student graduate growth finance policy latin america role contract compliance law interaction material people volunteer position relief growth agency job board institution interaction material link position ngo institution growth relief country job fair conference area law student career bar association justice diversity center july registration april close lawyer group job june registration close law conference june bar association minority law student job june registration damali booker diversity job bar association registration delaware diversity job ddjf submission april attorney pipeline program dapp submission august december kansa city job july graduate close minority recruitment conference mmrc student registration april end prosecutor conference job july registration latinao law student association conference march registration lgbtq bar association lavender law conference career july nut bolt patent law interview program plip june registration march property law association registration open close property job sipjf june registration december close justice work conference career interest law career conference mpilcc registration association counsel child bird registration component aid defender association justice conference close bar association clerkship job july registration june veteran career fellowship fellowship profellow psjds fellowship service career database fellowship program listing access register account fellowship interest law student graduate center innovation fellow program bar association center innovation encourages accelerates innovation affordability effectiveness efficiency accessibility service law school graduate year year residence headquarters fellow stipend benefit time program bristow program department justice office solicitor law solicitor court brief argument fellow year term candidate record experience appellate judge writing skill fellowship experience litigation insight proceeding career law academia service georgetown law public policy fellowship program offer fellowship interest lawyer womens right fellow womens issue washington interest institution government agency engage growth activity program fellowship submission august phyllis interest law independence foundation support service region fellowship program fund salary benefit lawyer interest work representation client foundation fellow student loan repayment fellowship program law student worker right labor law honor labor attorney peggy fellowship law student summer internship labor union worker advocacy institution government agency justice attorney worker right november summer internship right project fellowship fellowship state agency litigation community engagement resident right diverse government leader work right justice issue population fellowship stipend health benefit justice fellowship program fellowship law advocacy skill health right justice field community fellow handson policy advocacy experience issue fellowship stipend benefit fellowship foundation interest law fellowship program arp slate meagher flom fellowship law school graduate clerk service fellow project issue lowincome community project work service policy advocacy litigation community fellow salary benefit associate salary law firm submission steel postgraduate fellowship fund lawyer interest law project gay transgender community state year fellowship fulltime year pride law fund project impact applicant law student following lawyer year law school government fellowship state attorney office term fellowship honor program chance attorney honor program postgraduate program attorney california department justice division solicitor fellowship fellowship earlycareer lawyer experience advocacy california solicitor office issue attorney program graduate clerk policy matter colorado department law georgia attorney honor program fellowship law experience attorney georgia department law massachusetts attorney honor program fellowship earlycareer attorney chance division massachusetts attorney office issue attorney honor program program graduate clerk skill placement jersey department law safety division department justice honor attorney program program attorney chance experience law division oregon doj ralph carr fellowship colorado attorney fellowship litigation fellow behalf state colorado appellate court washington state attorney honor program program attorney experience service law placement division agency honor program fellowship honor attorney program entrylevel program law graduate judicial clerk gain experience government agency institution program year agency program consumer protection bureau cfpb honor attorney program department homeland security dhs secretary honor attorney program attorney rotation office security safety expertise department justice doj attorney program doj honor recruitment program place attorney component right criminal security division department labor dol attorney honor program selects graduate issue labor standard benefit workplace safety department labor department transportation dot honor attorney program place attorney office dot transportation safety regulation policy issue protection agency honor program program website usajobscom attorney position communication commission attorney honor program law grad policy issue communication law communication commission deposit insurance corporation fdic honor attorney program train attorney banking law housing growth honor program law hud housing right growth law revenue service irs counsel honor program place attorney office counsel tax law litigation labor relation board nlrb honor attorney program offer experience labor relation law security agency office counsel honor program attorney chance security issue commission law graduate program attorney training safety licensing compliance office comptroller currency occ honor attorney program grad banking service law occ matter corp engineer office counsel honor attorney program attorney contract law work project office barbara ringer honor program attorney experience copyright policy litigation work interest fellowship fellowship liberty union aclu fellowship law graduate attorney liberty right issue program area justice freedom immigrant right fellowship year litigation fellowship law litigation focus class action interest law fellow cohen milsteins client right job experience year prettyman fellowship law fellowship attorney defense teaching fellow client court law student career defense education fellowship entrepreneur jds fellowship fund service project potential impact fellow support leadership growth justice fellowship fund year work project partner interest institution summer submission year fellowship interest project applicant collaboration host institution justice corp fellowship law law student nonprofit institution immigration service training mentoring term justice catalyst fellowship support law interest project injustice change fellow nonprofit venture renewal soros justice fellowship society foundation fellowship fund individual justice system fellowship medium work month</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>find job job posting job posting job board american bar association career american bar association legal career central legal job job alert resume enhance career association corporate counsel acc job board listing include internships fellowship entry work suitable law student recent graduate interested house position attorney job usa job board tailor legal position set keyword filter sign weekly update useful target specific practice area geographic post grad lateral position careerjet employment engine draw job publish worldwide firm prospect require active wustl address log law student focus job_search platform detailed firm data hire trend job posting helpful track law firm recruit activity identify potential employer flo recruit forward require active wustl address log platform virtual legal recruiting event interview oci student participate interview network session hire fair host law_school employer gobiglaw focus biglaw hire law student seek summer associate entry position firm resume interview tip insight large law firm recruit handshake log washu key job internship platform university include law_school tailor listing student employer event interview focus non job china comprehensive job board allow job seeker legal nonlegal employment comprehensive job board allow job seeker legal nonlegal employment lawjobs filter include experience initial linkedin professional networking platform law student apply job connect alumnus follow law firm helpful career path recruiter post legal job nalp legal employer comprehensive accessible resource maintain national association law placement nalp depth law firm government agency interest organization corporation resume include practice area office hire criterion salary data billable expectation diversity statistic nalp job comprehensive accessible resource maintain national association law placement nalp depth law firm government agency interest organization corporation resume include practice area office hire criterion salary data billable expectation diversity statistic symplicity log washu key feature posting internship externships post graduate job coordinate recruit resume book career counsel appointment event house representative employment house representative job posting include legal counsel work committee staff senate employment senate legal legislative job posting judicial clerkships clerkship application primary portal federal clerkship applicant law_school official federal judge manage clerkship application store platform federal judge staff oscar collect application material include resume resume resume transcript write sample resume recommendation cora national state court ncsc court recruitment cora free portal court showcase clerkship internship externship student recent graduate state court parallel oscar jersey court jersey court recent law graduate clerkship various court include supreme appellate tax superior court hand legal experience competitive salary improved career prospect judicial national state court ncsc resource non clerkship court job posting cles update state court unite state court job posting position federal court probation pretrial defender organization judicial branch agency suggest term include career law clerk judicial law clerk staff attorney supervisory staff attorney magistrate judge interest finance defense internship job internship job country finance defense berkeley law_school equal justice job ejw nonprofit organization facilitate interest legal career fellowship law student career_development resource connect law student lawyer serve underserved community advance equal justice idealist nonprofit organization nationwide contain job article support networking fundraise legal aid job posting volunteer internship list dropdown legal professional national district attorney association ndaa ndaa career national legal aid defender association nlada job board post position equal justice community posting include position civil legal aid defender organization interest organization interest law firm academia state defender association support criminal defense community post nationwide criminal defense job nonprofitjobs job listing searchable job title salary skill psjd free account job public_service mind law firm legal employer interest law initiative pili illinois nonprofit organization foster interest law job internship fellowship initiatives support law student recent graduate legal professional serve low income marginalized client society nonprofit nonprofit job listing job good nonprofit organization classified keyword organization position state country geographic international europe american lawyer ealg ealg association independent law firm member country legal include member firm country euro job posting board euro european affair united kingdom allaboutlaw job posting law career various american society international law asil job posting submit asil organization career counsel law student member institution asil nonprofit organization base foster international law relation member country include attorney academic judge student united nation career job united nation legal job network geographic united state alabama alabama state bar alaska alaska bar association arizona attorney magazine arkansas arkansas bar association account lawyer association colorado colorado bar association connecticut connecticut bar association delaware delaware state bar association job board florida florida bar georgia state bar georgia state bar georgia list judicial vacancy government attorney position hawaii hawaii state bar association idaho idaho state bar illinois illinois state bar association indiana indiana state bar association iowa iowa state bar association bar association kentucky kentucky bar association louisiana louisiana state bar association maine maine bar association maryland maryland state bar association massbar association michigan state bar michigan minnesota minnesota state bar association job board mississippi mississippi bar missouri bar montana state bar montana nebraska nebraska state bar association state bar nevada hampshire hampshire bar association jersey jersey state bar association mexico state bar mexico state bar association north carolina north carolina bar association north dakota state bar association north dakota ohio ohio bar oklahoma oklahoma bar association oregon oregon state bar pennsylvania pennsylvania bar association rhode island rhode island bar association carolina south carolina bar south dakota state bar south dakota tennessee tennessee bar association texas state bar texas virgin islands virgin island bar association utah utah state bar vermont vermont bar association virginia state bar state bar association district columbia bar west virginia west virginia state bar wisconsin state bar wisconsin wyoming wyoming state bar special interest afl cio lcc hire afl cio lawyer coordinate committee national organization union side lawyer firm union legal department hire hall list union side law position state american immigration lawyer association immigration job posting animal legal defense fund aldf aldf list employment various law firm non profit organization career animal law international trademark association inta job bank feature trademark related attorney non attorney job_opportunities internship worldwide tax talent position tax difficult limit legal position usa job federal government job special interest corporate law association corporate counsel acc job board valuable resource law student interested specialized career corporate law house counsel work listing experienced attorney company post internship externships entry compliance privacy environment social corporate governance special interest environmental law environmentalcareer job category keyword ecojobs subscription update week include legislative advocacy job green dream job sustainablebusiness job skill state interest pirg listing opening state interest special interest immigration refugee law american immigration lawyer association law student valuable networking mentorship career resource immigration law include job listing training local chapter event immigration detainee guide american bar association student find hand volunteer internship work organization legal immigration detainee practical experience interest immigration law special interest international african bank internship young professional law student graduate interested international finance policy africa legal work involve contract project finance procurement institutional governance asian bank legal internship early career law student focus law international finance partnership asia pacific legal intern assist sovereign lending compliance legal policy global policy orient active engagement issue policy community focusing policy industrial country affect prospect poor country cgd partnership find participant similar job european bank reconstruction internship early career law student graduate interested international finance legal reform legal intern assist banking law investment agreement regulatory framework emerge global policy forum global policy forum internships ngos globalization international inter american bank internship legal fellowship law student recent graduate interested international finance policy latin america caribbean legal work involve international contract compliance institutional law interaction several key resource helpful seek pay volunteer position international relief agency interaction ngo job board nongovernmental organization interaction several key resource include internet pay volunteer position ngo organization focus international relief different country job fair conference bay area law student career fair bar association san francisco justice diversity july registration april close boston lawyer annual job fair june registration april close break law conference june cook county bar association ccba minority law student job fair june registration close march damali booker diversity job fair bar association january registration close january delaware diversity job fair ddjf application due april diverse attorney pipeline dapp direct january application august close december kansa city heartland legal job fair july recent graduate registration close june minnesota minority recruitment conference mmrc august last hold august student registration april close end national black prosecutor association conference job fair july registration close july national latina law student association conference march registration close march national lgbtq bar association lavender law conference career fair july judicial nut bolt academy loyola patent law interview plip june registration march close april san francisco intellectual property law association sfipla june registration close southeastern intellectual property job fair sipjf june registration december close january equal justice job ejw conference career fair october virtual interest law career conference mpilcc february registration january close january national association counsel child nacc august early bird registration close june component november virtual national legal aid defender association equal justice conference registration close april indianapolis bar association clerkship job fair july registration close june veteran legal career fair september fellowship fellowship profellow psjd postgraduate fellowship public_service legal career database contain funded fellowship listing free account fellowship interest law student graduate aba innovation fellow american bar association aba innovation encourages accelerates innovation improve affordability effectiveness efficiency accessibility legal recent law_school graduate last spend residence aba headquarters chicago fellow receive stipend benefit bristow fellowship prestigious department justice office solicitor recent law graduate job solicitor supreme court assist draft brief prepare oral argument conduct legal fellow term eligible candidate excellent academic record clerkship experience federal appellate judge outstanding writing analytical skill fellowship valuable experience appellate litigation insight high legal proceeding lead distinguish career law academia public_service georgetown woman law policy fellowship fellowship interest lawyer dedicate advance woman right fellow job woman issue interest organization government agency engage educational professional activity fellowship application august honorable phyllis beck interest law fellowships independence foundation support free legal philadelphia fellowship fund salary benefit talented young lawyer commit interest job focus direct representation disadvantaged client foundation fellow student loan repayment brown fellowship design inspire educate law student worker right labor law honor labor attorney peggy brown fellowship law student summer internship labor union worker advocacy organization government agency aim promote social justice develop skilled attorney commit advance worker right apply november summer internship right project fellowship fellowship support local state agency affirmative litigation community engagement enforce resident right aim develop diverse talented government fellows job civil right economic justice environmental issue affect vulnerable population fellowship stipend health benefit reproductive justice fellowship policy focus fellowship recent law graduate aim build legal advocacy skill reproductive health right justice field marginalized community fellow gain hand policy advocacy experience key issue fellowship include stipend benefit skadden fellowship foundation prestigious interest law fellowship found skadden arp slate meagher flom llp fellowship aim support law_school graduate outgo judicial clerk dedicate public_service fellow develop project address civil criminal legal issue affect low income underserved community project involve various legal job include direct policy advocacy impact litigation community outreach skadden fellow receive salary benefit comparable associate start salary major law firm fellows application due september tom steel post graduate fellowship fund lawyer job innovative interest law project serve lesbian gay bisexual transgender community united state fellowship support job full pride law fund aim support project potential last impact eligible applicant law student set graduate following lawyer graduate law_school government fellowship state attorney office post graduate term fellowship honor include attorney honor postgraduate attorney job important legal various department justice division geoffrey wright solicitor fellowship prestigious fellowship early career lawyer experience appellate advocacy job solicitor office complex legal issue colorado attorney fellowship recent graduate judicial clerk job impactful legal policy matter colorado department law georgia attorney honor fellowship pay fellowship recent law graduate gain practical legal experience job attorney georgia department law massachusetts attorney stephanie lovell honor fellowship early career attorney rotate key division massachusetts attorney office handle diverse legal issue jersey attorney honor recent graduate judicial clerk develop legal skill placement jersey department law safety division oregon department justice honor attorney offering attorney chance gain broad experience law job various division oregon doj ralph carr appellate fellowship colorado attorney focus fellowship appellate litigation allow fellow brief argue behalf state colorado appellate court state attorney honor selective design train develop attorney direct experience public_service law placement different division numerous federal agency post graduate honor fellowship honor attorney competitive entry allow law graduate former judicial clerk job high impact legal gain experience government agency organization vary include agency note cancel delay financial protection bureau cfpb honor attorney department homeland security dhs secretary honor attorney entry attorney rotation dhs legal office develop national security safety expertise department justice doj attorney honor know doj honor premier entry recruitment attorney various component civil right criminal national security division department labor dol attorney honor selects recent graduate job complex legal issue involve labor standard benefit workplace safety department labor department transportation dot honor attorney attorney legal office dot job transportation safety regulation policy issue environmental protection agency honor fellowship hire usajobs attorney position federal communication commission fcc attorney honor recruit recent law grad assist legal policy issue involve communication law federal communication commission federal deposit insurance corporation fdic honor attorney train entry attorney banking regulatory receivership law fdic housing urban hud legal honor bring recent law graduate hud job housing civil right urban law internal revenue irs chief counsel honor entry attorney irs office chief counsel focus federal tax law litigation national labor relation board nlrb honor attorney career legal experience labor relation law nlrb national security agency nsa office counsel legal honor give entry attorney chance job national security legal issue nsa nuclear regulatory commission honor law graduate attorney legal training nuclear safety licensing regulatory compliance office comptroller currency occ honor attorney engage recent grad banking financial law occ focus regulatory supervisory matter army corp office chief counsel civilian honor attorney train attorney environmental contract administrative law relate military civil job project copyright office barbara ringer copyright honor give early career attorney hand experience copyright policy litigation regulatory job interest fellowship fellowship american civil liberty union aclu fellowship recent law graduate young attorney job civil liberty civil right issue specific area racial justice reproductive freedom immigrant right fellowship last cohen fellowship litigation fellowship allow recent law graduate job complex civil litigation focus training action interest law fellow cohen milstein client civil right employment practice barrett prettyman fellowship georgetown law fellowship train attorney criminal defense clinical teaching fellow represent client court assist supervise law student ideal pursue career indigent defense clinical legal education echo green fellowship social entrepreneur include jds prestigious fellowship fund innovative public_service project potential large scale impact fellow receive financial support leadership train equal justice job fellowship fund job project develop partner interest organization summer application span entire fellowship fund interest legal project design applicant collaboration host organization immigrant justice corp fellowships fellowship recent law graduate law student nonprofit community base organization direct immigration legal training mentoring term justice catalyst fellowships fellowships support law graduate pursue innovative interest project address injustice push systemic change fellow job nonprofit venture potential renewal soros justice fellowship administer society foundation fellowship fund job reform criminal justice fellowship advocacy medium scholarly job last month</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>9</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>南加州大学  图情专业.doc</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
-        <is>
-          <t>南加州大学  图情专业.doc</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
         <is>
           <t>Library &amp; Information Science *
 Library Careers
@@ -1753,22 +1723,19 @@
 This summary report about Librarians has been created by the Occupational Information Network (O*NET) is being developed under the sponsorship of the US Department of Labor/Employment and Training Administration (USDOL/ETA) through a grant to the North Carolina Department of Commerce.</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>information science library career information science job website website information management position residency interest group graduate interest library place college residency joblist job library information science technology hiring librarian librarian site repository interview question moment question question interview job hundred information science position run information science career state canada job department information job listing material job listing listing job posting lab post email isnet posting record order date department information job listing material job website glassdoor career material user job site newspaper company career user million job library user access job chance company rating employee job seeker salary interview question thousand company place position internship institution job digital tech sector place search job search function website government job site book career ebooks link lead library catalog record ebooks link access ebook ebook publisher account content restriction description publisher author career level ebook publication date career level publishing presenting brand recognition area expertise proposal publication presentation place manager leader edward ebook publication date management context world work guidance information work kim dority call ebook publication date stateoftheart guide world information science reader insight field tool range information science career option skill strength field career lois stickell bridgette sander ebook publication date mlis skill job career step way employer guide science student priscilla shontz call ebook publication date book reader job search stepbystep student experience job author advice year realworld inthefield experience career jane monson call ebook publication date familiarity experience information career book foundation discipline book library list book heading science guidance link outlook guide outlook guide information librarian environment pay job outlook occupation information visit bureau labor statistic department labor outlook guide edition librarian internet httpswwwblsgovooheducationtrainingandlibrarylibrarianshtm library information science listservs listservs way network career variety specialty list listservs library congress keywords job list keywords job searching inaljcom list term job volunteer job work information taxonomist taxonomy database database designer management user interface designer community manager knowledge architect data management analyst information medium marketer intelligence analyst source trainer technology trainer technology database designer metadata coordinator content curator law researcher content strategy experience design project analyst information material officer record manager data scientist data information policy information privacy information recovery data curator dba database administration administrator information officer cio information system program analyst intelligence data visualization market analyst diligence analyst vendor information specialist asset management onet online report librarian information network onet sponsorship department laboremployment training administration grant department commerce</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>library science library career library science job take library position acrl residency interest recent lis graduate interest job academic library academic university residency ala joblist job library science technology hiring librarian take inside hire librarian fantastic repository interview take moment submit ask interview library job library science position find run library science professional united state canada international job ucla department job listing resource job listing webpages contain listing job posting receive lab include receive post receive net posting record list order receive ucla department job listing resource job glassdoor glassdoor free career resource allow job report company career apply million job glassdoor usc library explore job_opportunities company rating write employee job seeker salary interview take company idealist great position internship non profit organization mashable job digital technology sector great boolean advanced job_search function usajobs federal government official job recent book library career come library ebooks lead usc library catalog record ebooks ebook ebook publisher unique account content restriction vary description publisher author take library career next hibner mary call ebook article take library career next participate publishing presenting librarians establish brand recognition area expertise suggest write win proposal article presentation publish manager edward evans call ebook article put library unique context profit job invaluable guidance manage library rethink job kim dority call ebook article state art guide library science give valuable insight field practical tool succeed identify broad library science career option identify professional skill strength lis field library career lois stickell bridgette sander call ebook article mlis skill set library job build library career mean know maximize potential employer want guide library science student priscilla shontz call ebook article book guide plan job_search divide major section student experience job_search author critical advice derive combined real field experience jump start career jane monson call ebook isbn article familiarity digital practice important professional book solid foundation discipline find book custom usc library generate list book ebooks subject heading library science vocational guidance librarians occupational outlook handbook occupational outlook handbook following uptodate librarian summary job environment pay job outlook similiar job visit bureau labor statistic department labor occupational outlook handbook edition librarian internet bls ooh education training library librarian htm visit june library science listservs listservs great network lis professional specialty handy list best listservs curated library congress keywords job_searching helpful list keywords job_searching inalj list term library job volunteer suggest job relate library job librarian library professional taxonomist taxonomy database database designer knowledge interface designer community manager knowledge architect data analyst architect social medium social marketer intelligence analyst trainer technology trainer technology futurist database designer metadata knowledge coordinator indexer digital content curator transactional law researcher content strategy experience design uxd project analyst resource officer certify record manager marc informationist informatician data scientist big data policy privacy recovery data curator dba database administration administrator chief officer cio geographic archivist archives analyst competitive intelligence data visualization analyst due diligence analyst library vendor sit conflict specialist digital asset dam net librarians summary report librarian occupational network net develop sponsorship department labor employment training administration usdol eta grant north carolina department commerce</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>10</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>南加州大学 图情专用.doc</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
-        <is>
-          <t>南加州大学 图情专用.doc</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
         <is>
           <t>Library &amp; Information Science *
 A resource for the USC Libraries as well as our MMLIS.
@@ -1882,22 +1849,19 @@
 This summary report about Librarians has been created by the Occupational Information Network (O*NET) is being developed under the sponsorship of the US Department of Labor/Employment and Training Administration (USDOL/ETA) through a grant to the North Carolina Department of Commerce.</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>information science material library mmlis library information science job website website information management position residency interest group graduate interest library place college residency joblist job library information science technology hiring librarian librarian site repository interview question moment question question interview job hundred information science position run information science career state canada job department information job listing material job listing listing job posting lab post email isnet posting record order date department information job listing material job website glassdoor career material user job site newspaper company career user million job library user access job chance company rating employee job seeker salary interview question thousand company place position internship institution job digital tech sector place search job search function website government job site book career ebooks link lead library catalog record ebooks link access ebook ebook publisher account content restriction description publisher author career level career level publishing presenting brand recognition area expertise proposal publication presentation place manager leader edward management context world work guidance information work kim dority stateoftheart guide world information science reader insight field tool range information science career option skill strength field career lois stickell bridgette sander mlis skill job career step way employer guide science student priscilla book reader job search stepbystep student experience job author advice year realworld inthefield experience career jane monson familiarity experience information career book foundation discipline book library list book heading science guidance link outlook outlook guide information librarian environment pay job outlook occupation information visit bureau labor statistic department labor outlook guide edition librarian internet httpswwwblsgovooheducationtrainingandlibrarylibrarianshtm library information science listservs listservs way network career variety specialty list listservs library congress keywords job list keywords job searching inaljcom list term job volunteer job work information taxonomist taxonomy database database designer management user interface designer community manager knowledge architect data management analyst information medium marketer intelligence analyst source trainer technology trainer technology database designer metadata coordinator content curator law researcher content strategy experience design project analyst information material officer record manager data scientist data information policy information privacy information recovery data curator dba database administration administrator information officer cio information system program analyst intelligence data visualization market analyst diligence analyst vendor information specialist asset management onet online report librarian information network onet sponsorship department laboremployment training administration grant department commerce</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>library science resource usc library mmlis library science job take library position acrl residency interest recent lis graduate interest job academic library academic university residency ala joblist job library science technology hiring librarian take inside hire librarian fantastic repository interview take moment submit ask interview library job library science position find run library science professional united state canada international job ucla department job listing resource job listing webpages contain listing job posting receive lab include receive post receive net posting record list order receive ucla department job listing resource job glassdoor glassdoor free career resource allow job report company career apply million job glassdoor usc library explore job_opportunities company rating write employee job seeker salary interview take company idealist great position internship non profit organization mashable job digital technology sector great boolean advanced job_search function usajobs federal government official job recent book library career come library ebooks lead usc library catalog record ebooks ebook ebook publisher unique account content restriction vary description publisher author take library career next hibner mary take library career next participate publishing presenting librarians establish brand recognition area expertise suggest write win proposal article presentation publish manager edward evans put library unique context profit job invaluable guidance manage library rethink job kim dority state art guide library science give valuable insight field practical tool succeed identify broad library science career option identify professional skill strength lis field library career lois stickell bridgette sander mlis skill set library job build library career mean know maximize potential employer want guide library science student priscilla shontz book guide plan job_search divide major section student experience job_search author critical advice derive combined real field experience jump start career jane monson familiarity digital practice important professional book solid foundation discipline find book custom usc library generate list book ebooks subject heading library science vocational guidance librarians occupational outlook handbook occupational outlook handbook following uptodate librarian summary job environment pay job outlook similiar job visit bureau labor statistic department labor occupational outlook handbook edition librarian internet bls ooh education training library librarian htm visit june library science listservs listservs great network lis professional specialty handy list best listservs curated library congress keywords job_searching helpful list keywords job_searching inalj list term library job volunteer suggest job relate library job librarian library professional taxonomist taxonomy database database designer knowledge interface designer community manager knowledge architect data analyst architect social medium social marketer intelligence analyst trainer technology trainer technology futurist database designer metadata knowledge coordinator indexer digital content curator transactional law researcher content strategy experience design uxd project analyst resource officer certify record manager marc informationist informatician data scientist big data policy privacy recovery data curator dba database administration administrator chief officer cio geographic archivist archives analyst competitive intelligence data visualization analyst due diligence analyst library vendor sit conflict specialist digital asset dam net librarians summary report librarian occupational network net develop sponsorship department labor employment training administration usdol eta grant north carolina department commerce</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>11</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>南加州大学 通用型.doc</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
-        <is>
-          <t>南加州大学 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
         <is>
           <t>Careers
 Search for jobs with USC resources
@@ -2019,22 +1983,19 @@
 FAQ</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>career job material career material guide job internship networking chance guide marshall business library list company industry company financials executive competitor industry information market size trend material search marshall career service school business career program undergraduate graduate business major link information marshall career service graduate career service career center career center career advice handshake enables job institution webinars network trojan trojan network student alumnus employer addition center usc career center advisor job skill department labor website skill salary program school certification search job listing data search job posting job company location data axle jobsinternship job material area tool resume interview tip estimate internship education advice job offer skill business experience master realworld business skill transition campus workplace module data analytics leadership communication professionalism search million job company employee job access tool job search company linkedin business medium platform network relationship skill career ebooks business career growth communication company company login click searchfunding search date location company capital login analysis company industry market news market insight company performance industry data screener database company equity business growth people criterion vpn vpnuscedu company industry screener screen company menu industry field search filter etc view result report company choose company profile news subsidiary industry news news company factiva information company industry article newspaper trade magazine press blog business forecaster diligence company mention news search field enter start company ticker company factiva expert search tab click news newsand language choice click search right industry industry market database content industry login measurement assessment market chance market frost sullivan login industry technology consulting firm market area information communication technology aerospace defense healthcare chemical material food automation control measurement instrumentation electronics security energy power system transportation building technology downloading report student information technology company document form ibisworld industry market report industry risk rating state data market find market report type business cover market login mintel report mintel trend consumer market analysis trend product database product data product food beauty care health hygiene home care pet market login passport gmid market information database range consumer market industry information country world company analysis country briefing sector market industry watch article consumer lifestyle report find executive terminal business library jff company record mgmt function company management team list age position executive company investor relation company executive investor relation company investor relation capital login analysis company industry market vpn vpnuscedu search company record peopleprofessionals column executive company executive information email orbis login search company director manager advisor navigation column association website association industrycareer jobstarscom careeronestop glassdoor directory association trend link report future job career forecast future job report world forum workplace trend tech trend technology trend outlook dream challenge world job outlook institution alumnus database access library student privilege access database material semester term semester enrollment course interlibraryloan eligibility student period alumnus access library database material alumnus loan service alumnus library access business material angeles database business insight essential data axle reference solution demographic hoover company mergent archive morningstar netadvantage srds value line database gale business insight demographic data axle santa database morningstar referenceusa value line california material graduation information material content information borrowing privilege alumnus tab borrowing policy information access policy business accounting library guide part series material topic course marshall usc hour operation contact information faq</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>career job usc resource career resource guide job internship professional networking guide usc marshall business account library build list company preferred industry specific company finance key executive competitor find industry trend identify university resource aid usc marshall career_services marshall university business robust career advise undergraduate graduate business major marshall undergraduate career_services usc marshall graduate career_services usc career usc career resume career advice network handshake enables job organization attend webinars network fellow trojan trojan network student alumnus employer addition usc university base career advisor assist job skill careeronestop sponsor department labor explore skill salary find university certification resume job listing data axle job posting job company data axle job internship module job resource area tool resume write interview tip salary estimate internship continue education advice relate job sage skill business practice master real business professional skill transition workplace module include data analytics entrepreneurship leadership organizational communication professionalism glassdoor million job company former employee job tool job_search resume company linkedin business employment focus social medium platform professional network build relationship skill succeed career iglibrary ebooks business career_development corporate communication company find company privco usc require funding preferred find company fund finance usc require analysis company investable industry financial contain financial insight company performance industry data screener large database company equity business criterion note vpn vpn usc find company industry screen quick screener screen company drop industry field continue remain filter geography result cap detail report company university lexis nexis academic find company locate resume include subsidiary finance swot industry find negative company factiva find company industry include article report trade magazine press release blog business forecaster conduct due diligence company require find negative mention field enter start company ticker pop company factiva expert sentiment negative language choice low right industry industry usc libraries subscribe databases industry specific database content span multiple related industry bcc usc require bcc objective unbiased measurement assessment detailed report frost sullivan usc require industry technology global consulting firm resume international area communication technology aerospace defense healthcare chemical material food industrial automation control measurement instrumentation electronics security energy power automotive transportation environmental technology single downloading entire report enable student gartner detailed technology advisory company report full text ibisworld industry report industry risk rating focus united state data global marketresearch academic find lengthy detailed report brief white describe business resume international mintel usc require mintel report mintel trend comprehensive depth analysis trend mintel global product database include detailed product data product food drink beauty personal care health hygiene care pet passport usc require passport gmid global database wide industry country include company resume swot analysis country briefing sector briefings industry watch article detailed lifestyle report euromonitor international find executive bloomberg terminal locate business library jff company record mgmt function show company list age position long executive company investor relation company list executive investor relation google company investor relation finance usc require analysis company investable industry financial vpn vpn usc company record professional left column nexis university lexis nexis academic know executive company find executive personal career include orbis usc require company director manager advisor left navigation column professional association list allow professional association industry career jobstars careeronestop glassdoor association trend recent report resume future job career forecast trend future job report economic forum workplace trend aspirant technology trend deloitte mckinsey technology trend outlook big dream big challenge handshake employment social outlook trend international labour organization alumnus database usc library extend student borrow privilege remote database electronic resource semester academic term last semester enrollment training unable extend interlibrary loan eligibility graduate student period alumnus remote usc library database electronic resource alumnus eligible usc interlibrary loan alumnus encourage visit local library popular business resource los angeles library include database business insight essential abi inform data axle solution demographic hoover company resume mergent intellect mergent archive dossier morningstar global netadvantage srds statista value line hill library include database morningstar gale business insight global demographic usa data axle santa monica library include database morningstar referenceusa value line find library southern library cooperative library resource graduation accessible resource scholarly content additional borrowing privilege check alumnus borrowing policy additional check library policy business accounting library guide aim resource business relate topic training marshall usc additional contact operation contact faq</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>12</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>南加州大学—通用就业指南.docx</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
-        <is>
-          <t>南加州大学—通用就业指南.docx</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
         <is>
           <t>Home
 Career Resources Research Guide
@@ -2148,22 +2109,19 @@
 For additional information about access, please check our library policies page.</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>home career material guide job internship networking chance guide marshall business library list company industry company financials executive competitor industry information market size trend material search marshall career service school business career program undergraduate graduate business major link information marshall career service graduate career service career center career center career advice handshake enables job institution webinars network trojan trojan network student alumnus employer addition center usc career center advisor job skill department labor website skill salary program school certification search job listing data search job posting job company location data axle jobsinternship job material area tool resume interview tip estimate internship education advice job offer skill business experience master realworld business skill transition campus workplace module data analytics leadership communication professionalism search million job company employee job access tool job search company linkedin business medium platform network relationship skill career ebooks business career growth communication company company click searchfunding search date location company capital analysis company industry market news market insight company performance industry data screener database company equity business growth people criterion vpn vpnuscedu company industry screener screen company menu industry field search filter etc view result report company choose company profile news subsidiary industry news news company factiva information company industry article newspaper trade magazine press blog business forecaster diligence company mention news search field enter start company ticker company factiva expert search tab click news newsand language choice click search right industry market database content industry bcc measurement assessment market chance market industry technology consulting firm market area information communication technology aerospace defense healthcare chemical material food automation control measurement instrumentation electronics security energy power system transportation building technology downloading report student information technology company document form ibisworld industry market report industry risk rating state data market find market report type business cover market mintel report mintel trend consumer market analysis trend product database product data product food beauty care health hygiene home care pet market passport gmid market information database range consumer market industry information country world company analysis country briefing sector market industry watch article consumer lifestyle report find executive terminal business library jff company record mgmt function company management team list age position executive company investor relation company executive investor relation company investor relation capital analysis company industry market vpn vpnuscedu search company record peopleprofessionals column executive company executive information email search company director manager advisor navigation column association website association industrycareer jobstarscom careeronestop glassdoor directory association trend job trend link report future job career forecast future job report world forum workplace trend tech trend technology trend outlook dream challenge world job outlook institution alumnus database access library student privilege access database material semester term semester enrollment course interlibraryloan eligibility student period alumnus access library database material alumnus loan service alumnus library access business material angeles database business insight essential data axle reference solution demographic hoover company mergent archive morningstar netadvantage srds value line database gale business insight demographic data axle santa database morningstar referenceusa value line california material graduation information material content information borrowing privilege alumnus tab borrowing policy information access policy</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>career resource guide job internship professional networking guide usc marshall business account library build list company preferred industry specific company finance key executive competitor find industry trend identify university resource aid usc marshall career_services marshall university business robust career advise undergraduate graduate business major marshall undergraduate career_services usc marshall graduate career_services usc career usc career resume career advice network handshake enables job organization attend webinars network fellow trojan trojan network student alumnus employer addition usc university base career advisor assist job skill careeronestop sponsor department labor explore skill salary find university certification resume job listing data axle job posting job company data axle job internship module job resource area tool resume write interview tip salary estimate internship continue education advice relate job sage skill business practice master real business professional skill transition workplace module include data analytics entrepreneurship leadership organizational communication professionalism glassdoor million job company former employee job tool job_search resume company linkedin business employment focus social medium platform professional network build relationship skill succeed career iglibrary ebooks business career_development corporate communication company find company privco funding preferred find company fund finance analysis company investable industry financial contain financial insight company performance industry data screener large database company equity business criterion note vpn vpn usc find company industry screen quick screener screen company drop industry field continue remain filter geography result cap detail report company university lexis nexis academic find company locate resume include subsidiary finance swot industry find negative company factiva find company industry include article report trade magazine press release blog business forecaster conduct due diligence company require find negative mention field enter start company ticker pop company factiva expert sentiment negative language choice low right industry usc libraries subscribe databases industry specific database content span multiple related industry bcc bcc objective unbiased measurement assessment detailed report sullivan industry technology global consulting firm resume international area communication technology aerospace defense healthcare chemical material food industrial automation control measurement instrumentation electronics security energy power automotive transportation environmental technology single downloading entire report enable student gartner detailed technology advisory company report full text ibisworld industry report industry risk rating focus united state data global marketresearch academic find lengthy detailed report brief white describe business resume international mintel mintel report mintel trend comprehensive depth analysis trend mintel global product database include detailed product data product food drink beauty personal care health hygiene care pet passport passport gmid global database wide industry country include company resume swot analysis country briefing sector briefings industry watch article detailed lifestyle report euromonitor international find executive bloomberg terminal locate business library jff company record mgmt function show company list age position long executive company investor relation company list executive investor relation google company investor relation finance analysis company investable industry financial vpn vpn usc company record professional left column nexis university lexis nexis academic know executive company find executive personal career include orbis company director manager advisor left navigation column professional association list allow professional association industry career jobstars careeronestop glassdoor association trend job trend recent report resume future job career forecast trend future job report economic forum workplace trend aspirant technology trend deloitte mckinsey technology trend outlook big dream big challenge handshake employment social outlook trend international labour organization alumnus database usc library extend student borrow privilege remote database electronic resource semester academic term last semester enrollment training unable extend interlibrary loan eligibility graduate student period alumnus remote usc library database electronic resource alumnus eligible usc interlibrary loan alumnus encourage visit local library popular business resource los angeles library include database business insight essential abi inform data axle solution demographic hoover company resume mergent intellect mergent archive dossier morningstar global netadvantage srds statista value line hill library include database morningstar gale business insight global demographic usa data axle santa monica library include database morningstar referenceusa value line find library southern library cooperative library resource graduation accessible resource scholarly content additional borrowing privilege check alumnus borrowing policy additional check library policy</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>卡内基梅隆大学-10本就业指南 职业与就业研究指导.docx</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
-        <is>
-          <t>卡内基梅隆大学-10本就业指南 职业与就业研究指导.docx</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
         <is>
           <t>Start your Research
 About this Guide
@@ -2306,22 +2264,19 @@
 The Career and Professional Development Center (CPDC) is Carnegie Mellon University’s centralized career services center. We provide a comprehensive range of services, programs, and materials focusing on career exploration, professional development, experiential learning and employment assistance to meet today’s evolving workplace and student goals of finding satisfying work!</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>guide guide print material variety career job library tandem cmu growth center cpdc book material topic jobcareer exploration tab guide material employer interview graduate education material book recommendation topic career book hundred book career exploration resume kind occupation catalog try job guidance title book recommendation keyword field career statistic mather doganaksoy gerald hahn career ebook aaron bayles johnny foster christopher klaus foreword brindley ebook wood peter petocz anna career planning bioscientists sarah blackford basic outlook guide bureau labor statistic editor publication date encyclopedia career guidance staff contribution dream job ideal career college leibman publication date color parachute manual jobhunters careerchangers richard bolles publication date employer company hoover hoover list company competitor hand side downloading company axle module company consumer data job posting healthcare office listing business filing data visualization mapping submission depth onesource module information firm company financials information deal valuation venture capital equity etc company investor intelligence note account cmu email database purpose insight database company investor activity contains search company investor deal information equity venture capital news market material startup note account cmu email salary relocation information salarycom climbtheladder glassdoor job listing hundred cmu handshake handshake recruiting platform find job internship chance company career option job internship job internship area check material cpdc job search site job trend data thousand job government site job field internshipscom marketplace internship job search site data job listing job chronicle education hnet job announcement humanity science job historian job association advancement science nonprofit hoover hoover link window company listing institution kind leadership leadership library link window institution kind contact information profile information financials nonprofit advantage register search result institution university center center petersons prep guide experience test school exam gre toefl school search feature user account access content interview prep employer background hoover hoover company nonprofit leadership history financials product marketline company section swot analysis glassdoorcom million user report cover company salary experience information company guide cpdc material interview platform student experience interview skill interview training mock interview industry job experience level cmuniverse cmuniverse mentoring platform student alumnus alumnus group group carnegie mellon student faculty staff network share job chance business venture touch interview prep industry field ibisworld link window industry market report analysis data condition segmentation market share company outlook link window market report analysis technology aspect industry industry defense chemical consumer product electronics healthcare report pdfs material industry guide discover contact leadership leadership library link window people company nonprofit government medium law etc phone bios researcher expert government agency institution association job association membership job board word finance association pittsburgh pittsburgh association career book interview guide sudheer jonna publication date system design interview publication date data engineering interview kedeisha bryan taamir ransome publication date graduate education graduate school exploration school guide prosanta chakrabarty school science kersey relles book experience test school info petersons prep guide experience test school exam gre toefl school search feature user account access content doctor of philosophy job exploration guide career linder kevin tobin publication date book career book topicarea cmu library cmu career growth center cpdc book cmu faculty staff student book print sampling title topic area interest career exploration speaking communication management leadership dei ask question faq answer question library location material search option arrow option enter show book library video camera equipment eat schedule consultation people university submit ticket coding data science project data support link scroll bottom consultation team career growth center career growth center cpdc mellon career service center range service program material career exploration growth learning job assistance today workplace student goal work</t>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>start guide guide design find print electronic resource career job cmu library tandem cmu career professional cpdc collect book resource topic job career exploration check various guide contain resource find employer interviewing networking graduate education resource book recommendation topic career book book book interview career exploration network resume kind job find library catalog try job hunt vocational guidance check additional title book recommendation keyword field examples career statistic ebook mather necip doganaksoy gerald hahn infosec career hack ebook aaron bayles chris hurley johnny foster christopher klaus foreword brindley mathematician ebook leigh wood peter petocz anna reid career planning bioscientists book sarah blackford basic occupational outlook handbook bureau labor statistic editor article encyclopedia career vocational guidance ferguson publish staff contribution dream job ideal career university pete leibman article color parachute practical manual job hunter career changer richard bolles article find employer company listings hoover build list find company interested check competitor left hand side international downloading company resume data axle various module canadian company sizes data job posting healthcare office personal listing business filing data visualization mapping application depth onesource module extensive corporate global firm privco company finance deal valuation venture finance equity company resume good locate investor competitive intelligence note account cmu database academic purpose insight comprehensive global database company investor activity contains advance company investor deal equity venture finance great emerge excellent resource startup entrepreneurship note account cmu salary relocation salary climbtheladder glassdoor job listing seem recommended cmu handshake handshake cmu recruit platform allow explore find apply job internship connect great company career option pittsburgh job internship cpdc job internship local area check resource cpdc comprehensive international job_search give salary employment trend data usajobs job government official federal employment field internships large internship include pay unpaid full internship comprehensive international job_search give salary data academic job listing job advertise chronicle higher_education net job guide announcement humanity social science job historian scientist job american association advancement science nonprofit hoover hoover company listing contain nonprofit organization kind leadership connect leadership library international major organization kind extensive contact quick resume guidestar full include finance nonprofit full advantage free advance best result idealist nonprofit organization university peterson test prep guide practice test graduate_school exam mcat gmat lsat gre toefl graduate_school feature account content interview network interview prep employer background hoover hoover international company nonprofit brief description leadership history finance product marketline datamonitor find company section leave swot analysis glassdoor base million report resume specific company salary interview experience job check company guide cpdc interview networking resource big interview digital platform cmu student practice interview skill big interview hand training mock interview tailor specific industry job experience cmuniverse cmuniverse virtual mentoring platform student want engage alumnus cmu alumnus linkedin carnegie mellon alumni student faculty staff network share job start business venture touch interview prep industry field ibisworld industry report analysis data segmentation share primary company outlook sullivan report analysis technology aspect industry industry include aerospace defense automotive chemical product electronics healthcare report pdfs resource academic purpose industry guide network discover background locate contact leadership connect leadership library important company nonprofit government medium law include phone bios pivot researcher expert universities government agency organization network professional association job association support find student membership forget job board try google key word finance association pittsburgh turn pittsburgh association financial professional book interview react interview guide sudheer jonna andrew baisden article ace design interview zhiyong tan article crack data engineering interview kedeisha bryan taamir ransome article graduate education graduate_school exploration graduate_school amanda seligman guide academia prosanta chakrabarty graduate_school science kersey sturdivant noelle relles test book practice test graduate_school peterson test prep guide practice test graduate_school exam mcat gmat lsat gre toefl graduate_school feature account content doctor of philosophy job exploration alt guide alternative academic career kathryn linder kevin thomas tobin article recommend book career book topic area cmu library cmu career professional cpdc job updated career relate book cmu faculty staff student book print sampling title add different topic area interest check career exploration speaking communication leadership dei interview networking ask ask consult faq answer frequent library resource option arrow browse option enter show return library book library close borrow video camera multimedia equipment eat drink library schedule consultation find departmental librarian job university libraries sure meet submit ticket coding data science project data code support scroll bottom schedule consultation career professional career professional cpdc carnegie mellon university centralize career_services comprehensive material focus career exploration professional experiential learning employment assistance meet today evolve workplace student goal find satisfy job</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>卡内基梅隆大学-就业指南.docx</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
-        <is>
-          <t>卡内基梅隆大学-就业指南.docx</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
         <is>
           <t>Home
 Need more help?
@@ -2470,22 +2425,19 @@
 Tepper Guide</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>home need question person phone email university reference team form hour oneonone consultation library workshop semester visualization management check list workshop register cmu guide guide material strategy employer interview material guide contain information industry business trend company type information swot analysis analyst report guide tab link find information career interest create list target company industry location size criterion companiesstartups industry trend data news trade journal company industry business economics splenda email book meeting contact hunt carnegie mellon university street pittsburgh subjectsbusiness career campus economics management reference career investiage career salary data amount data agency overview career data trend projection material analysis career interest outlook guide ooh info hundred career data requirement outlook information work environment department labor data info careersoccupations people career video career job salary data information network onet data occupation activity data info job opening outlook bureau labor statistic article data career trend target company list company criterion insight insight link window database company investor activity contains search company investor deal information equity venture capital news market material startup note account cmu step search right corner company option criterion interest list criterion side criterion list edit button company list check box icon company download option ribbon top note row data user year capital capital link window financialvaluation data material information equity credit rating transaction hundred data point list company market executive excel plugin data analysis account cmu email address direction capital user pittsburgh campus step company criterion interest order list criterion center box criterion add criterion order function criterion view result button right info list customize display column tab display info procedure step excel icon result popup window download link spreadsheet note downloading row data time hoover hoover link window firm company industry overview financials analyst report lot information note yer campus step company list select criterion interest order list criterion side criterion select view result button right company download button list note limit downloads year data data module company business filing consumer lifestyle data visualization mapping good company step business search tab criterion interest order list criterion side click count button result list view result button result company download button list result max company time downloads company company profile material information company financials executive business segment product service competitor capital link window financialvaluation data material information equity credit rating transaction hundred data point list company market executive excel plugin data analysis account cmu email address direction capital user pittsburgh campus value line investment survey link window stock report performance projection ranking analyst consensus beta ratio industry source swot weakness chance threat hundred company position industrymarket health stability datamonitor link window report company industry country swot force analysis deal investor database market data consumer product analyst report analyst company basis report information health direction business competition hoover link window company company analyst report side company company information lot information firm database specialize information startup company place employer space insight link window database company investor activity contains search company investor deal information equity venture capital news market material startup note account cmu email privco link window company financials information deal valuation venture capital equity etc company investor intelligence note account cmu email database purpose industry data stats link window market industry company statistic report dossier format easytouse bls industry glance workforce compensation price industry data production quantity value nation industry material overview hundred industry information industry size revenue projection player ibisworld link window industry market report analysis data condition segmentation market share company outlook state datamonitor link window select industry profile menu access hundred industry report perspective industry link window background intelligence report kind industry term industry solar search box refine report valuation multiple industry report material report niche industry market coverage technology healthcare manufacturing iot sphere link window market report analysis technology aspect industry industry defense chemical consumer product electronics healthcare report pdfs material link window market report industry material biotechnology chemical energy healthcare sensor plastic nanotechnology technology industry gartner core link window analysis forecasting information technology product service report subscription cmu qatar subscription newsliterature trade journal journalspublications information company industry product service way happening field database access trade journal literature publication type journal newspaper magazine collection link window article industry source periodical report dissertation business management strategy landscape database guide business source premier link window industry periodical business discipline industry company country report business news access business news platform interface sign account cmu email address street journal dow jones link window article business newspaper platform content year backfiles affiliate account cmu address wsj app login access york time access pas link window access york time account logging cmu student access december graduation year faculty access year time account visit link walk direction activation pittsburgh business time link window company business news list business industry note access change user logon email click link right click create account mark box pittsburgh business time access account access link andrew email password guide</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ask ask person phone mail contact university libraries fill library consultation library workshops library training semester conduct literature data visualization check list training cmu libraries training guide guide contain library resource strategy prospective employer prepare interview resource guide contain industry business trend specific company include swot analysis analyst report navigate guide find career interest list target company industry criterion investigate company startups understand analyze industry trend data find trade article company industry business economics librarian ryan splenda book meeting contact hunt library carnegie mellon university libraries frew pittsburgh social linkedin subject business career cmu pittsburgh economics career investiage career salary data great amount data various governmental agency overview various career salary data trend projection resource give high analysis career interest occupational outlook handbook ooh different career include salary data educational requirement outlook job environment careeronestop department labor data different career job include career quick video career project employment salary data occupational network net data various job include job related activity salary data job opening career outlook bureau labor statistic article data career economic trend target company list locate company want job accord specific criterion insight insight comprehensive global database company investor activity contains advance company investor deal equity venture finance great emerge excellent resource startup entrepreneurship note account cmu advanced upper right corner sure company option criterion interest build list criterion locate left hand side criterion add list refine edit columns add subtract company list check icon company option green ribbon appear top note row data finance finance depth financial valuation data resource include equity credit rating transaction data generate list company executive include excel plug data analysis account cmu address follow direction finance pittsburgh screen top company criterion interest order build list criterion locate multiple add criterion sure add criterion order execute function criterion added result upper right additional list desire customize display column browse display columns additional procedure outline excel icon result pop appear excel spreadsheet note unlimited downloading row data hoover hoover resume global firm company industry overview swot finance analyst report lot note yer entire judicious follow build company list apply criterion interest order build list criterion locate left hand side criterion added blue result upper right check company wish blue format list note limit downloads judicious data referenceusa data various module canadian company directories business filing lifestyle data visualization mapping good company follow business database advanced criterion interest order build list criterion locate left hand side blue update count refresh result list green result result check company wish format list result note max company limit total downloads company detail company resume resource depth robust detailed company finance ratios executive business segment product competitor finance depth financial valuation data resource include equity credit rating transaction data generate list company executive include excel plug data analysis account cmu address follow direction finance pittsburgh value line investment survey stock report financial performance projection ranking analyst consensus beta key ratio commentary short industry survey classic swot analyse strengths weakness threat company inform company position industry overall health stability marketline datamonitor report company industry country contain swot force analysis financial deal investor statistical database data product analyst report analyst evaluate company regular basis report contain detailed company financial health direction business stand competition hoover resume company company analyst report left side company non trade company difficult gain disclose lot trade firm database specialize start ups company good specific prospective employer operate insight comprehensive global database company investor activity contains advance company investor deal equity venture finance great emerge excellent resource startup entrepreneurship note account cmu privco company finance deal valuation venture finance equity company resume good locate investor competitive intelligence note account cmu database academic purpose industry quick data stats statista industry company demographic statistic data report dossier downloadable various format international easy bls industry glance workforce compensation price establishments trends international industry data industrial production physical quantity monetary value united nation industry overviews resource depth overview establish specialized industry include industry revenue projection trend major player ibisworld industry report analysis data segmentation share primary company outlook china state marketline datamonitor industry resume drop industry report several geographic perspective industry resume background intelligence report kind industry enter term describe industry solar refine find recent report valuation multiple industry specialize niche report resource find report specialized niche industry good coverage technology healthcare advance manufacturing iot specialized sphere frost sullivan report analysis technology aspect industry industry include aerospace defense automotive chemical product electronics healthcare report pdfs resource academic purpose bcc report industry specialize advanced material biotechnology chemical energy healthcare sensor plastic nanotechnology emerge technology traditional industry gartner core analysis forecasting technology product note dataquest report subscription cmu qatar include subscription literature trade article trade article article contain great company industry trend product great stay happening field database trade article literature article academic article report magazine abi inform collection article industry scholarly periodical report dissertation business corporate strategy competitive landscape database guide business premier academic industry periodical business discipline industry company country report business several business platform native interface sign personal account cmu address wall article dow jones article major business report wsj platform content include roll backfiles cmu affiliate initial account cmu andrew address wsj app digital academic pas require account logging cmu address student last december graduation faculty last authenticate nyt account authenticate visit walk direction activation pittsburgh business western company business list top local business industry note change logon end andrew cmu sign upper right free account continue mark pittsburgh business account sign andrew password tepper guide</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>哈佛大学-资源列表.docx</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
-        <is>
-          <t>哈佛大学-资源列表.docx</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
         <is>
           <t>Library Resources for Your Job Search
 Getting Help
@@ -2582,22 +2534,19 @@
 Search using using terms like jobs or internships.</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>material job search guide article book job search industry company think tank search tool access directory information institution government company tool institution submission job interview office career advancement career_advancementhksharvardedu hks service create account alert access post graduation countryspecific career job info internship job posting listing profile regulation resumecv guideline advice directory government leadership harvard login contact data staff company government agency office law firm news medium outlet institution nonprofit click button return access login database contact information congress staff material medium activity news report executive order press release almanac politics login directory agency administration staff account list account association leadership harvard login contact data staff company government agency office law firm news medium outlet institution nonprofit click button return access guidestar login guidestar information institution charity foundation information information trend analysis leadership information governance experience compensation data demographic encyclopedia association search series encyclopedia association institution encyclopedia association association state address description society trade association labor union institution fan club group type center login information government university institution world login database institution institution yearbook institution database institution type institution structure network body club leadership harvard login leadership directory contact data hundred thousand thought leader america email phone address background information directory institution profile information company government agency office law firm news medium outlet institution nonprofit capital login ciq people intelligence screen company executive board member company jobboard function education criterion registration consultant institution directory harvard firm individual section field activity agriculture specialty finance computer boardex harvard detail company board board director manager company globe network director time spent institution database screen education university kennedy school government account librarian material account company industry company orbis harvard login company database unique breadth geography extent company availability company information emis harvard country company information source market asia europe east country material country profile statistic forecast analysis report market company industry rate analyst report business news preqin harvard login information equity venture capital company fund deal industry harvard login report growth food energy healthcare transportation technology industry integrates topic data fact source platform source information market researcher publication journal government database book article collection harvard login abiinform summary citation management marketing business journal sample search job interview search box select drop menu search result publication date business source harvard login database citation summary text article journal magazine trade publication search job interview search box term drop menu search result publication date career growth book career growth login collection ebooks aspect career growth job resume cover letter communication skill interview tip addition hks library harvard range title example compassionate career living difference harvard loginby jeffrey pryor alexandra mitchell information career field story people career path job harvard whiteman guide government job internship fellowship tip template submission directory internship management training program fellowship interview harvard loginby jay light chance impression job element style harvard loginby scott bennett reader compelling résumés cover letter growth assistance print onlyby maia gedde career guide growth emergency sector etiquette advantage business print onlyby peter post anna post lizzie post daniel post guide business etiquette attire communication world print onlyby jonathan larry powell aspect technique job interview interview question employer answer employee dianna podmoroff variety question employer job seeker search search term job internship</t>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>library resource job_search guide find article book job_search various industry company useful think tank tool databases organization government company tool identify target organization prepare application job interview office career advancement career_advancement hks harvard hks library library_research hks harvard goinglobal account set alert continue post graduation country specific career employment internship job posting employer listing corporate resume job permit regulation cross cultural resume guideline interview cultural advice government leadership connect harvard contact biographical data staff company government agency congressional office law firm medium outlet healthcare organization nonprofit attempt sign prompt say return legistorm comprehensive database contact biographical congress congressional staff resource include social medium activity report executive order press release almanac american politics congressional federal agency administration staff account export list excel contact account association non profit leadership connect harvard contact biographical data staff company government agency congressional office law firm medium outlet healthcare organization nonprofit attempt sign prompt say return guidestar guidestar irs recognize organization include charity foundation include historic financial financial trend analysis historic leadership governance practice historic compensation data organizational demographic encyclopedia association harvard different include encyclopedia association international organization encyclopedia association national encyclopedia association regional state local address description professional society trade association labor union cultural religious organization fan club harvard government university independent nonprofit organization europa harvard database resume academic institution cultural scientific educational organization yearbook international organization searchable database international organization organization include formal structure informal network professional body recreational club corporate leadership connect harvard leadership contact biographical data thought america phone address background base depth organization resume verify contact company government agency congressional office law firm medium outlet healthcare organization nonprofit finance ciq intelligence screen company executive board member company job board function education criterion registration require consultant consult organization harvard firm list arrange subject section field consult activity agriculture specialty represent include finance computer fund raise boardex harvard full detail company board board director senior manager company globe network director map base spend organization database update screen education include harvard university harvard kennedy university government account require ask librarian determine right resource set account company industry company orbis harvard global company database unique breadth geography extent company resume availability company financial emis harvard country company emerge africa asia europe middle east arrange country resource include country resume macroeconomic statistic forecast analysis report financial company industry exchange rate analyst report business preqin harvard equity venture finance company fund deal industry harvard report major economic scientific technological food energy healthcare transportation technology industry statista integrates diverse topic data fact single platform include researcher trade article scientific article government database article book article inform collection harvard abi inform summary citation academic marketing business article hks alumni sample employment interview subject head adjoin drop conduct sort result article recent business complete harvard database citation summary full text article academic article magazine trade article sample employment interviewing subject term adjoin drop conduct refine result article career_development book library career_development harvard extensive collection book aspect career_development job write resume resume resume communication skill interview tip addition hks library harvard wide career relate title compassionate career living difference harvard jeffrey pryor alexandra mitchell find career idealistic field include personal story follow career path land top pay federal job harvard lily madeleine whiteman guide secure government job internship fellowship include tips template write win application expand internship track training fellowship late helpful websites suceed interview harvard jay show best possible light maximize chance brilliant impression job element resume style harvard scott bennett show craft clear compelling target resume resume job job international humanitarian assistance print maia gedde career guide interested international humanitarian emergency sector post etiquette advantage business print peter post anna post lizzie post daniel post senning classic guide business etiquette resume proper attire effective communication interview changing print jonathan amsbary larry powell resume aspect interview technique include limit job interview great interview employer best answer prospective employee print dianna podmoroff contain wide word employer job seeker think term job internship</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>16</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>哈佛大学-针对法律.docx</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
-        <is>
-          <t>哈佛大学-针对法律.docx</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
         <is>
           <t>Employer Research
 How to research employers whether for EIP, judicial clerkships or any other job search.
@@ -2797,22 +2746,19 @@
 You may reproduce any part of it for noncommercial purposes as long as credit is included and it is shared in the same manner.</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>employer employer clerkship job search service law school service law school material career interview clerkship source place harvard law school office career service material job search question job search office interest career service office interest law appointment harvard law student alumnus attorney advisor material interest career job harvard law school website access material information employer clerkship clerkship clerkship similarity law firm job way submission clerkship deadline step component search harvard law office career service clerkship interview overview clerkship submission material clerking judge judge clerkship interview library directory print online information judge book bench bench publication judge print almanac judiciary almanac judiciary publication lawyer comment print library catalog hollis search feature keyword subject drop menu search statesdirectories judge book material judge judge university cincinnati learn judge tool type judge tool sense pattern decisionmaking westlaw litigation analytics judge tool information majority district court state court judge litigation analytics coverage information lexis litigation analytics judge information district court state court judge user judge behavior courtroom trend time district court bloomberg law clerkship material collection material clerkship opening prepare interview judge offer judge opinion interview thought analysis argument opinion judge westlaw lexis database search julastname jufirstname judgeslastname judgesfirstname lastname learn court judge place court structure court webpage information court structure contact information court website state court court strategy decision judge court system conversation law firm lawyer law firm data law firm interview interview question step interview firm overview law firm view statistic law firm start harvard career service employer directory employer intelligence compass focus experience area field investigate firm work material field market law property finance news firm experience area vault firm experience area interviewer firm client ranking lexis westlaw source lawyer law firm directory information law firm attorney martindale hubbell westlaw profiler information attorney judge expert arbitrator property career link document work history news database transaction client firm ranking law firm law firm ranking guide ocs law firm ranking law firm law firm ranking guide guide survey ranking search feature hollis information law firm search keyword subject drop menu search law office state directory eip statistic interview program interview program information hiring experience eip statistic evaluation information year eip law litigation litigation experience employer institution type law lobbying firm government state association nonprofit leadership connect lawyer region law school criterion visit job leadership interest interest chance interest job site material office interest aid defender service career access justice job justice work law firm transaction financing guide governance security regulation law governance lilliott rydin view year security regulation enforcement lilliott rydin view year sec filing contract language deal transaction equity issuance governance issue proxy law list filing law edgar search firm equity venture capital hedge fund guide venture capital equity fund venture capital equity cynthia churchwell sep view year equity venture capital hedge fund lisa lilliott rydin sep view year prequin tool financing stage region role deal region deal information firm lawyer search navigation template search employer material congress form book state committee jkb publication date directory michael call isbn publication date government website contact information directory representative information directory addition information senator representative source assistant secretary court official establishment department agency government official governor state territory diplomat member press radio television gallery contact information legislator staff member leadership youd legislator start member youll option way search location party affiliation area interest location party affiliation search factor location party affiliation staff search legistorm congress leadership area interest experience legislator area expertise legislator interest committee caucus part interest service information leadership connect list area expertise search search policy area legistorm committee member committee caucus member caucus education institution interviewer conversation question information interviewer employer leadership connect school link select education law search suggestion drop menu legistorm search staff institution background issue news issue jurisdiction legislator awareness source issue policy tracking tool area legistorm news news capitol hill legistorm eye feed tweet post reason interest amusement concern medium account offer link medium account facebook twitter staffer section medium information legistorm function update press release account member congress trending hashtags town meeting town meeting way constituent information town meeting material town hall event town hall legistorms tip town hall business nonprofit business list industry nexis company dossier spreadsheet employer criterion subsidiary etc size revenue sale employee industry description scope country state city zip code company guide tip company industry market lilliott rydin view year kennedy school material job search byu business career guide encyclopedia association industry information institution mission association institution trade publication publication website publication search title harvard library catalog guide enterprise guide question knowledge base chat researchlawharvardedu contact collection meet online consult hour hour class calendar license guide common state part purpose credit manner</t>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>employer employer eip judicial clerkship job_search guide harvard law_school library start start harvard law_school resource legal career prepare interview apply judicial clerkship great start harvard law_school office career_services ocs resource job_search answer specific job_search bernard koteen office interest advise hls career_services office specialize interest law advise appointment harvard law student alumnus attorney advisor resource plan interest career land job harvard law_school library material gather background potential employer judicial clerkship judicial clerkship apply judicial clerkship similarity apply law firm job different application clerkship rigid important start miss important deadline start component clerkship apply familiarize harvard law office career_services judicial clerkship interview_process find overview clerkship application resource decide clerking right specific judge judge important decide clerkship apply early speak interview library judicial print judge judicial yellow book american bench american bench include representative article lead judge print library almanac federal judiciary almanac federal judiciary include article blurbs lead lawyer comment print library try library catalog hollis advanced feature hollis replace keyword subject drop judge united state judge interested find book write additional resource judge compile judge guide university cincinnati interview judge analytical tool judge hear tool sense pattern decision westlaw litigation analytics judge tool majority district court state court judge westlaw litigation analytics coverage lexis litigation analytics judge district court state court judge allow compare judge behavior courtroom trend federal district court know expect bloomberg law clerkship resource collection resource find potential clerkship opening prepare interview judge succeed land judge want discuss opinion interview examine thought listen analysis legal argument find representative opinion judge westlaw lexis database following westlaw lastname firstname lastname lexis judge lastname judge firstname lastname court judge want understand court structure check court court structure contact recent federal court state court websites recent court good strategy notable decision judge court come conversation understanding recent useful law firm lawyer law firm data prepare law firm interview require decide interview prepare ask good guide prepare interview_process comfortable firm overview relevant law firm key statistic law firm start harvard career_services employer nalp legal employer alm intelligence legal compass focus practice area know want job specialized field investigate firm job additional resource include specific field corporate law intellectual property finance firm practice area vault firm practice area interviewer firm client ranking lexis westlaw rich lawyer law firm law firm attorney find martindale hubbell westlaw next profiler biographical attorney judge expert arbitrator intellectual property professional report reflect job history want legal database recent transaction representative client firm meet ranking law firm try law firm ranking guide ocs include law firm guide ranking law firm try ocs law firm ranking guide vault guide alm survey ranking advanced feature hollis law firm advanced replace keyword subject drop law office united state check past eip statistic harvard conduct early interview hls early interview past hiring practice eip statistic evaluation past several eip harvard law litigation litigation practice potential employer organization law lobbying firm government federal state local association nonprofit visit leadership connect find lawyer law_school criterion visit job_searching leadership interest interest find interest job follow resource office interest advise list national legal aid defender association public_service legal career justice job equal justice job impact fund transactional law firm advise sec transaction include financing start consult guide corporate governance security regulation corporate law corporate governance lisa lilliott rydin last updated aug security regulation enforcement lisa lilliott rydin last updated aug sec filing contract precedential language deal transaction include equity issuance governance issue corporate proxy bloomberg law contain curated list sec filing edgar bloomberg law edgar firm advise equity venture finance hedge fund start consult guide venture finance equity hedge fund venture finance equity cynthia churchwell last updated sep equity venture finance hedge fund lisa lilliott rydin last updated sep prequin tool financing work narrow deal specific deal give firm lawyer advanced left navigation template customize prequin legislative legislative employer resource congress congressional yellow book united state congress joint committee print call isbn article official congressional michael call isbn article government following congressional contact representative senate contact congressional addition senator representative contain congressional administrative assistant secretary court official military establishment federal department agency government official governor state territory foreign diplomat member press radio television gallery contact biographical legislator staff member visit leadership connect legistorm apply know job legislator good start member congress narrow option effective narrow include party affiliation area interest party affiliation limit factor include party affiliation advanced staff legistorm congress advance leadership connect area interest leverage experience focus legislator job area expertise determine legislator interest consider committee serve caucus listed interest compile leadership connect build list limit base area expertise advanced limit key policy area legistorm locate committee member committee caucus member caucus interview education organization diligent connect interviewer conversation ask insightful consider biographical interviewer potential employer leadership connect university education harvard law suggestion drop legistorm advance find legislative staff educational institution military background issue useful aware issue relevant jurisdiction legislator job find awareness politicopro subject base issue policy tracking tool multiple area legistorm curates capitol hill legistorm catch eye feed long tweet short blog post daily reason interest amusement concern social medium account legistorm verify staffer social medium account include linkedin facebook twitter staffer biographical section social medium legistorm compile legistorm stormfeed function update press release twitter account member congress relevant trending hashtags town hall meeting town hall meeting unique legislator constituent care town hall meeting following resource legistorm town hall event legistorm town hall faqs legistorm tip town hall business non profit business customized firm list industry nexis university company dossier nexis customized spreadsheet employer base different criterion include subsidiary base revenue sale employee industry description sic naic geographic scope country state city zip code company consult following guide additional tip company industry lisa lilliott rydin last updated aug kennedy university library resource job_search byu business career guide non profit encyclopedia association industry specific organization mission association organization support trade article find article visit specific specific article title harvard library catalog consider explore follow guide library social enterprise guide contact ask submit knowledge base chat chat librarian law harvard contact historical special collection specialc law harvard meet schedule consult librarian library training train calendar license guide license creative common attribution noncommercial share united state license reproduce noncommercial purpose credit include share manner</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>哥伦比亚大学 研究生实习项目.docx</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
-        <is>
-          <t>哥伦比亚大学 研究生实习项目.docx</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
         <is>
           <t>Job &amp; Internship Opportunities
 The Graduate Student Internship Program in Primary Sources is designed to enrich graduate studies and professional training in primary sources through an introduction to archival work, supplemented with a program of lectures, workshops and tours.  Participating Columbia University Libraries include the Avery Architectural &amp; Fine Arts Library, the Burke Library at Union Theological Seminary, and the Rare Book &amp; Manuscript Library.  Graduate or professional students, currently matriculated at Columbia University, are eligible to apply.  This is a paid internship. For more information and application guidelines, please see the Internship Program in Primary Sources page. 
@@ -2820,22 +2766,19 @@
 The Ask a Librarian Internship provides current and recently-graduated library school students with hands-on experience in various areas of academic librarianship. Interns will receive training and support from a librarian supervisor in order to assist users through the Ask A Librarian chat reference service. Additionally, interns will work with their supervisor to conduct a specific project, which can be conducted remotely or in-person, such as designing and delivering a workshop session, creating topical research guides, or processing special collections. For more information and application guidelines, please visit the Ask a Librarian Internship Program page.</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>job internship graduate student internship program source graduate training source introduction work program lecture workshop tour university library fine art burke library union seminary book manuscript graduate student columbia university internship information submission guideline program source program student librarian technologist scholarship campus student applicant stipend handson experience field publishing humanity music data information submission guideline program ask internship school student experience area librarianship intern training support supervisor order user ask chat reference service intern supervisor specific project workshop session guide collection information submission guideline ask internship program</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>job internship graduate student internship primary design enrich graduate professional training primary introduction archival job supplement lecture training tour participate columbia university library include avery architectural fine art library burke library union theological seminary rare book manuscript library graduate professional student matriculate columbia university eligible apply paid internship application guideline internship primary digital internships graduate student wish collaborate librarian technologist job digital scholarship student recruit competitive successful applicant receive stipend hand experience job field digital publishing digital humanity digital music compute digital data geospatial application guideline visit digital internships ask librarian internship graduate library university student hand experience various area academic librarianship intern receive training support librarian supervisor order assist ask librarian chat intern job supervisor conduct specific project conduct person design deliver training session topical guide special collection application guideline visit ask librarian internship</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>埃默里大学 通用型.doc</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
-        <is>
-          <t>埃默里大学 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
         <is>
           <t>Career Services
 Target Company Lists
@@ -3212,22 +3155,19 @@
 Military to Civilian Careers</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>career service company company target industry list firm top mind list company database firm target location industry target company criterion atozdatabases company create custom target list business profile geography industry size result hoover bradstreet create custom target list worldwide business geography industry revenue company profile analysis pitchbook netid firm deal industry financing history startup venture capital company mature firm company operation create custom list firm presence country result ranking survey book list business journal book list company ranking firm employer industry leader netid rank employer internship variety business area year finance consumer product street oasis netid ranking banking race gender veteran status varsity athletics place employee choice award winner employee culture mit sloan culturex data rank firm agility collaboration customer diversity execution innovation integrity performance forbes employer diversity survey partnership employer employee class company class category company institution result progress category representation succession workplace inclusion retention accountability board diversity netid company ranking variety industry data market researcher institution government data workspace netid search screen company criterion dei rating firm strategy thomson poor netid industry profile list market leader industry visa strategy job search visa company visa past approach student company list list cross custom target list firm target industryfunctiongeography interest target company list company year government data source firm visa past data range position search company visa goinglobal data department labor employer data hub company state citizenship immigration service employer data hub firm visa employer data hub file list download csv list firm job title prevailing wage link slide data data sort classification business school student pilot physician professor file emory log firm location company operation create list company operation country country region state company industry code revenue result information address contact sale employee subsidiary operation contact information operation subsidiary affiliate branch emory netid identify company parent subsidiary location company parent company source directory affiliation country state example parent spain state salary negotiation benchmarking compensation data variety material compensation data company industry survey data self data street oasis netid finance career material interview course peer company interview insight data focus finance service firm data data point submission offer letter statement etc comparablycom self company culture data focus tech industry company industry data salarycom compiles salary methodology search calculator job function experience level geography data range entry level level position methodology indeeds search compiles salary employee user job advertisement month idea range target city industry ziprecruiter calculator information employer job title location ziprecruiter salary transparentcareercom filter program type location registration level information specific report fee job seeker calculator information association college employer guide finance accounting register download data labor certification government data source firm visa past data range position data company visa data labor certification data center department labor labor certification flc data center disclosure file list firm visa past compensation data disclosure data excel criterion data data sort classification business school student pilot physician professor file emory log bba range master of business administration range msba range metro area bureau labor statistic bureau labor statistic breadth data compensation chart cover state area compensation data compensation survey wage state data set employer cost employee compensation ecec series goodcalculators calculator state calculator data job statistic survey data state metro area cover occupation negotiation ace negotiator conflict york time job offer street journal linkedin learning course job offer human resources min min negotiator woman experience negotiation essential job negotiation business negotiation color parachute difference cost data cost account city suburb northeast southwest bankrate cost calculator data point cost criterion calculator salary geography ranking variety quality life consideration cost index metro area school data point guide exploration target company malisa andersonstrait jul view year negotiation malisa andersonstrait jan view year job search strategy visa malisa andersonstrait sep view year career malisa andersonstrait feb view year career malisa andersonstrait feb view year executive job search malisa andersonstrait jan view year program malisa andersonstrait sep view year job searching networking malisa andersonstrait jan view year cover letter malisa andersonstrait year malisa andersonstrait jan view year interview malisa andersonstrait jan view year time job search malisa andersonstrait feb view year program list program program login open company program list overview type program point master of business administration exchange growth program ranking program industry geography email ranking search strategy program job board filter leadership growth program slice program time idea example experience glassdoors program linkedins program job list program powersearch command google program term functionindustry interest supply chain logistics internship sitecom operation leadership growth sitecom program filetypepdf time job search position job posting handshake material search bit start mark dalton book hour job search cover hour job search dalton hour job search forum linkedin forum job site job board position youre resume type position skill job alert million posting association job site company job search browse job function location work remoteio posting startup company location benefit posting work posting management finance sale marketing programming design position focus tech marketing sale keyword search master of business administration role finance marketing sale role data analytics marketing human resources operation finance startup search master of business administration role sale workingnomads search master of business administration position education finance health care human resources marketing sale bbas aftercollege job alert area youre alert grad college recruiter internship grad master of business administration msbas career data science graduate degree position search industry role work irelaunch site material program job board individual work career break veteran job goizueta job site member family resume search occupation code employer individual disability filter state industry site employer individual veteran disability posting posting entry level career fair program college student disability internship time position agency student graduate employer award magazine careerguidance recruitment people disability graduate level position industry job board industry career guide career guide job site target industry association netid state institution irs data association job posting event career netid career guide company ranking finance estate marketing energy industry workplace therapist inventory job workplace therapist brandon smith linkedin career change course skill value strength career transition material career network wsjs email challenge harvard business knowledge jaymin patels blog tip trick advice leader master of business administration world linkedin search networking course secret networking min network min alumnus meet student alumnus company youre alumnus community school linkedins alumnus group goizueta group group interest search goizueta alumnus city consider class year student graduate youre connects warmer connection platform network linkedin facebook account question eaaemoryedu emory chapter chapter networking learning student emory county resident access language county county library language learning information access material county card course lesson greeting talk trip country taste language culture course lesson patron basic culture language grammar networking atlanta company interning consulate trade representative chamber commerce world trade center check event news section volunteer event newsletter institution part network check office state country interest letter cover letter edition brilliant cover letter book mistake winning element résumé style knock collection knock knock cover letter resume resume linkedin profile power verb job seeker hundred verb phrase resume letter job interview life cover letter career guide résumé tip half solution tip job section suggestion resume cover letter advice career advice section recommendation resume letter career guide résumé tip half solution tip job section suggestion resume cover letter advice career advice section recommendation resume letter resume linkedin strategy college executive resume cover artknock collection knock knock cover letter resume resume job resume edition resume resume linkedin profile power verb job seeker hundred verb phrase resume letter job interview life notch executive resume plan job submission executive interview vault netid interview career guide finance estate marketing energy industry search section hiring technique self tip interview question street oasis netid offer interview course interview feedback company estate finance industry career advice job interview preparation tip career advice thankyou email interview wsj career advice job interview preparation tip muse job search section example star story interview method interview question answer interview question question job programming interview answer interview question marketing interview cmo interview insider interview answer question job interview edition highimpact interview question interview question answer book knock collection knock knock cover letter resume career material career career responsibility company andor industry people career level role area scope career achievement business degree serf learning curve student work business unit time student direction career work material graduate career management center coach plan conference board report management trend experience data analysis linkedin class linkedin set skill concept thing peer coworkers career hbr blog career advancement wsj management forbes executive level tip career career career mentor mentor role viewpoint question role question initiative goal team mentor variety experience network issue year mentorship component career growth team conversation people career time honesty respect order boundary conversation bos level leader report conversation direction career family member respectful time intention communication strategy conversation responsive decision goal value job search office executive career conference board report management trend experience data analysis executive recruiter book list business journal book list list executive recruiter city digital business journal business trend headhunter industry search career physician business career science risk management insurance career finance career business analytics career career finance accounting career foundation nonprofit career health care career material career advertising career estate career enterprise career sport business career supply chain operation career</t>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>career_services target company list start know top company target industry expand list firm top mind customize list company wish consider job database firm target industry target company custom criterion atozdatabases target company list emory custom target list business resume geography industry result excel hoover dun bradstreet emory custom target list worldwide business geography industry revenue company resume include swot analysis pitchbook emory netid require firm deal industry financing history include startup back company mature firm uniworld american foreign company global operation emory custom list domestic international firm global presence country result excel explore ranking survey book list business article emory book list company ranking large firm employer fast grow industry firsthand emory netid require rank top employer top internship business area consult finance product wall oasis emory netid require ranking consult banking include race gender veteran status varsity athletics glassdoor best job employee choice award winner update base employee feedback culture mit sloan culturex sing data glassdoor rank firm agility collaboration customer diversity execution innovation integrity performance forbes best employer diversity survey partnership statista include employer employee diversity best training company best training category recognize company organization outstanding result significant progress category recruitment representation succession plan workplace inclusion retention accountability board diversity statista emory netid require include company ranking industry data researcher trade organization government data lseg workspace eikon emory netid require screen company financial criterion dei esg rating target esg firm strategy thomson standard poor netadvantage emory netid require industry resume include list industry visa strategy job_search seek identify company sponsor visa past frequent approach student seek target company likely sponsor visas several list react list large useful cross custom target list firm focus target industry function geography interest target company list guide started list company sponsor last government data authoritative identifying firm apply sponsor visa past data salary_range position goinglobal company apply sponsor visa goinglobal pull data department labor employer data hub great quick company united state citizenship immigration uscis employer data hub firm apply sponsor visa past employer data hub file extensive list csv file present list include sponsoring firm job title legal prevailing wage simplify browse slide data pre filter several popular data sort include salary professional classification pursue graduate business_school student remove pilot physician professor file emory log locate firm uniworld american foreign company global operation emory customized list domestic company operation country country state company industry code revenue result include parent contact address contact sale employee subsidiary operation contact operation owned subsidiary affiliate branch nexis university lexisnexis academic emory netid require identify company base parent subsidiary include company international parent company serch corporate affiliation parent country united state parent spain united state salary negotiation benchmarking benchmarking compensation data resource benchmarking compensation data self report base company industry survey data self report crowdsourced data wall oasis emory netid require finance consult career resource include technical interview training peer report company interview insight emolument self report data heavy focus finance professional firm fyi include audit submit data verify salary data base submission resume statement self report salary company culture data heavy focus technology industry company industry collect data salary compiles salary base internal methodology browse salary calculator job function experience geography data entry senior position salary methodology salary compiles salary employee job advertisement last month idea target city industry ziprecruiter salary calculator salary employer job title ziprecruiter salary major transparentcareer filter degree free registration require salaryexpert high free specific report fee job seeker salary calculator salary nace national association university employer robert half international annual salary guide resume finance accounting free salary data foreign labor certification database government data authoritative identifying firm apply sponsor visa past data salary_range position goinglobal salary data company apply sponsor visa pull dol data easy format foreign labor certification data department labor foreign labor certification flc data disclosure file list firm apply sponsor visa past related compensation data disclosure file scroll raw data excel sort filter fit criterion simplify browse data pre filter several popular data sort include salary professional classification pursue graduate business_school student remove pilot physician professor file emory log common bba salary_range common master of business administration salary_range common msba salary_range great atlanta metro area bureau labor statistic bls data bureau labor statistic bls include breadth salary data regional compensation chart update monthly resume state metro area compensation data national compensation survey occupational wage united state national data set include employer cost employee compensation ecec goodcalculators salary calculator state salary calculator bls data bls occupational employment statistic survey data state metro area resume job negotiate negotiation tip ace salary negotiator hate conflict negotiate counter job wall article linkedin learning training include negotiate job salary min confidently negotiate salary min salaries naked negotiator woman ask best practice negotiation essential job negotiation hbr negotiation practical business negotiation color parachute split difference relocate relocate cost live data remember take cost live account consider salary large city suburb northeast southwest bankrate cost live salary calculator include data cost live criterion payscale salary calculator enter salary compare geography bestplaces net include ranking quality life consideration expatistan cost live include international metro area international university data career guide career exploration target company list malisa anderson strait last updated jul salaries negotiation anderson strait last updated jan job_search strategy visa malisa anderson strait last updated sep accelerate career malisa anderson strait last updated feb change career malisa anderson strait last updated feb executive job_search malisa anderson strait last updated jan rotational malisa anderson strait last updated sep job_searching interview networking malisa anderson strait last updated jan resume resume malisa anderson strait last updated malisa anderson strait last updated jan interview malisa anderson strait last updated jan job_search malisa anderson strait last updated feb rotational list rotational rotational netid require xls company add remove rotational consider inclusive list overview starting master of business administration exchange ranking rank master of business administration rotational industry geography free ranking strategy target rotational job board include filter leadership slice give valuable generate idea typical experience glassdoor rotational linkedin master of business administration rotational job list rotational list power command google find replace suggested term function industry interest supply chain logistics rotational internship operation rotational leadership rotational rotational filetype xls rotational filetype pdf job_search start seek position check target job posting handshake resource advance feel bit overwhelmed start mark dalton book job_search resume job_search steve dalton job_search forum consider join affiliated linkedin forum favorite job post job board helpful related position revise resume explore position align skill hire set job alert browse million posting include association job company linkedin job_search browse job function remote job remote include posting startup large company remoteok salary benefit posting technology focused remote job posting include finance sale marketing programming design pangian global position focus technology marketing sale dev remotive keyword master of business administration include work finance marketing sale wellfound work data analytics marketing operation finance startup jobspresso keyword master of business administration work include sale workingnomads keyword master of business administration global position education finance health care consult marketing sale bbas aftercollege customize job alert area interested interested customize alert target recent grad university recruiter target internship recent grad master of business administration msbas relish career master of business administration data science graduate degree position industry work return pay job irelaunch resource corporate job board focus return pay job career break veteran vet job found goizueta apply job list veterans member military family post resume job military job code military friendly employer disability gettinghired filter state industry dedicate inclusive employer hire professional veteran disability abilityjobs posting post resume posting entry doctor of philosophy career fair workforce recruitment university student disability wrp internship full position federal agency student recent graduate career disabled annual employer award magazine focus career guidance recruitment disability focus undergraduate graduate professional position industry specific job board industry career guide check career guide recommended job target industry association unlimited emory netid require international regional state local non profit organization include irs data non profit association include job posting network event change career start firsthand emory netid require career guide company ranking finance consult real estate marketing energy industry workplace therapist take self inventory evaluate want next job check workplace therapist professor brandon smith linkedin career change several training leverage transferable skill identify value strength prepare career transition network resource start start career network wsj week challenge harvard business job knowledge network jaymin patel network blog tip trick advice master of business administration networking linkedin professional networking training include super connect secret professional networking min network network min connect alumnus meet fellow student alumnus job job company target forget alumnus community university attended linkedin goizueta alumnus join goizueta professional interest goizueta alumnus browse city live job consider limit training student recent graduate start emory connects emory specific warm connection platform expand professional network linkedin facebook account eaa emory emory alumnus chapter chapter meet multinational networking learning languages languages student enrol emory consider dekalb county resident mango language dekalb county library dekalb county library databases language learning resource dekalb county library card basic training lesson focus polite greeting small talk perfect plan short trip foreign country want taste foreign language culture complete training lesson design patron know basic culture language want increase vocabulary improve grammar speak international networking atlanta want job multi national company consider interning volunteer consulate trade representative foreign chamber commerce trade atlanta check event section volunteer event newsletter organization wtc global network check office state country interest resume resume killer resume resume third edition brilliant resume resume book avoid common mistake write winning element style knock dead collection knock dead knock dead resume resume knock dead resume motivate resume linkedin resume power verb job seeker verb phrase bring resume resume resume job interview life ultimate resume resume resume start wsj career guide write tip stand robert half talent solution tip land job section suggestion resume resume resume career advice career advice section recommendation resume resume resume interview wsj career guide write tip stand robert half talent solution tip land job section suggestion resume resume resume career advice career advice section recommendation resume resume resume interview resume linkedin strategy university graduate write stellar executive resume resume artknock dead collection knock dead knock dead resume resume knock dead resume lose resume land job top secret resume fourth edition resume talk motivate resume linkedin resume power verb job seeker verb phrase bring resume resume resume job interview life top notch executive resume career plan job application executive interview start vault emory netid require interview career guide finance consult real estate marketing energy industry linkedin section hiring interview browse interview technique include answer tell self tip answer common interview wall oasis emory netid require technical behavioral interview training peer report interview feedback company account consult real estate finance related industry wsj career advice job interview preparation tip stand wsj career advice write thank interview wsj career advice job interview preparation tip stand muse job_search section tactical tell star story interview method great interview ask hire knockout answer tough interview ask right right job ace programming interview brilliant answer tough interview crack marketing interview cmo ace interview insider extreme interview great answer great job interview edition high impact interview interview answer book knock dead collection knock dead knock dead resume resume knock dead resume accelerate career resource accelerate career accelerate career attain responsibility company industry want move career target adjacent high work area job broaden scope career achievement business degree serf accelerate learning curve prepare student quantitative qualitative job business unit student explore direction career put job remember leverage resource graduate career include coach discuss plan conference board emory require report global trend practice economic data analysis linkedin take training linkedin refine specific skill set skill expose concept give talk peer worker professional engage hbr blog position career advancement wsj forbes reach next executive career advance tip mentor job advance career productive successful professional move career start surround mentor mentor work viewpoint listen ask good mentee work show good take initiative goal intentional build mentor experience network support discuss issue grow mentorship big component career_development late start build challenge conversation move career honesty respect require order good boundary authentic productive conversation bos senior direct report tough conversation direction career family member struggle honest respectful hear feel intention communication strategy know conversation remain confident responsive decision align goal value executive job_search start corner office executive career conference board emory require report global trend practice economic data analysis executive recruiter book list business article emory book list include list top executive recruiter city weekly digital business article local business trend recruit headhunter industry specific guide career physician business career actuarial science risk insurance career analytical finance career business analytics career consult career finance accounting career foundation nonprofit career health care career human_resources career advertising career real estate career social enterprise career sport business career supply chain operation logistics military civilian career</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>威斯康辛大学 lis专业.doc</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
-        <is>
-          <t>威斯康辛大学 lis专业.doc</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
         <is>
           <t>LIS Jobs
 UW-Madison Campus Career Resources
@@ -3262,22 +3202,19 @@
 Federal Government- Government Job Search</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>job campus career material student service career material college career collection pathfinder career material college graduate school career planning letter career service material association job site job placement joblist career material library society arlisna jobnet arma international placement service job site mlanetemployment chance music association job list job bulletin job search job web libjobs job posting internet library journalcom career job web city madison matc dane county state wisconsin government government government job search</t>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>job madison career resource adult student career plan resource university library career collection pathfinder career resource university library print graduate_school career planning resume science career_services slis career resource lis association job aall job placement list ala joblist career resource art library society north america arlis jobnet arma international career placement lita job mlanet employment music library association job list saa employment bulletin sla job_search job sit inalj libjobs library job posting internet library article career job sit city madison madison matc dane county state wisconsin federal government federal government government job_search</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>威斯康辛大学职业收藏.doc</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
-        <is>
-          <t>威斯康辛大学职业收藏.doc</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
         <is>
           <t>Featured Collections
 Our featured collections provide a topical focus in areas of current interest, allowing you to browse and expand your awareness. All materials circulate according to our regular loan periods.
@@ -3296,22 +3233,19 @@
 Search the Ethnic Studies Collection through the Library Catalog.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>collection collection focus area interest awareness material loan period student success book resume cover letter interview job hunting choosing preparing career college career student success collection collection room book collection side floor college search career student success collection catalog computer computer collection material student faculty learn hardware web design computer topic material book collection training software submission software manual design training material collection room computer medium center side floor college search computer collection catalog venture dean student office council collection awareness area collection scope collection book dvd matter topic interest student faculty department course collection health issue material collection room side floor college search catalog</t>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>feature collection featured collection topical focus area interest allow browse expand awareness material circulate accord regular loan period career student success book write resume resume resume prepare interview job hunting choosing preparing career contain university library career student success collection collection locate room book collection locate east side university library career student success collection library catalog computer computer collection include material student faculty hardware design computer topic material book dvds collection training software application software manual design training material collection locate room computer medium locate east side second university library computer collection library catalog ethnic ethnic collection begin collaborative venture dean student office multi cultural council call ethnic collection design awareness multicultural area support ethnic requirement collection expand scope rename ethnic collection include book dvd resume training related subject matter topic interest student faculty ethnic department training fulfill ethnic requirement collection resume contemporary socio economic political health issue literary artistic historical material collection locate room locate west side university library ethnic collection library catalog</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>宾夕法尼亚大学-就业服务简历实验室.docx</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
-        <is>
-          <t>宾夕法尼亚大学-就业服务简历实验室.docx</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
         <is>
           <t>Career Services Resume Lab
 Join the Career Services program for this interactive, hands-on session. Bring your laptop and resume document to build or update during this drop-in lab, where peer learning is encouraged. We’ll provide the tips and tools to perfect your resume and have advisors on hand to answer individual questions.
@@ -3325,22 +3259,19 @@
 Hosted by: Research Data &amp; Digital Scholarship</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>career service join career service program handson session laptop document dropin lab peer learning tip tool resume advisor hand question event september data scholarship exchange van library center floor group student data scholarship</t>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>career_services resume lab join career_services interactive hand session bring laptop resume report build update drop lab peer learning encourage tip tool perfect resume advisor hand answer event occur calendar_month september location_on data digital scholarship exchange van pelt dietrich library penn student host data digital scholarship</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>宾夕法尼亚大学-职业服务检索策略研讨会.docx</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
-        <is>
-          <t>宾夕法尼亚大学-职业服务检索策略研讨会.docx</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
         <is>
           <t>Career Services Job &amp; Internship Search Strategy
 Join this workshop to discover effective search strategies for finding internships and jobs. Take this opportunity to reflect on your goals and explore opportunities that align with your interests.
@@ -3354,22 +3285,19 @@
 Hosted by: Research Data &amp; Digital Scholarship</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>career service job search strategy join workshop search strategy internship job chance goal chance align interest event location_on space van center floor group student data scholarship</t>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>career_services job internship strategy join training discover effective strategy find internship job take reflect goal explore align interest event occur calendar_month february location_on rddsx van pelt dietrich library penn student host data digital scholarship</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>宾夕法尼亚大学-通用资源表.docx</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
-        <is>
-          <t>宾夕法尼亚大学-通用资源表.docx</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
         <is>
           <t>Overview
 Getting Started
@@ -3526,22 +3454,19 @@
 Where do I find information on executive compensation?</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>overview vault career guide career information material penn career service career material career service community interest industry community career management action plan career management industry skill student faculty staff member access linkedin subscription pennkey password linkedin learning course resume skill app growth program excel tableau education penn library book video topic guide company information consumer behavior demographic industry company list information city business journal access city business journal philadelphia business journal book list employer region type company fact living area access book list city city edition list create list access company profile information material profile company investor list company note company record experience insight investment information news industry trend company investment stage capital profile firm financials officer director ownership relationship transaction security growth estimate document credit rating filing news comparables analysis nexis company financials filing stock performance activity news affiliation directory structure company subsidiary listing linkage information parent company affiliate information mids hoover company profile company strategy market position event information company search company company dossier company list list database data axle reference solution information business health care listing search company area business type industry code listing revenue location employee combination directory privatelyheld company company information business summary overview institution list competitor industry description financials revenue employee deal multiple valuation equity deal history family ownership data company company material list company set criterion industry employee factiva company market company company addition information click report ratio comparison report company industry lseg enter ticker access profile information fundamental filing analyst report article company search box companyorg menu keywords interest search box search business source company search box company entity dropdown menu keywords interest search click search start search toolbar top search builder click arrow right company field search company box click orange keywords interest text search box youre click search button bottom screen faq information company analyst report investment bank industry industry industry guide material report industry industry classification system naics report range niche sector report statistic segmentation market characteristic industry condition competitor industry performance outlook poor advantage source business investment information access poor product industry survey stock report corporation record outlook fund report cover capital market solution industry report country outlook guide bureau labor statistic benchmark job outlook information climbtheladder browse career description requirement job outlook salary advancement chance department labor career cluster industry consumer market consumer behavior demographic guide material gmid euromonitor internationalpassport gmid market business intelligence industry country consumer access statistic market share market size distribution pricing briefing report coverage consumer market mintel market report consumer market report market driver size trend market segmentation consumer attitude habit industry analysis market trend data market segmentation size growth industry coverage service consumer product food beverage industry life science technology medium coverage state subscription provider focus report mind commerce fact sbi information statista access statistic market researcher institution publication government source news market information market country language publication industry technology telecommunication energy industry finance health care industry investment management merger acquisition industry industry equity venture capital people database people peop terminal library huntsman people tool bio search bio search directory company investment trend transaction equity venture capital sector company information profile company investor information hoover find contact search field list search option menu source category directory search filter directory web material people website click search people job title company news book book catalog subject job interview job job title lippincott information desk cover point interview preparationcase point interview preparation marc cosentino contribution hdc publication date street journal point master of business administration cosentino interview interview type question share ivy system confidence book strategy exercise way cost interview secretscase interview secret victor cheng call hdc publication date interview secret instruction job interview worldthe interview victor mckinsey management consultant insider interview job offer mckinsey bain company monitor lek wyman kearney handson realworld perspective job offer crack system ohrvall call hfi isbn publication date crack system training program interview consulting firm fortune companiesdavid expert interview interview stepbystep approach ctc combine guidance communication analytics thinking insider tip insight thousand edition content exercise drill integration video mbacasecom compensation salary wage data government source bureau labor statistic wage data job wage statistic data occupationspecific data compensation survey data state region company type occupation web material salary search job title location payscale scroll individual navigation bar company job title degree skill compensation tab topic wage change time graduate school option finder search engine bls wage data compensation information occupation location cost living location information mit living wage calculator tool living wage state area county level cost calculator tool cost living location cost calculator expense location globe note data user price area bestperforming city report set metric job creation wage gain performance area faq information executive compensation</t>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>overview start take vault career guide career interview resource penn career_services digital career resource penn career_services community career interest industry community master of business administration career action plan map wemba career industry tool build skill student faculty staff member linkedin university subscription pennkey password linkedin learning training interviewing resume write skill build app excel tableau higher_education penn library book video resume similar topic related lippincott library guide company behavior demographic industry company list city business article city business article philadelphia business article book list list top employer company fact living area book list city city past digital edition list list company resume resource pitchbook include resume company investor save list company add note company record personalize experience insight investment industry trend relate company investment finance resume firm worldwide include finance officer director ownership advisory relationship transaction security key estimate key report credit rating filing comparables analysis nexis company resume finance sec filing stock performance activity include corporate affiliation report international corporate structure company subsidiary listing corporate linkage parent company affiliate include historical mid hoover company resume company histories strategy position major event international company nexis university company company dossier company list list database downloadable data axle solution referenceusa canadian business health care residential listing company geographic area business industry code yellow listing revenue employee combination privco hold company company consist business summary overview corporate organization list competitor industry description finance revenue employee deal deal multiple firm valuation fund equity deal history family ownership data company company resume resource list company base set criterion industry employee factiva company company enter company addition resume report ratio comparison report company compare industry lseg workspace enter ticker complete resume fundamental filing analyst report article inform enter company company drop include related keywords interest additional business complete company company entity drop include additional keywords interest factiva start black toolbar top builder arrow right company field company appear highlight orange add additional keywords interest free text finish bottom screen relate faq find company find analyst report investment bank industry industry overviews industry guide additional resource ibisworld report china industry categorize north american industry classification naics specialized report resume wide niche sector report key statistic segmentation characteristic industry key competitor industry performance outlook standard poor net advantage comprehensive business investment standard poor relate product industry survey stock report corporation record outlook mutual fund report resume finance bmi fitch solution global industry report browsable country occupational outlook handbook bureau labor statistic find salary benchmark job outlook climbtheladder browse depth career description include requirement job outlook salary common advancement careeronestop sponsor department labor career cluster fastest grow industry overviews behavior demographic guide additional resource passport gmid euromonitor international passport gmid contain business intelligence industry country statistic include share distribution pricing comprehensive briefing report global coverage industrial represent mintel report resume european report analyze driver trend segmentation attitude purchase habit marketresearch academic qualitative industry analysis quantitative trend include data segmentation growth industry coverage include product food beverage heavy industry life science technology medium primary geographical coverage united state penn subscription include following provider freedonia focus report kalorama mind commerce package fact sbi simba statista statistic gather researcher trade organization scientific article government emis financial economic focus emerge country include native language article related industry guide consult digital technology telecommunication energy industry finance health care industry investment merger acquisition pharmaceutical industry retail industry equity venture finance library database bloomberg peop bloomberg terminal lippincott library huntsman subscriber tool bio quick advanced bio international company pitchbook investment trend transaction equity venture finance sector company include resume company investor financial deal hoover find contact widget conduct basic expand additional field full list option nexis university expand category add filter nexis university resource conduct extensive linkedin advanced conduct advanced job title company facebook google book find book franklin library catalog subject employment interviewing resume employment job hunt find helpful title lippincott library desk resume complete interview preparation complete interview preparation marc cosentino contribution call isbn article wall article call master of business administration bible cosentino demystify consult interview take typical interview explore various share acclaim ivy give confidence answer sophisticated book include strategy ten start exercise cut cost resume interview secret interview secret victor cheng call isbn article interview secret discover instruction dominate consider complex difficult intimidating corporate job interview infamous interview victor cheng former mckinsey consultant reveal proven insider method ace interview secure job mckinsey bain company monitor wyman kearney mckinsey interviewer hand real perspective take land job resume crack crack david ohrvall call isbn article crack complete training challenging interview favor top consulting firm grow fortune company david global expert interview crush interview approach ctc combine practical guidance communication structure analytics integrated thinking insider tip insight gain train candidate edition include updated content exercise drill integration video mbacase compensation salary wage data government bureau labor statistic bls wage data occupational employment wage statistic data job specific data national compensation survey data state company job resource glassdoor conduct salary job title specific payscale scroll navigation bar explore salary company job title degree skill compensation depth compensation relate topic wage change graduate different university compensate option careeronestop salary finder engine bls wage data retrieve compensation job cost living mit living wage calculator tool calculate living wage state metro area county payscale cost live calculator tool calculate cost living compare expatistan cost live calculator compare expense globe note data supply expatistan base price area subject error base report milken institute best perform city report set metric job creation wage gain track economic performance large metro area related faq find executive compensation</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>宾西法尼亚大学 为会计准备的资源.doc</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
-        <is>
-          <t>宾西法尼亚大学 为会计准备的资源.doc</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
         <is>
           <t>Accounting  Career Resources
 Professional Associations
@@ -3570,22 +3495,19 @@
 Career Development &amp; Job Search Resources</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>career material association institute accountant career advice job search tool woman profession worklife balance cpa network accounting association career fair meeting information information section management society accountant student membership scholarship foundation state institution institute accountant student membership career informatioin entry level job position database outlook outlook guide website department labor profile hundred type job profile training requirement salary job growth job description condition growth job search material</t>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>account career resource professional association aicpa american institute certified accountant career advice job_search tool mentor woman profession job life balance young cpa network american accounting association career fair annual meeting regional section account national society accountant nsa student membership scholarship foundation affiliate state organization pennsylvania institute certified accountant picpa student membership career informatioin entry job position career database websites occupational outlook handbook occupational outlook handbook maintain department labor resume job resume include training educational requirement salary expect job growth job description job career_development job_search resource</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>宾西法尼亚大学 为智力障碍.doc</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
-        <is>
-          <t>宾西法尼亚大学 为智力障碍.doc</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
         <is>
           <t>Career Studies Program at Penn State Harrisburg
 Jobs
@@ -3599,22 +3521,19 @@
 Your rights at work. Also, help for people with disabilities.</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>career program state harrisburg job outlook guide career job job harrisburg onet online career skill worker disability right work people disability</t>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>career penn state harrisburg job occupational outlook handbook facts career pennlive job job harrisburg net career base skill careeronestop worker disability right job disability</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>宾西法尼亚大学 实习与奖学金.doc</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
-        <is>
-          <t>宾西法尼亚大学 实习与奖学金.doc</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
         <is>
           <t>Awards, Scholarships, Internships, and Graduate Assistantships
 Penn State University Libraries offers a number of awards, scholarships, and internship opportunities to undergraduates and assistantships for graduate students.  Our awards recognize outstanding research or scholarly work. Our scholarships are awarded based on a number of factors including merit, financial need, interest in librarianship, and your major. Our internships and graduate assistantships are paid positions that allow undergraduate and graduate students apply their disciplinary background to library-related projects.
@@ -3634,22 +3553,19 @@
 Juniors and seniors in good academic standing many apply for a variety of paid internships throughout the University Libraries. Graduate students from a variety of disciplines may apply for library-centered assistantships located at the University Park Libraries.</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>award scholarship internship graduate assistantships state university award scholarship internship chance undergraduate assistantships graduate student award work scholarship factor merit need interest librarianship internship graduate assistantships position undergraduate graduate student background project award university library award student information literacy guentter thesis award thesis phi beta kappa honor schreyer scholar honor discipline phi beta kappa contribution field judy art education award project archive growth judy award flower artist educator knowledge student award graduate student project aspect knowledge linda stein award honor joyce diane froot action justice linda education collection teaching technology impact award work accomplishment penn state faculty member work transforms technology material champion award faculty work education scholarship assistance student variety discipline art information technology interest science scholarship student internship graduate assistantships junior senior apply variety internship university student variety discipline assistantships university park library</t>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>award scholarship internship graduate assistantships penn state university libraries award scholarship internship undergraduate assistantships graduate student award recognize outstanding scholarly job scholarship award base factor include merit financial interest librarianship major internship graduate assistantships pay position allow undergraduate graduate student apply disciplinary background library related project award university library undergraduate award recognize student showcases outstanding literacy skills robert guentter outstanding undergraduate thesis award find best thesis submit undergraduate phi beta kappa honor thesis prize award schreyer scholar honor thesis complete discipline include phi beta kappa significant contribution field judy chicago art education award acknowledge project base primary incorporate archive collaborate judy chicago portal award present flower scholars educator white indigenous knowledge student award support graduate undergraduate student pursue project focus aspect indigenous knowledge linda stein upstander award honor joyce diane froot inspire publishable promote upstander action justice base archival linda stein art education collection teaching technology impact award celebrate job accomplishment penn state faculty member job transforms education technology affordable educational resource oaer champion award recognize faculty job education scholarships scholarship financial assistance undergraduate student discipline include liberal art technology interest library science scholarship base student apply internship graduate assistantships junior senior good academic stand apply pay internship university libraries graduate student discipline apply library assistantships locate university park library</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>27</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>宾西法尼亚大学 就业指南.doc</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
-        <is>
-          <t>宾西法尼亚大学 就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
         <is>
           <t>Career Development &amp; Job Search Resources
 Career Readiness &amp; Preparation
@@ -3761,22 +3677,19 @@
 PSUL's Test Prep Resources guide highlights resources for preparing for common standardized tests including the GRE, MCAT, and LSAT.</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>career growth job search material readiness preparation psul material career readiness sage skill business student experience skill topic data analytics diversity equity inclusion belonging accessibility entrepreneurship finance basic leadership marketing operation management communication professionalism workplace conflict negotiation access psu alumnus harvard business collection collection business management ebooks title career readiness competency communication thinking equity inclusion leadership teamwork access psu business press library collection ebooks business topic bisac category business economics selfhelp title readiness topic access psu book career growth workbook leadership campus writing job college bet breakthrough chance career world work career exploration networking website career exploration outlook guide job website department labor profile information salary job growth access community information database description hundred occupation access community career expert state career service center career guidance information career path major access community book career game loop career chance career myth marketing technique job cool guide color jobhunters job therapy job search internship search penn state material internship job search expert state career service center advice internship job search list website position access community lion career platform student alumnus employer access psu alumnus career fair university park information career fair event university park material link information collegespecific career fair access community state career site information psu job listing candidate access community information job level title industry location employer state job bank resume job search state job bank component careeronestop suite web site department labor partnership agency state government sector institution place pennsylvania material employer rank size city industry book guide job search cover letter material communication sage skill business communication module sage skill business information writing workplace brand job book resume resume linkedin strategy college graduate interview preparation psul material communication sage skill business communication module sage skill business information writing workplace brand job job offer salarywage information relocation salary wage information outlook guide job site department labor profile information job offer expert state career service center advice job offer offer calculator calculator cost area movecom homefair site expert report material wage workstats wage report title view data statewide area workforce investment area sage business material student experience business skill relocation information homefair relocation calculator sperlings place data population cost school test prep material material test prep material highlight material test gre mcat lsat</t>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>career_development job_search resource career readiness preparation psul resource career readiness sage skill business design student develop practice professional skill module topic include data analytics diversity equity inclusion belonging accessibility entrepreneurship finance basic leadership marketing operation organizational communication professionalism workplace conflict negotiation psu alumnus library harvard business publish collection collection business book include title career readiness competency include communication critical thinking equity inclusion leadership teamwork psu business expert press digital library collection ebooks business related topic browse bisac category business economics title relate career readiness topic psu feature book personal career_development workbook self leadership corporate writing job university career bet recognize implement breakthrough recalculate career changing job career exploration networking career exploration occupational outlook handbook job maintain department labor resume include salary expect job growth community net occupational database contain detailed description job community major career plan expert penn state career_services career guidance include career path associate various academic major community feature book career game loop master network forge career flex career myth debunk marketing technique great job good cool guide personal purpose color parachute job hunter workbook job therapy job_search internship penn state resource internship job_search expert penn state career_services advice navigate internship job_search include list position community nittany lion career recruit platform student alumnus employer psu alumnus career fair university park find career fair related event university park resource university specific specific career fair community penn state career job psu job listing internal external candidate community websites collegegrad find job title industry employer state job bank post resume job_search state job bank component careeronestop integrate suite national sponsor department labor partnership federal agency state government sector organization job pennsylvania resource allow sort employer rank city industry feature book hbr guide job_search hire resume resume resume psul resource organizational communication sage skill business organizational communication module sage skill business writing workplace establish personal brand apply job interview feature book resume talk resume linkedin strategy university graduate interview preparation psul resource organizational communication sage skill business organizational communication module sage skill business writing workplace establish personal brand apply job interview job negotiation salary wage relocation salary wage occupational outlook handbook job maintain department labor resume include salary job negotiate expert penn state career_services advice evaluate job negotiate salary calculator salary calculator compare cost live area move homefair salary expert salary report pay free resource occupational wage workstats pennsylvania wage report occupational title data statewide county metropolitan statistical area workforce investment area sage skills business digital resource student develop practice business professional skill relocation homefair include relocation calculator sperling best include data population cost live grad university plan test prep resource test prep resource psul test prep resource guide highlight resource prepare common standardized test include gre mcat lsat</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>28</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>密歇根大学-为建筑设计提供职业资源.docx</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
-        <is>
-          <t>密歇根大学-为建筑设计提供职业资源.docx</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
         <is>
           <t>Home
 Quick Links
@@ -4159,22 +4072,19 @@
 Resources and programs available right here on campus to help you with internships and job searches.</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>home quick link architecture engineering catalog catalog material university search college article article database article thousand publisher million document part search result article journal newspaper article thing article search way topic article search library article search database searching forget avery index jstor sciencedirect standard article search book catalog print search catalog architecture blog conversation dose architecture architecture lab archnewsnowcom bldg blog city design world foundation design architecture advocacy publication league reference guide citation tab information citation style tab citation style guide government document source information government document list link citation style mla book book architecture book architecture keyword title search catalog search title author search option material book youre book relevant search subject heading title search architecture book library congress call floor shelving aael book bound journal ana floor book oversize floor reference reference book dictionary architecture floor book architecture book book circulate reserve book reserve hour reserve desk floor folio storage size age andor condition book storage space level book building staff member reserve desk book collection book collection collection space level book price appointment book storage facility buhr book art architecture engineering library mirlyn buhr facility book series book part series series journal book series theme title instance series clog book title mall prison way book series title book search option series pull arrow series search index series title theme clog pamphlet architecture reference work architecture list reference work architecture topic guide dictionary book information architect building topic material reference section art architecture engineering library floor reference work multivolume architect period movement reference collection floor art architecture engineering mcgraw hill reference collection engineering subject access construction engineering title institute architect architecture call art artifact architecture law call building detroit history call encyclopedia century architecture call glossary art architecture design call guide campus university michigan graduate dictionary architect architecture call engineering online reference engineering construction material category encyclopedia architect art online sun angle calculator kit call aael storage timesaver standard building type university michigan survey call multimedia architecture material association lecture lecture theme association bbc radio architecture programme interview recording architect architect history project project contribution architect century sciarc medium archive hour architecture design lecture event sciarc california institute architecture article architecture database article subject index periodical avery index database artbibliographies abstract article book essay catalog dissertation artist movement century aspect art photography invention art source art index retrospective index englishlanguage art publication periodical bulletin competition award notice listing interview film text article jstor image image jstor image archive image art monument art image index periodical citation database periodical architecture field design history construction public planning design bibliography history art art antiquity bibliography history art index abstract book conference proceeding dissertation exhibition dealer catalog type building drawing photograph birkhäuser manual cumincad index publication computer design design art index daai reference article design craft journal data designer studio firm detail inspiration database content magazine detail jstor access archive journal book art humanity science science connexion database database material access source news business reference information search journal catalog institute architect lexicon actar publication book interview design issue article construction technology database engineering technology question issue construction structure material database engineering village proquest technology collection database combine journal indexing literature technology science material science aerospace engineering engineering engineering matter physic computer science engineering web science database image image image information finding image material architecture discipline libguide image material image access material link database architecture collection user range image collection university archivision archive image monument art jstor image image jstor image access image culture art photojournalism material type building drawing photograph birkhäuser manual inspiration database content magazine detail library congress map fire insurance map checklist database fire insurance map map company collection geography division image material web image material web city view city monument architecture ohio collection drawing illustration toledo county archnet online material archnet online community architecture art culture catena archive garden collection image landscape design villa city world database image city collection society diarna image site east north imaging project ann sullivan image architecture world professor sullivan bluffton college database housing type photograph making arbor image history architecture arbor france image information monument century france muschenheim photograph drawing william muschenheims york gallery access hundred thousand image discipline coast architecture database database architect architecture pacific coast washington oregon california wayne state image gallery image collection archive labor affair history growth politics right community view century photography digitization project image thcentury architecture database architecture profile architect country archive archive collection description collection online document aid content collection version content database guide archive record family history database manuscript collection repository archive entry finding aid limit search material university library database archive touch source material publication magazine focus archive list sampling search search archive americana news york time history vault shoah foundation history time vogue archive archive city library collection material project history museum encyclopedia art institute chicago archival collection library university society society encyclopedia burton collection walter library labor affair state hong kong heritage project hong kong architecture travel focus touch source institute architect collection archive record angeles archive california university museum archive architecture design collection york city museum city york skyscraper museum world trade center building york archive york collection wale state archive record wale government architect city archive directory guide posting world building city online material architecture posting world building country architecture city archive directory archive aael order university library member material order consortium harvard graduate school design rhode school design consortium collection partner creation material material description access material order collectionspace lyrasis standard experience approach management design collection material connexion material library access material connexion youll material floor art architecture engineering material collection space reserve desk contact rebecca rpwumichedu question collection stop material product information web building arcat building material product information community material architecture design click material sampling access material material material information source engineering design community building material sweet sweet directory product information manufacturer product product type clt cross timber guide guide clt usda softwood lumber council construction data cmd construction information browse product information search construction data news building code part site registration molybdenum association design material stainless steel stainless steel architecture intl molybdenum association search directory directory listing manufacturer supplier segment manufacturing marketplace state material district material district materia netherlands network material material austin directory material building product website student school architecture material institute description image material institute london source building material listing building material discussion aspect sustainability register manufacturer catalog product service info material material guide information material standard book standard book art architecture engineering library reference collection floor detail standard standard construction call standard timesaver standard call standard building type timesaver standard design space planning call timesaver standard landscape architecture call code material code cad building code collection plumbing fire maintenance code boca sbcci icbo icc nfpa state code code link code michigan upcodes company madcad link code access code state state state department licensing affair lara access state construction code regulation book building code book art architecture engineering library online title building code guide material douglas thornburg john henry isbn publication date building code code council publication date change building code call building code winkel david collins juroszek francis consultant editor isbn publication date building code guide building code call building code guide material isbn publication date building code guide material kimball chris isbn publication date building code guide material douglas publication date building code guide material douglas publication date institution institution society institute architect homepage institute architect site link career directory architect information society landscape architect asla website information news event firm institution program landscape architecture league institution mission excellence architecture design urbanism debate provoke thinking design building issue day association collegiate school architecture site acsa link competition information student publication school architecture education association computer design architecture site link conference competition publication computer design architecture foundation institution minority architect site link chapter information competition conference society historian sah website offer link activity project chapter site architecture group inst art architecture calearth possibility art architecture homelessness ground institution homelessness housing solution biotecture michael site biotecture effort architecture material growth design mad atlanta institution action homeless mass model architecture society msaada architect growth group empowers nation housing solution reservation community studio studio student solution community housing growth need shelter settlement reconstruction community conflict disaster architecture group city design planning art competitionscareers competition competition architect artist planner website competition listing competition world journal journal shelf competition institute architecture student competition student competition assoc collegiate school competition student architecture pritzker architecture prize site award winner biography portrait acceptance speech architect newspaper competition list competition design award listing competition competition site ireland rest world career association collegiate school architecture acsa material student career school architecture career choice institute architecture student aias student institution guide career taubman college career service material program campus internship job search</t>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>quick art architecture engineering library library catalog catalog material university michigan library library taubman university architecture urban plan find article library article multiple database library article allow publisher million report limit result article scholarly article report article fulltext remember library article good start particular topic library article great multi disciplinary inter disciplinary library article replace subject specific database specialized searching forget avery jstor sciencedirect standard accustomed library article book catalog contain ebooks want print ebooks library catalog architecture blog conversation daily dose architecture architecture lab archnewsnow bldg blog city sound inhabitat design save michigan architectural foundation roguehaa design architecture urban advocacy collaborative streetsblog urban article architectural league nyc cite guide citation fourth apa citation style fifth mla citation style guide cite government report include cite government report extensive list various citation style apa mla book find book architecture find book architecture keyword title library catalog start simple know title author want jump advanced option locate material find book book relevant want subject heading list title guide architecture book categorize library congress call begin shelve third second library shelving aael book bound article call begin shelve third call begin book designate oversize shelve second book encyclopedias dictionary relate architecture locate second library book call begin find architecture book book circulate library reserve book keep reserve desk check ask reserve desk second library folio storage age book keep storage low book ask staff member reserve desk book special collection book collection consider rare keep special collection low book contact rebecca price arrange appointment buhr book store offsite storage facility buhr buhr book send art architecture engineering library log mirlyn visit buhr shelve facility find book find book publish difficult different article serial book theme title instance clog include book title render national mall prison easy find book publish know title book advanced option enter pull arrow popular title architectural theme clog pamphlet architecture important job architecture list useful job architecture related topic include encyclopedias handbook dictionary book useful specific architect topic print resource non circulate section art architecture engineering library second job architecture multivolume job important architect period movement feel free browse collection second art architecture engineering library accessengineering mcgraw hill collection civil engineering subject construction engineering title aia detroit american institute architect guide detroit architecture call art artifact architecture law call detroit history call encyclopedia century architecture call glossary art architecture design call guide university michigan call graduate library international dictionary architect architecture call knovel engineering scientific civil engineering construction material category macmillan encyclopedia architect call oxford art sun angle calculator kit call aael storage saver standard call university michigan encyclopedic survey call multimedia architecture resource architectural association lecture lecture architectural theme post architectural association london bbc radio architecture programme archive interview recording several major architect chicago architect oral history project project report contribution architect chicago century sci arc medium archive archive architecture design lecture event sci arc southern institute architecture article databases architecture appropriate database find article architectural subject avery architectural periodical avery relevant database list artbibliographies modern abstract article book essay exhibition catalog dissertation resume movement late century aspect modern contemporary art include photography invention present art art retrospective key international english language art article include periodical museum bulletin competition award notice exhibition listing interview film include full text article jstor image image jstor image artstor rich archive image art architectural monument landscape architecture art cultural image architectural periodical citation database focus periodical architecture related field emphasize architectural design history construction arts urban planning design bibliography history art resume european american art late antiquity present bibliography history art abstract relate book conference proceeding dissertation exhibition dealer catalog build searchable author texts architectural drawing photograph manual cumincad cumincad cumulative article computer aid architectural design design apply art daai contain annotated article design craft article publish worldwide data designer craftspeople studio workshops firm detail inspiration database visual textual content german architectural magazine detail present jstor full text archive article book art humanity social science science material connexion database searchable browseable database innovative material nexis university full text business legal proquest library multi disciplinary academic popular article riba library library catalog royal institute british architect urbannext lexicon organize actar article article book interview urban design issue article construction architectural technology database focus engineering suit architectural technology job issue construction structure material try database engineering village proquest technology collection global database combine full text article indexing global literature technology apply science include material science aerospace engineering mechanical engineering civil engineering condense matter physic computer science electronic engineering sciencedirect science database image find architectural image aael image guide finding image visual resource architecture discipline libguide image several resource find architectural image resource library database architecture collection allow architectural image collection university michigan digital library archivision architectural image rich archive image architectural monument landscape architecture art jstor image image jstor image artstor image visual material culture include architecture art photojournalism material build searchable author texts architectural drawing photograph manual detail inspiration database visual textual content german architectural magazine detail present library congress sanborn map collection sanborn fire insurance map checklist searchable database fire insurance map publish sanborn map company house collection geography map division architectural image resource several image resource city panoramic city monument landscape architecture northwest ohio browsable collection drawing illustration toledo lucas county library archnet resource archnet community devote islamic architecture art culture catena digital archive historic garden landscape searchable collection historic contemporary image landscape design italian villa city database digital image represent city photographic collection american geographical society library diarna image endangered jewish middle east north africa digital imaging project mary ann sullivan last updated image architecture professor sullivan bluffton university urbanitarian browseable searchable database multi family housing photograph making ann arbor image history architecture ann arbor map gothic france image built monument century france muschenheim digital archive photograph drawing william muschenheim architectural job library digital gallery image cross discipline pacific coast architecture database searchable rich database architect architecture pacific coast oregon reuther library wayne state image gallery several image collection archive labor urban affair relate history detroit include urban politics civil right ethnic community century canada canadian architectural photography digitization project image century canadian architecture vitruvio searchable database historical contemporary architecture architects resume contemporary architect searchable country archival find archive archive hold collection personal institutional description collection report call finding aid outline content collection include digital version content database find personal institutional hold guide archive historical record personal family history archive finder database manuscript special collection repository ireland archive include entry finding aid worldcat limit archival material university library subscribe database describe archive put touch primary resource include single article vogue magazine particular subject focus archive following list sampling find library archive archive americana google archive proquest history vault shoah foundation visual history archive london digital archive vogue archive architectural archive organize city list specialized library architectural collection resource relate project chicago chicago history museum encyclopedia chicago art institute chicago archival collection detroit bentley historical library university michigan detroit historical society historical society encyclopedia detroit detroit library burton historical collection walter reuther library labor urban affair wayne state univ hong kong kong heritage project foreign architect hong kong contemporary architecture guide travel focus put touch london riba royal institute british architect library collection national archive find architectural record los angeles archive include university museum archive getty architecture design collection city museum city skyscraper museum trade historic low manhattan library archive manuscripts library digital collection sydney south wale state archive record south wale archive colonial government architect sydney city archive national archive australia guide architect posting organize city resource contemporary architecture architect posting organize country contemporary architecture city guide archive hub archive aael join material order university michigan library member material order consortium found harvard graduate_school design rhode island university design consortium bring material collection partner creation share resource material description material order power collectionspace lyrasis utilizes develops standard best practice community base approach design material collection material material connexion material library library onsite innovative cool material material connexion find material art architecture engineering library material collection reserve desk contact rebecca rpw umich collection stop touch material product design arcat material build product architectural spec write community independent resource architecture design material sampling material material material engineering design community material mcgraw hill sweets sweet build product manufacturer product product clt cross laminate timber handbook handbook clt publish usda binational softwood lumber council cmd reed construction data cmd commercial construction browse product construction data code require free registration international molybdenum association architectural design resource stainless steel stainless steel architecture publish int molybdenum association iqs industrial quick iqs comprehensive listing manufacturer supplier serve major segment oem industrial manufacturing united state canada material district material district materia base netherlands global network innovative material material lab austin material product student austin university architecture material library institute description image material curated institute london sustainable green material listing typical material discussion aspect sustainability thomas american manufacturer searchable catalog industrial product material material collection guide material library graphic standard book graphic standard book art architecture engineering library collection second architectural detail call architectural graphic standard call architectural graphic standard residential construction call interior graphic standard call saver standard architectural light call saver standard call saver standard interior design planning call saver standard landscape architecture call build code electronic resource build code mad cad code comprehensive cross collection build electrical mechanical plumbing fire maintenance code boca sbcci icbo icc nfpa state local code michigan build code build code michigan code commercial company madcad municipal code municode local municipal code state seach state locale state department licensing regulatory affair lara state construction code regulation book code book art architecture engineering library title international code handbook electronic resource douglas thornburg john henry isbn article international code international code council isbn article significant change international code call residential code illustrate steven winkel david collins steven juroszek francis ching consultant editor isbn article code illustrate guide understand international code call international code illustrate handbook electronic resource isbn article international exist code handbook electronic resource kimball chris isbn article international code illustrate handbook electronic resource thornburg douglas isbn article international code illustrate handbook electronic resource thornburg douglas isbn article organization societies architectural organization society american institute architect official homepage american institute architect include aia career architect american society landscape architect asla asla event firm academic institution list accredited landscape architecture architectural league organization base nyc mission nurture excellence architecture design urbanism stimulate debate provoke thinking design issue association collegiate university architecture acsa student competition student article university architecture architectural education association computer aid design architecture include conference competition article relate computer aid design architecture michigan architectural foundation national organization minority architect noma include noma chapter competition conference society architectural historian sah sah activity project chapter humanitarian architecture inst earth art architecture cal earth explore possibility earth art ceramic architecture solve homelessness break ground organization devote end homelessness develop supportive housing solution earthship biotecture michael reynold devote earthship biotecture effort self sufficient architecture recycled material international design summit mad housers atlanta base organization engage action shelter homeless mass model architecture serve society msaada architect red red feather empowers american indian nation sustainable housing solution reservation community rural studio rural studio engage student address seek solution community housing shelter centre ngo support transitional settlement reconstruction community affect conflict natural disaster terreform architecture smart city design ecological planning art competition career architectural competition competition architect planner competition article featuring listing major competition article find article shelf competition list american institute architecture student competition student competition list assoc collegiate university architecture competition gear student pritzker architecture prize pritzker architecture prize present include past present award winner biography photo portrait acceptance speech architect report competition list list national international competition update award international interior design award give thearchitectureroom listing architectural competition competition ireland rest career architecture association collegiate university architecture acsa resource student young professional regard university architecture career choice american institute architecture student aias student run national organization enrich educational guide career taubman university career_services resource internship job_searches</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>29</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>密歇根大学-为环境提供职业资源.docx</t>
+        </is>
       </c>
       <c r="B31" t="inlineStr">
-        <is>
-          <t>密歇根大学-为环境提供职业资源.docx</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
         <is>
           <t>Environmental Engineering
 Use the tabs to the left to learn more about finding information in Environmental Engineering.
@@ -4447,22 +4357,19 @@
 Need help finding data or working with GIS software? Contact the Clark Library or SAND North lab.</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>engineering tab left information engineering find link database engineering book book online art architecture engineering standard guide standard material material engineering institution associationssocieties engineer material information engineering career job service link service library guide material science engineering landscape architecture material science engineering environment sustainability geosicences essential video library series video tutorial interest topic interest book title title purchase library request form collection access engineering guide engineering online version reference book engineering science access book publisher reference guide conference proceeding library access journal book wileyblackwell life health science science humanity book book engineering word search catalog search word search starting point title subject heading title search guide dictionary material online university michigan student staff faculty knovel taylor francis ebooks reference work engineer bela liptak editor david liu editor isbn publication date engineer edition source information depth factor principle environment past today future engineering guide chen editor richard liew editor isbn publication date engineering guide field reference engineering guide richard dorf editor isbn publication date engineering guide expert area specialty knowledge mature practitioner engineering novice guide ecomaterials myriam torres editor oxana vasilievna kharissova editor boris kharisov editor isbn publication date guide editor ecomaterials material material ecology protection material society health material energy criterion source function ecomaterials material environment life cycle guide engineering calculation edition tyler hick publication date guide engineering calculation calculation align experience code standard water wastewater calculation edition dar lin isbn publication date water wastewater calculation principle experience calculation surface water groundwater drinking water treatment wastewater engineering hydrogeology field publication date hydrogeology field information submission groundwater sampling waterquality assessment aquifer characterization contamination issue submission water wastewater engineering design principle experience edition mackenzie davis isbn publication date indepth guide water wastewater engineering advance procedure regulation material contains coverage design construction water wastewater facility management library tool footnote bibliography tool expert endnote software computer endnote guide information firefox extension computer machine material visit zotero guide information mendeley mendeley citation management tool citation document bibliography mendeley guide information article citation style guide citation style reference section chapter asce website text report asce authordate method example smith smith jones report reference section reference author reference thesis dissertation article exception rule style source book evans biotechnology theory submission chapter chapter title article element method analysis appl mech rev httpsdoiorg journal article source example style journal article conference proceeding kulicki mertz cracking steel girderfloorbeamstringer bridge proc int bridge conf pittsburgh engineer society pennsylvania index abstract journal article conference report database list database engineering database citation article mgetit access water content water environment foundation water quality career conference proceeding manual experience standard article fact sheet report database science database coverage trade literature water material supply water quality water waste analysis water treatment underground service water sewage effluent effect pollution science fishery pollution quality policy contamination ocean lake river estuary engineering village compendex area engineering science coverage technology transportation chemical engineering light technology engineering engineering abstract index journal engineering aspect air water quality safety energy production science database database coverage science abstract citation serial journal conference proceeding report book government publication scholar availability link google link holding greenwire report energy material issue house agency court state medium country user email alert news story library literature oil gas exploration production industry pollution pollution abstract access information government policy emission action response pollution issue technology collection database text journal indexing literature technology science material science aerospace engineering engineering engineering matter physic computer science engineering engineering collection proquest technology collection proquest material science collection indexing technology scholarship web science index article journal area science technology article article footnote reverse scifinder chemical abstract journal patent report dissertation conference proceeding book biochemistry inorganic chemistry water material coverage water material issue groundwater lake estuary water supply desalination water yield water quantity groundwater management watershed water quality wastewater water law citation management library tool footnote bibliography tool expert scholarspace endnote software computer endnote guide information firefox extension computer machine material visit zotero guide information mendeley mendeley citation management tool citation document bibliography mendeley guide information standard finding standard standard information industry standard society standard standard art architecture engineering copy standard art architecture engineering access standard issuing agency standard society material compass aami association advancement instrumentation aami standard esubscription access click access link association state highway transportation official compass concrete institute standard manual experience online aiaa institute aeronautics astronautics standard online aerospace standard institute steel construction online website specification steel building standard society engineer library society engineer standard boiler pressure vessel code asme standard collection access click access link standard welding society compass awwa standard water association compass awwa standard standard knovel search awwa example awwa standard institute record standard code regulation reference ibr standard standard iec aham society format downloading printing option cost eosesd association standard electrostatics standard downloads esdaorg website iec standard commission compass ieee standard institute electronics engineer ieee ieee institution standardization publishes standard topic standard compass society engineer publishes standard mobility engineering ground vehicle aerospace aerospace material standard sae standard online mobilus society motion picture television engineer standard topic broadband control system file image format ieee xplore standard state formulary online access user account email account subscription blank account access content online building energy code building fire energy code standard code council icc building code fire protection association society refrigerating engineer state michigan building code online cad fire protection association code online underwriter laboratory standard format cost access account site payment printing downloading site health insurance portability accountability act hipaa outline standard health care transaction code set health identifier security overview regulation health service department osha safety health administration osha standard online osha website safety health administration miosha standard online miosha specification department defense dod standard registration approval access dod website coverage access user access dod person art architecture engineering library code access code ordinance government state standard architecture engineering library collection standard print format spreadsheet standard holding standard aael standard engineering enginlibrariansumichedu university michigan arbor campus affiliate library standard access nonum user standard collection material affiliate architecture engineering library source art architecture engineering library library area standard internet standard supplier document delivery service store material material link library university michigan department engineering cee blue work author staff student cee department center system factsheets factsheets statistic chart topic energy material material sustainability indicator change protection agency epa information protection agency document regulation department energy multimedia physic material cleanup energy technology energy state survey range information area earth science biology geology map water wastewater engineering www library link website field wastewater engineering institution association engineering science professor association engineering science professor professor program world education science technology protection institution aeesp member university world society engineering education asee society engineering education institution individual institution education engineering engineering technology mission excellence instruction service experience leadership education society quality product service member society soil mechanic engineering issmge issmge body interest activity engineer academic contractor world engineering union agu vision community cooperation understanding earth space benefit humanity society engineer society engineer member engineering profession worldwide engineering society asces vision position engineer leader quality life water association iwa water career science technology experience member country water association awwa awwa material water member knowledge water material growth water wastewater treatment technology water storage distribution utility management operation knowledge info advocacy quality supply water america advance health safety welfare effort spectrum water community water environment federation water environment federation association education training thousand water quality career water environment wef member health community water worldwide career material company industry profile intelligence company compilation career information management tool internship industry profession company data insight time employer selection decision report range industry ibisworlds industry market report industry month industry data ibisworld industry data enables analysis growth environment issue industry orbis orbis information company company country company company company company company career collection art achitecture engineering library collection material collection test guide book tip resume cover letter information job engineering book catalog online floor aael whats collection reference desk computer cluster material engineering career material center office engineer world internship job job link link career information job website engineering job material center ums center assistance workshop training session year student job search career exploration job book text online subscription catalog search ebooks job search topic resume martin yate isbn publication date edition knock resume example resume example sample stage career career yate advice profile keywords search engine resume top pile dont flipflops interview paul power publication date dont flipflops interview strategy technique market killer cover letter edition sandra podesta paxton isbn publication date guide cover letter competition interview question dummy rob yeung isbn publication date interview question dummy teach interview condition interview williams publication date interview guidance interview dream job job interview manager answer job martin isbn publication date job interview factor job question element résumé style scott bennett isbn publication date element résumé style reader compelling résumés cover letter service mlibrary lot service ask question material service ask service messaging service mind copyright copyright website right instructor andor creator blue data work blue access repository article data set image database groundwork poster edit video clip groundwork place duderstadt center consultant day poster printing ampm weekday loan doesnt article book loan service website poster bibliography software scholarspace workshop sort software oneonone session data need data software clark library sand north lab</t>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>environmental engineering left find environmental engineering find articles database environmental engineering find book book art architecture engineering library standard quick guide find industrial standard resource internet resource useful environmental engineering professional organization association society important environmental career resource engineering career job hunt useful library library useful guide apply climate resource climate science civil engineering landscape architecture material science engineering environment sustainability virtual geosicences library essential library video tutorials library put short video tutorial interest relevant topic interest find book suggest title recommend title purchase library fill find ebook collection accessengineering complete mcgraw hill engineering handbook knovel engineering scientific electronic version popular book engineering applied science feature book different publisher include handbook conference proceeding wiley library article book publish wiley blackwell resume life health physical science social science humanity find book find book environmental engineering word title library catalog word best starting appropriate title find want subject heading list title guide encyclopedias handbook dictionary resource university michigan affiliate student staff faculty visit knovel accessengineering taylor francis ebooks job environmental handbook bela liptak editor david liu editor isbn article environmental handbook second edition single resume depth interrelated factor principle affect environment deal past deal today deal future civil engineering handbook chen editor richard liew editor isbn article publish civil engineering handbook know field definitive engineering handbook richard dorf editor isbn article engineering handbook design enlighten expert area specialty refresh knowledge mature practitioner educate engineering novice handbook ecomaterials leticia myriam torres editor oxana vasilievna kharissova editor boris kharisov editor isbn article handbook editor present maximum possible known eco material include cyclic material material ecology environmental protection material society human health material energy base main criterion function material material enhance refrain damage environment life cycle handbook civil engineering calculation third edition tyler hick isbn article handbook civil engineering calculation feature organize calculation align late practice code standard water wastewater calculation manual third edition shun dar lin isbn article water wastewater calculation manual basic principle best practice detailed calculation surface water groundwater drinking water treatment wastewater engineering hydrogeology field manual willis weight isbn article hydrogeology field manual late applied application groundwater sampling water quality assessment aquifer characterization contamination issue karst application water wastewater engineering design principle practice second edition mackenzie davis isbn article depth guide water wastewater engineering revise reflect late advance procedure regulation authoritative resource contains comprehensive coverage design construction municipal water wastewater facility citation tool library different tool manage footnote bibliography tool endnote mendeley expert fromscholarspace endnote buy software install computer endnote guide free firefox extension computer library sit machine good cite resource beta visit zotero guide mendeley mendeley citation tool collect organize citation insert report format bibliography visit mendeley guide article asce citation style complete guide asce citation style section chapter find asce text report asce author method smith smith jones report include section list last author publish job thesis dissertation forthcoming article exception rule examples asce style referenced follow book evans furlong environmental biotechnology theory application chichester wiley specific chapter chapter title inclusive include article article beskos boundary element method dynamic analysis appl mech rev doi asce article article asce long asce style asce article article conference proceeding eschenaur kulicki mertz retrofit distortion induce fatigue cracking noncomposite steel girder floorbeam stringer bridge proc annual int bridge conf pittsburgh society western pennsylvania abstract article article conference report database complete list database environmental engineering library database citation wish find article library mgetit mget top databases water content water environment foundation water quality professional include conference proceeding manual practice standard article article fact sheet technical report ebooks scopus international multi disciplinary abstract database scientific medical technical social science database aqualine coverage trade technical scientific literature water resource supply water quality water waste analysis water treatment underground water sewage industrial effluent effect pollution aquatic science fishery abstract aquatic pollution environmental quality devote policy contamination ocean seas lake river estuary engineering village compendex broad subject area engineering apply science represent coverage include nuclear technology bioengineering transportation chemical engineering light optical technology agricultural engineering environmental engineering abstract abstract article relate engineering aspect air water quality environmental safety energy production agricultural environmental science database multidisciplinary database comprehensive coverage environmental science abstract citation draw serial include scientific article conference proceeding report monographs book government article google scholar availability michigan google mgetit library holding greenwire report national environmental energy natural resource issue address white house federal agency court state major medium country sign daily alert important story onepetro library literature oil gas exploration production industry pollution abstract pollution abstract environmental concern scientific government policy atmosphere emission environmental action response global pollution issue proquest technology collection database combine full text article indexing global literature technology apply science include material science aerospace engineering mechanical engineering civil engineering condense matter physic computer science electronic engineering incorporate proquest engineering collection proquest advance technology aerospace collection proquest material science collection deep indexing technology scholarship science key article major article area science technology find article cite specific article footnote reverse scifinder chemical abstract article patent technical report dissertation conference proceeding book biochemistry physical inorganic analytical chemistry water resource abstract comprehensive coverage water resource issue include groundwater lake estuary water supply desalination water yield water quantity groundwater watershed water quality wastewater water law citation tool library different tool manage footnote bibliography tool endnote mendeley expert scholarspace endnote buy software install computer endnote guide free firefox extension computer library sit machine good cite resource beta visit zotero guide mendeley mendeley citation tool collect organize citation insert report format bibliography visit mendeley guide standard finding standard standard find industry standard astm iso society standard standard art architecture engineering library copy standard art architecture engineering library standard base issuing agency astm standard american society test material astm compass aami association advancement medical instrumentation aami standard aami esubscription institutional american association state highway transportation official astm compass aci american concrete institute standard publish aci manual concrete practice aiaa american institute aeronautics astronautics standard aerospace central standard american institute steel construction aisc include ansi aisc specification structural steel asce standard american society civil asce library asme american society mechanical standard include boiler pressure vessel code asme standard collection institutional aws standard american welding society astm compass awwa standard american water job association astm compass awwa standard knovel awwa standard knovel enter awwa standard awwa ansi american national standard institute compile record standard code federal regulation cfr incorporate ibr standard standard iso iec aham aws iapmo society host format downloading printing option cost esd eos esd association produce standard electrostatics esd standard complimentary downloads esda iec standard international electrotechnical commission astm compass ieee standard institute electrical electronics ieee accessible ieee iso iso international organization standardization publishes standard topic iso standard astm compass sae society automotive sae publishes standard mobility engineering include ground vehicle aerospace aerospace material standard historical sae standard sae mobilus smpte society motion picture television standard topic audio broadband control file image format ieee xplore usp standard united state pharmacopeia national formulary find usp personal account umich account leave subscription key blank personal account content log usp energy code fire energy code include standard international code council icc international code national fire protection association nfpa american society heat refrigerating air state michigan code mad cad nfpa national fire protection association code free nfpa underwriter laboratory standard format cost free require personal account payment require printing downloading hipaa health insurance portability accountability act hipaa outline national standard electronic health care transaction code set unique health identifier security find overview hipaa regulation health human department osha miosha occupational safety health administration osha standard osha michigan occupational safety health administration miosha standard miosha military specification department defense dod military standard free registration approval require dod assist coverage gain dod assist person art architecture engineering library municipal code municipal code ordinance local government united state municode historical standard art architecture engineering library maintain small collection supersede historical standard print format searchable spreadsheet standard holding historical standard aael standard list contact engineering librarian enginlibrarians umich affiliate university michigan arbor dearborn flint affiliate contact respective library standard non affiliate want standard collection visit library resource non affiliate art architecture engineering library art architecture engineering library include library area military standard internet standard supplier pay report delivery ansi accuris store resource internet resource following library find useful university michigan department civil environmental engineering cee deep blue job affiliate author faculty staff student cee department sustainable factsheets informative factsheets statistic chart topic energy material resource sustainability indicator climate change environmental protection agency epa environmental related environmental protection agency resume fulltext epa report regulation sciencecinema department energy multimedia physic chemistry material biology environmental cleanup energy technology renewable energy united state geological survey usgs usgs perform broad area earth science include biology geology map water wastewater engineering virtual library virtual library field wastewater engineering professional organization association environmental engineering science professor aeesp association environmental engineering science professor aeesp professor academic education science technology environmental protection found nonprofit organization aeesp member university american society engineering education asee found american society engineering education nonprofit organization institution commit education engineering engineering technology accomplish mission promote excellence instruction public_service practice exercise worldwide leadership foster technological education society quality product member international society soil mechanic geotechnical engineering issmge issmge pre eminent professional body represent interest activity academic contractor participate geotechnical engineering american geophysical union agu agu vision worldwide scientific community advance unselfish cooperation understanding earth benefit humanity american society civil asce found american society civil asce represent member civil engineering profession worldwide america old national engineering society asce vision position global build good quality life international water association iwa comprise leading water professional science technology practice corporate member spread country american water job association awwa found awwa authoritative resource safe water member worldwide share knowledge water resource water wastewater treatment technology water storage distribution utility operation awwa knowledge advocacy improve quality supply water america advance health safety welfare unite effort full spectrum water community water environment federation water environment federation profit association technical education training water quality professional clean water return environment wef member protect health serve local community support clean water worldwide career resource company industry resume vault career intelligence depth company resume compilation career tool internship industry profession company data insight frame employer selection decision ibisworld report wide industry ibisworld industry report resume wide industry update month ensure late industry data ibisworld industry data enables detailed analysis key growth trend competitive environment key issue face industry orbis orbis company include european company country canadian company central american company japanese company chinese company african company aael career collection art achitecture engineering library small collection dedicate career resource collection include standardized test guide book tip write resume resume resume job engineering book catalog come aael collection locate desk computer cluster resource engineering career resource office dedicate prepare find internship job ecrc job find career job specific engineering job resource career career assistance training training session student job_search career exploration job_searching book follow book full text library subscription library catalog find additional book job_search topic knock dead resume martin yate isbn article edition knock dead resume include resume industry specific examples sample resume professional career yate valuable advice include social network resume keywords engine move resume top pile flip flop interview paul power isbn article flip flop interview pack strategy technique practical easy humorous killer resume resume third edition sandra podesta andrea paxton isbn article guide write resume resume stand competition answer tough interview dummy rob yeung isbn article answer tough interview dummy teach perform stressful interview ultimate interview lynn williams isbn article ultimate interview give guidance prepare ace interview dream job say job interview understand manager ask give answer land job carole martin isbn article say job interview show focus factor job answer element style scott bennett isbn article element style show craft clear compelling target resume resume job useful library mlibrary lot check useful know ask librarian quick library resource try ask librarian instant messaging librarian library wide keep mind librarian speak aael check copyright sure copyright want copyright right instructor creator deep blue deep blue data want scholarly job archive deep blue institutional repository love article videos data set image database groundwork print poster edit video audio clip groundwork duderstadt consultant poster printing weekday interlibrary loan article book interlibrary loan scholarspace want poster bibliography software scholarspace host training sort software session schedule geospatial data map find data job software contact clark library sand north lab</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>30</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>密歇根大学-为表演艺术创业与领导力提供职业资源.docx</t>
+        </is>
       </c>
       <c r="B32" t="inlineStr">
-        <is>
-          <t>密歇根大学-为表演艺术创业与领导力提供职业资源.docx</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
         <is>
           <t>Overview
 Selected Subject Headings
@@ -4778,22 +4685,19 @@
 Global Music Rights - The newest music rights organization, formed in 2013, GMR seeks to be an active and progressive advocate for copyright holders in the current performing rights marketplace, protect the integrity of music rights, and promote the value of intellectual property on behalf of creators.</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>overview heading example heading leadership performing art catalog heading catalog search select subject menu search field heading list search field phrase result print material artist management music business ebook borwick doug community future art state hatcher cleveland art place artist work community institution art cutler music teacher blueprint income impact music flight class competition talent hatcher shapiro richard rise class shapiro gelb michael genius history mind community art growth gram diane betty community diversity change art aael hatschek keith dictionary music industry music reference journal art management ivey bill art greed neglect right art jones mark dancer watsonguptill guide program internship apprentice program artistinresidence program studio school teacher workshop festival music reference kaiser michael art turnaround art institution music kolb bonita marketing institution strategy audience passman donald music business music robinson mind power ebook schrag art life guide community music fine art jason ball guide art community growth ebook tharp habit life guide shapiro management art aael wacholtz larry entertainment insider career entertainment music industry music material school music theatre dance excel excellence career empowerment leadership excel lab success student alumnus workshop student project venture funding art seek performing art experience program student art way connection experience institution student role creator audience member leader art community endowment art agency funding support partnership state art agency leader agency philanthropic sector nea art affirms heritage work access art american art recognition support value art serve network institution individual art america assist artist art institution level ecosystem medium material support womenarts institution woman artist material work networking fundraising advocacy service york foundation art artist information award service publication artist art career work press publishes information career artist photographer designer author institution idealist people chance action collaboration michigan council art affair state michigan agency art culture policy grantmaking collaboration variety sector partner society art education institution training standard art education capital institution artist discipline country counsel gathering career growth service createquity tank issue art institution people place economy michigan advocacy experience communication dataarts institution art leader highquality data material insight challenge impact print material art entrepreneurship music fitterman introduction music industry approach ebook gordon future music business technology guide artist entrepreneur shapiro hjorth daniel chris steyaert approach entrepreneurship movement entrepreneurship book ebook kander diana startup idea line kolb entrepreneurship industry art matthew charles innovation competency framework aael munoz mark julienne shield art art shapiro nytch muse career music music rabideau mark artist entrepreneurship stcentury music sabino career passion fulfilling aael shapiro sorin gretchen sullivan session entrepreneurship institution hatcher varbanova entrepreneurship art material entrepreneurship journal entrepreneurship art center entrepreneurship experience student faculty class program individual chance problem institution endeavor alliance art university work range curriculum program experience articulate role education society michigan association membership institution nonprofit sector advocacy training material culture source member association art institution southeast michigan work institution expression region art blog aim understanding art community interview spotlight project post content endowment art agency funding support partnership state art agency leader agency philanthropic sector nea art affirms heritage work access art council art affair leader program growth initiative advancement michigan art leader state michigan agency art culture policy grantmaking collaboration variety sector partner art approach concept entrepreneurship perspective relationship producer consumer art community exchange nonprofit consulting firm strategy tool institution people life change partnership nonprofit foundation government agency york foundation art entrepreneurship material material institution artist information award service publication artist art career work institution business owner manager arbor area experience knowledge business owner success innovate hub entrepreneurship innovation work idea action connecting network community aim foster collision experience art design engineering technology potential student faculty campus institution community driven passionate student platform comfort zone community leader startup incubator student step ideation ginsberg center partnership community university michigan order change detroit entrepreneurship network network student school student share passion entrepreneurship revival career material material career career center student transition university michigan material service career guide film television medium career school education career service team suite service material student alumnus skill training order career success material career job posting job career navigator guide career planning site position relates market title career family classification system england conservatory bridge subscription material thousand job chance year world orchestra job position festival competition art administration role art grant job job listing site art industry classified job listing part digest art journalism englishspeaking world culture source job chance job listing section website member association art institution southeast michigan work institution expression region art deadline list site art commission competition job internship scholarship grant fellowship residency festival entriesproposalsprojects chance discipline art student teacher artist age skill level discipline subscription list guarantee access announcement york foundation art growth chance offer institution artist information award service publication artist art career work job chance job listing section website institution people place economy michigan advocacy experience communication material stcentury singer leap university world mohini century tip trend technique film stage digital medium stephanie bartonfarcas call aael shapiro business mistake success actor paul russell call actor york city actor need apple alterman call talent career music myles call music career opera school james music business basic musician guide start success bobby borg call music career dance guidance field duffy call music composing screen scott hallgren music dance experience workplace challenge chance dance career student educator pickard doug risner music career audio industry tucker call eat time sequel donts acting job tom music business tip loyal living herstand call music music business management production concert festival reynolds ebook band guide management stephen marcone philp call music music business career duality industry cheryl slay carr call music shapiro music business essential guide career mark cabaniss call music shapiro music business guide career guide baskerville tim baskerville call shapiro music industry document musician feist call music music producer chaos creativity career music jackson call project management musician recording concert studio feist call music singer audition career guide claudia friedlander call music ballet dancer jennifer carlynn music stage actor tradition protocol etiquette michael kostroff julie garnyé call aael wing career broadway haas glatzer call music musician success value world kris hawkins music fundingfinance print material path artist audience income career sustainability zane forshee manceor mcginness call artist guide artist performing art peter cobb felicity hogan michael art shapiro funding material library grant database school music theatre dance excel funding chance graduate school funding chance chance institution foster collision experience art design engineering technology potential student faculty campus art chance institution student role creator audience member leader art community peer mentorship minigrants music theatre dance student performance residency community council art affair chance state michigan agency art culture policy grantmaking collaboration variety sector partner chance member association art institution southeast michigan work institution expression region material institution woman artist material work networking fundraising advocacy service annuityfreedomnet grant artist institution information online finance material finance database finance partner community infrastructure service tax compliance planning student service material planner rackham graduate school student service credit union wellness program workshop knowledge artist support group student artist selfadvocacy advocate change cost education way student loan debt budget income artist safety craft emergency relief fund cerf serf artist craft discipline safety net career core service education program network building emergency relief deloitte article art finance material service provider audit assurance risk tax service material music law age music charlotte waelde guide property industry champion walter kirk willis thornton property law sport entertainment industry field corey entertainment law fundamental experience music gordon contract artist songwriter producer music halloran mark musician business guide music moser david cheryl slay music copyright law music reference schulenberg aspect music industry insider music reference shapiro enterprising musician contract music material law patent trademark database student service student right county court copyright office information individual decision sharing material endeavor center property basic series material institution experience student faculty class program individual chance problem institution endeavor arbor area score material list material institution business owner manager arbor area experience knowledge business owner success material individual problem lawyer lawyer economy service institution people place economy michigan advocacy experience communication directory volunteer lawyer art lawyer art service material client area art effort individual institution business issue contract copyright trademark area medium right art property volunteer lawyer institution list program california school law service creator entrepreneur journalist internet user art labor union actor equity association art theatre component society career member wage condition range benefit health pension plan actor federation television radio artist work jurisdiction wage condition health pension benefit member chance contract member work guild variety artist artist stage manager performance variety field singer dancer touring show revue nonbook theme park performer skater performer comedian comic cabaret club artist lecturerspoetsmonologistsspokespersons variety performer party event writer america east individual content motion picture television news medium contract creative right member program workshop event issue interest writer writer view body government director america seek team right freedom ability career alliance stage employee technician artisan craftspersons entertainment industry theatre motion picture television production trade show director adg individual world production designer director title artist designer model maker illustrator artist artist artist designer artist craftspeople department coordinator craft standard condition wage entertainment art industry stage director choreographer community stage director choreographer right health livelihood exchange idea information chance negotiating support guild artist artist discipline dance heritage institution labor experience federation musician union musician world labor experience member right institution performance song behalf songwriter composer music publisher society composer author publisher song score songwriter composer music publisher member music inc music right institution performance work songwriter composer music publisher music right music right institution gmr seek advocate copyright holder performing right marketplace integrity music right value property behalf creator</t>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>overview subject heading subject heading relate entrepreneurship leadership performing art useful browse library catalog subject heading library catalog advanced subject pull next field enter heading list field quote phrase precise result print resource allen paul music_business book borwick doug build community audiences future art united state hatcher cleveland art job america community social institution fine art cutler savvy music teacher blueprint maximize income impact music florida flight creative training global competition talent hatcher shapiro florida richard rise creative training revisit shapiro gelb michael discover genius think history ten revolutionary mind goldbard arlene creative community art cultural aael gram diane betty farrell enter cultural community diversity change nonprofit art aael hatschek keith historical dictionary american music_industry music international article art hatcher article ivey bill art inc greed neglect destroy cultural right fine art jones mark dancer resource watson guptill guide academic internship apprentice residential residence studio university teacher training festival music kaiser michael art turnaround maintain healthy art organization music kolb bonita marketing cultural organization strategy attract engage audience aael passman donald know music_business music robinson ken mind power creative book schrag brian art good life guide job community music fine art schupbach jason ball eds creative placemaking action orient guide art community book tharp creative habit life practical guide shapiro lidia strategic art aael wacholtz larry monetize entertainment insider handbook career entertainment music_industry music resource university music theatre dance excel lab excellence entrepreneurship career empowerment leadership excel lab catalyze success smtd student alumnus weekly training mentor student project venture funding art michigan seek integrate visual performing literary art undergraduate experience engage student art meaningful build connection academic curricular experience organization job support student diverse work creator audience member university art community national endowment art independent federal agency funding support partnership state art agency local federal agency philanthropic sector nea support art affirms celebrates america rich diverse cultural heritage extend job promote equal art american art job build recognition support extraordinary dynamic value art lead serve advance diverse network organization cultivate art america fracture atlas assist art organization cultural ecosystem creative medium fiscal sponsorship educational resource personalized support womenarts organization dedicate woman resource creative job free networking fundraising advocacy foundation art job empower complete accurate award article art professional facilitate artistic job allworth press publishes job practical creative professional photographer designer author idealist organization job connect idealist want good action collaboration michigan council art cultural affair state michigan lead agency charge develop art culture policy grantmaking collaboration wide sector partner society art entrepreneurship education organization commit advance formal training high educational standard art entrepreneurship education creative finance organization support creative discipline country fund counsel gathering career_development createquity think tank investigate important issue art address creative statewide organization develop creative creative creative economy michigan advocacy professional practice communication dataarts organization seek empower art cultural high quality data evidence base resource insight overcome challenge increase impact print resource beckman gary discipline art teach entrepreneurship context music fitterman radbill catherine introduction music_industry entrepreneurial approach book gordon steve future music_business succeed digital technology guide entrepreneur shapiro hjorth daniel chris steyaert narrative discursive approach entrepreneurship second movement entrepreneurship book book kander diana startup launch idea line kolb bonita entrepreneurship creative cultural industry fine art matthew charles innovation entrepreneurship competency framework aael munoz mark julienne shield art entrepreneurship fine art shapiro nytch jeffrey entrepreneurial muse inspire career classical music music rabideau mark revolutionary entrepreneurship century musician music sabino creative career turn passion fulfilling rewarding lifestyle aael shapiro sorin gretchen sullivan lynne session eds cultural entrepreneurship relevant sustainable institution hatcher varbanova lidia international entrepreneurship art resource library entrepreneurship databases artivate article entrepreneurship art article entrepreneurship active experience student faculty training design prepared identify act solve problem organization entrepreneurial endeavor alliance art university job advance full art integrative curriculum creative practice acknowledge articulate expand vital work higher_education global society michigan association membership organization dedicate serve diverse nonprofit sector advocacy training resource culture member association non profit art cultural organization southeast michigan seek advance job organization cultivate creative cultural expression art job blog aim enrich understanding art art job community interview spotlight nea support project guest post content national endowment art independent federal agency funding support partnership state art agency local federal agency philanthropic sector nea support art affirms celebrates america rich diverse cultural heritage extend job promote equal art michigan council art cultural affair rise personal initiative commit advancement michigan art state michigan lead agency charge develop art culture policy grantmaking collaboration wide sector partner entrepreneurship art present different approach concept entrepreneurship various perspective relationship producer art community resource exchange nonprofit consulting firm seek strategy tool build sustainable high performing organization improve life drive social change partnership nonprofit foundation government agency foundation art entrepreneurship resource resource organization job empower complete accurate award article art professional facilitate artistic job score organization experienced business owner manager great ann arbor area volunteer experience knowledge potential exist small business owner achieve success innovate blue hub entrepreneurship innovation job turn idea action support connecting expand michigan entrepreneurial network community artsengine aim inspire foster strengthen intellectual collision durable collaborative practice drive art design engineering technology maximize potential student faculty north mpowered student sponsor organization strive bring community driven passionate student platform push comfort zone give entrepreneurial community grow startu entrepreneurship student run startup incubator student job entrepreneurial ideation fund ginsberg aim cultivate steward equitable partnership community university michigan order advance social change good detroit entrepreneurship network network student mentor high university student share passion entrepreneurship revival detroit career resource resource library career databases career job support student transition university michigan numerous resource theatre drama career guide film television medium career university education career_services student commit comprehensive tailor suite resource empower student alumnus leverage skill training order achieve maintain lifelong career success human_resources career job posting job career navigator guide assist personal career planning show position relates title career family classification england conservatory bridge subscription resource list job orchestra job teach position festival competition art administration work art grant job international job listing large call art creative industry artsjournal classified job listing include digest art cultural journalism english speaking culture job_opportunities job listing section member association non profit art cultural organization southeast michigan seek advance job organization cultivate creative cultural expression art deadline list list art commission art competition art job internship art scholarship grant fellowship residency art festival call entry proposal project discipline art student art teacher age skill discipline subscription premium list guarantee announcement foundation art professional offering organization job empower complete accurate award article art professional facilitate artistic job creative job_opportunities job listing section statewide organization develop creative creative creative economy michigan advocacy professional practice communication print resource century singer leap university susan mohini kane call act audition century tip trend technique film digital medium stephanie barton farcas call aael shapiro act business avoid mistake achieve success job actor paul russell call shapiro actor guide city actor survive succeed big apple glenn alterman call aael talent successful career music angela myles beeching call music build career opera university operapreneurship james harrington call music_business basic musician complete handbook start success bobby borg call music career dance practical strategic guidance field ali duffy call music composing screen scott hallgren call music dance professional practice workplace challenge dance professional student educator angela pickard doug risner eds call music find career modern audio industry april tucker call book act eat sequel land professional acting job tom logan call aael music_business practical tip build loyal follow living musician ari herstand call music live music_business production concert festival andy reynolds call book manage band guide stephen marcone david philp call music music_business career career duality creative industry cheryl slay carr call music shapiro music_business essentials guide aspire professional mark cabaniss call music shapiro music_business handbook career guide david baskerville tim baskerville call shapiro music_industry important report modern musician jonathan feist call music shapiro music producer survival guide chaos creativity career independent electronic music brian jackson call project musician recording concert tour studio jonathan feist call music singer audition career handbook claudia friedlander call music want ballet dancer jennifer carlynn kronenberg call music actor handbook tradition protocol etiquette aspire professional michael kostroff julie call aael wait wing launch perform career broadway tiffany haas jenna glatzer call music shapiro job musician handbook professional success establish value real kris hawkins call music funding finance print resource path fund guide build audience generate income realize career sustainability zane forshee christina manceor robin mcginness call book profitable handbook performing literary visual art peter cobb felicity hogan michael royce call fine art shapiro funding resource library grant fundraise database university music theatre dance excel funding rackham graduate_school funding artsengine fund support organization aim inspire foster strengthen intellectual collision durable collaborative practice drive art design engineering technology maximize potential student faculty north art michigan fund organization job support student diverse work creator audience member university art community peer mentorship mini grant music theatre dance student educational performance residency underserved community michigan michigan council art cultural affair fund state michigan lead agency charge develop art culture policy grantmaking collaboration wide sector partner culturesource fund member association non profit art cultural organization southeast michigan seek advance job organization cultivate creative cultural expression womenarts fund resource organization dedicate woman resource creative job free networking fundraising advocacy annuityfreedom net grant micro grant organization free financial finance resource library finance database finance partner community financial infrastructure tax compliance planning student financial human_resources financial planner rackham graduate_school student financial credit union financial wellness educational training aim strengthen financial knowledge artists financial support seek educate student professional financial self advocacy advocate legislative institutional change cost education innovate manage student loan debt budget erratic income cerf safety net craft emergency relief fund cerf serf job craft discipline safety net support strong sustainable career core education advocacy network emergency relief deloitte article art finance resource lead global provider audit assurance consult financial advisory risk advisory tax relate legal lselected print resource bargfrede allen mak music law digital age music abbe charlotte waelde eds handbook intellectual property creative industry book champion walter kirk willis patrick thornton intellectual property law sport entertainment industry aael field corey entertainment law fundamental practice music gordon steve contract songwriter producer know music halloran mark musician business legal guide music moser david cheryl slay music copyright law music schulenberg richard legal aspect music_industry insider music shapiro williams david enterprising musician guide performer contract music resource library law legal databases library patent trademark database student legal advise student regard legal right represent washtenaw county court library copyright office decision sharing copyright material creative endeavor teach entrepreneurship intellectual property basic video resource organization active learning experience student faculty training design prepared identify act solve problem organization entrepreneurial endeavor ann arbor area score legal resource list resource organization experienced business owner manager great ann arbor area volunteer experience knowledge potential exist small business owner achieve success michigan legal resource handle legal problem lawyer creative lawyer creative economy statewide organization develop creative creative creative economy michigan advocacy professional practice communication national volunteer lawyer art lawyer creative art free legal resource eligible client area art effort assist organization business issue contract copyright trademark legal area medium right art intellectual property volunteer lawyer organization list fund non profit western university law legal creator entrepreneur journalist internet perform art labor union actor equity association seek foster art live theatre essential component society advance career member negotiate wage improve job wide benefit include health pension plan screen actor guild american federation television radio sag commit organize job jurisdiction negotiate best wage job health pension benefit preserve expand member job enforce contract protect member unauthorized job american guild represent perform manager live performance field include singer dancer touring show theatrical revue non book show theme park performer skater circus performer comedian stand comic cabaret club lecturer poet monologist spokesperson performer job party special event writer guild america east west represent write content motion picture television digital medium negotiate administer contract protect creative economic right member conduct seminar event issue interest writer present writer various body government director guild america seek protect directorial legal artistic right contend creative freedom strengthen ability develop meaningful credible career international alliance theatrical employee iatse represent technician artisan craftspersons entertainment industry include live theatre motion picture television production trade show art director guild iatse local adg represent job production designer art director scenic title graphic set designer model maker illustrator matte previs unite scenic iatse local represent designer craftspeople department coordinator job protect craft standard job wage entertainment decorative art industry director choreographer society seek foster national community professional director choreographer protect right health livelihood facilitate exchange idea administrative negotiating contractual support american guild musical represent numerous discipline america operatic dance choral heritage job guarantee artistic institution fair labor practice american federation musician large union musician advocate fair labor practice member perform right organization sesac license performance song behalf affiliated songwriter composer music publisher american society composer author publisher ascap license ascap song score songwriter composer music publisher govern member broadcast music inc large music right organization protect performance musical job songwriter composer music publisher global music right music right organization gmr seek active progressive advocate copyright holder performing right protect integrity music right promote value intellectual property behalf creator</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>31</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>密歇根大学-学生工作.docx</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
-        <is>
-          <t>密歇根大学-学生工作.docx</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
         <is>
           <t>Students
 Jobs for Students
@@ -4814,22 +4718,19 @@
 A 12-week internship for current and recent graduate students to work on an archival processing project.</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>student job student position student program lead project effort library student fellow ambassador scholar experience project focus internship design student position hardworking team lab data visualization fellowship summer chance project cohort support expert summer fellowship user experience chance graduate student experience design system mark theresa preservation internship program contribute preservation project internship student level collection center archival program week internship graduate student archival processing project</t>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>student job student browse pay position student student engagement take lead project promotional programmatic effort library paid student fellow ambassador michigan library scholar hand professional experience job project international focus paid internship design lab student position join hardworking keep lab run data visualization fellowship pay summer job project cohort support library expert summer fellowship library experience pay graduate student gain experience design digital library mark theresa lafer preservation internship contribute distinctive preservation project internship student various academic special collection archival internship week internship recent graduate student job archival processing project</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>32</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>密歇根州立大学 通用型.doc</t>
+        </is>
       </c>
       <c r="B34" t="inlineStr">
-        <is>
-          <t>密歇根州立大学 通用型.doc</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
         <is>
           <t>Business Career Research
 Business News
@@ -4904,22 +4805,19 @@
 CPA Salaries</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>business career business news wall street harvard business bloomberg economist analyst report link window statistic company interview preparation material company industry depth interview interviewer company position industry firm competitor advantage company move guide material job answer question link windowthis material staff student netid company profile industry report country city information deal industry medium influencers news article company profile analysis industry report porter force intellect link windowthis material staff student netid access hoover company data directory consumer industry profile privco link windowthis material staff student information financials company market deal venture capital funding market investor online material staff student netid company data company company company filing report link windowthis material staff student netid source newspaper state source company country company guide database option industry addition company industry sense landscape trend chance company competitor link windowthis material staff student netid company profile industry report country city information deal industry medium influencers news article company profile analysis industry report porter force ibisworld link windowthis material staff student netid level analysis industry state state canada china supply chain market share ease entry industry data mergent link windowthis material staff student netid industry report market analysis landscape characteristic condition business challenge industry industry growth state profile sale marketing communication template industry prospector industry characteristic passport gmid link windowthis material staff student netid job country industry information consumer lifestyle trend business dynamic link windowthis material staff student contains market report focus information freedonia industry category chemical component energy pharmaceutical plastic electronics life science industry topic biotechnology device diagnostics link windowthis material staff student netid market report consumer market emphasis market report market share segmentation trend consumer demographic product introduction consumer good market track trend ingredient market category food beverage beauty care household good pet care report mintel gnpd industry guide database option insight link windowthis material staff student netid material career guide career guide city job posting information employer directory outlook guide career profile duty occupation work environment occupation education training occupation pay worker occupation job outlook decade occupation career discover occupation industry state profile industry profile job wage trend state metropolitan county level career profile industry job information job duty requirement trend outlook msu career service career service connect russell career management center career center coach student career aspiration employer alumnus spartan world business internshipsjobs handshake career management platform student employer alumnus job internship chance interview company career management center event material profile resume education internship program type internship link windowthis material staff student netid material career guide career guide city job posting information employer directory filter area search job function area result job type internship calculation tool news job report cost calculator job seeker calculator bls wage estimate finder cpa salary</t>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>business career business wall article harvard business bloomberg economist analyst report mergent investext statistic statista company interview preparation resource company industry depth prepare interview interviewer ask perceive company position industry firm competitor competitive advantage company best move guide resource explore job prepare answer inform marketline windowthis resource faculty staff student log netid company resume industry report country city financial deal industry social medium influencers article company resume swot analysis industry report porter force analyse mergent intellect windowthis resource faculty staff student log netid hoover international company data contain industry resume privco windowthis resource faculty staff student log netid finance company deal venture finance funding investor mergent resource faculty staff student log netid comprehensive company data international company company company include sec filing historical annual report university windowthis resource faculty staff student log netid local regional national report united state strong legal company country company guide database option industry addition company industry operate give sense competitive landscape speak trend face company competitor marketline windowthis resource faculty staff student log netid company resume industry report country city financial deal industry social medium influencers article company resume swot analysis industry report porter force analyse ibisworld windowthis resource faculty staff student log netid readable high analysis industry united state state worldwide canada china include supply chain share ease entry industry data mergent windowthis resource faculty staff student log netid basic global industry report analysis include competitive landscape characteristic operate business challenge industry trend historical industry growth contain state resume sale marketing communication template industry prospector rank industry base certain characteristic passport gmid windowthis resource faculty staff student log netid helpful seek employment passport country specific industry lifestyle trend business dynamic marketresearch windowthis resource faculty staff student log netid contains report freedonia focus kalorama freedonia resume eighteen industry category include automotive chemical industrial component energy pharmaceutical plastic electronics kalorama resume life science industry topic include pharmaceutical biotechnology medical device diagnostics mintel windowthis resource faculty staff student log netid report resume global emphasis european report analyze share segmentation trend demographic product introduction package good useful keep track trend ingredient package category include food beverage beauty personal care household good pet care academic report mintel gnpd industry guide database option career insight global windowthis resource faculty staff student log netid resource country specific career guide city specific career guide large city canada job internship posting employer occupational outlook handbook career resume describe typical duty perform job job environment job typical education training enter job median pay worker job job outlook come decade job career discover comprehensive job industry state resume industry resume include employment wage trend national state metropolitan county climbtheladder depth career resume industry job include job duty salary requirement trend outlook msu career_services msu career_services msu connect russell palmer career broad career advise coach educate student realize career aspiration job lead employer alumnus send spartan business internship job handshake handshake msu career platform connect msu student employer alumnus job internship sign interview find company russell palmer career event resource complete resume upload resume broad education international internship international internship global windowthis resource faculty staff student log netid resource country specific career guide city specific career guide large city canada job internship posting employer internship filter pick geographic area job function area limit result job internship salary calculation tool best job report cnn cost live calculator job seeker salary calculator bls wage estimate salary finder cpa salary</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>布朗大学 艺术就业指南.doc</t>
+        </is>
       </c>
       <c r="B35" t="inlineStr">
-        <is>
-          <t>布朗大学 艺术就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
         <is>
           <t>Careers, Internships &amp; Grad Schools
 Copyright
@@ -4968,22 +4866,19 @@
 Regularly offered workshops include Grant Finding.</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>career internship school copyright school blog post state office benefit art statement statement guideline companyart project karen sht college art artist statement manifesto contains book website material artist statement statement hotchkiss site institution material architecture association karen caa news newsletter college art association america job residency community alliance job listing listing job art chronicle education journal education listing job chance user college association career center art job education material member caa order access listing job listing job education account resume printmaker reception street studio luna collection graduate school program program history caa directory edition college art association download website graduate program directory edition college art association download website association college art design consortium art school contains information program material architecture art school program karen list art school type link school tale poetry contest handscroll collection grant college art association information grant conference internship university fellowship program fellowship workshop tutorial workshop finding</t>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>career internship grad university copyright wish teach copyright art university blog post united state copyright office benefit art job statement statement guideline gyst ink run company art project karen cornish university art library statement manifesto contains book resource write statement write statement write sarah hotchkiss creative independent professional organization resource art architecture association maintain brown librarian karen caa newsletter university art association america present job internships residency community alliance job listing searchable listing job art field chronicle higher_education main article job higher_education include comprehensive listing job_opportunities limit brown university art association career find art job higher_education resource member caa order listing high job listing job higher_education searchable account free resume post unknown printmaker artists reception tenth studio wood engrave luna collection graduate_school graduate art_history caa late edition publish university art association free graduate visual arts caa late edition publish university art association free association independent university art design consortium lead art university canada contains resource art architecture art university maintain brown librarian karen wikipedia list art university categorize include university unknown japanese tale genji poetry guess contest handscroll luna collection grant fellowships university art association update grant conference internship brown university fellowship university sponsor include competitive fellowship library training tutorial training include grant finding</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>康奈尔大学  和理工学院合作，针对理学生.docx</t>
+        </is>
       </c>
       <c r="B36" t="inlineStr">
-        <is>
-          <t>康奈尔大学  和理工学院合作，针对理学生.docx</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
         <is>
           <t>Home
 Welcome!
@@ -5333,22 +5228,19 @@
 Skillsoft - All active students, faculty, and staff have access to Skillsoft's online learning and books through Cornell's enterprise account. Choose from thousands of courses, books, videos, and other resources to help you stay sharp. The following topics are repr...</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>home welcome welcome cornell tech library service career career management team cornell tech information company industry interview list company company swot report time information career service information need startup career material interview company email consultation business day database equity venture capital database time data deal identify comparables search investor detail user account cornell email address log log sso cornell email address capital capital platform data company investment firm transaction people financials company company indepth market strategy report technology transportation energy ibisworld industry report profile state industry range industry canada china newspaper time student faculty staff account cornell email address apps conjunction account york time access article york time factiva student law library access street journal cornell student faculty staff account cornell email address apps conjunction account news industry read question need information cornell tech library service thing suggestion exploration career exploration expertise time information career librarytechcornelledu example list employer database capital pitchbook guidestar premium intellect industry report overview material ibisworld frost sullivan mergent path day life information material example trade association report information linkedin material search network access job opening work library information networking networking library linkedin connection interest chance access job search article point harvard business issue guide job job strength tie network culture youre linkedin learn introduction access harvard business business source search article search publication link issue menu date issue article issue email librarytechcornelledu question alumnus cuelinks cuelinks cornell platform connect cornell alumnus peer friend cornell career goal material list core material career career planning vault vault guide job series career industry information work environment education requirement day life career outlook job tool career company capital company sheet feature factiva download custom company financials growth product news article industry insight report snapshot industry china state report industry performance outlook company chain demand structure barrier entry statistic indepth market strategy report coverage technology space growth chance technavio niche industry specialty chemical material health care energy user report month mergent intellect navigate report industry interest call prep executive insight section question informationals interview company news article factiva aka thousand newspaper business periodical article company official firm finance career book hour job search edition dalton call publication date approach interview employer ferrazzi tahl raz call publication date guide art networking reveals principle relationship ferrazzi tahl raz call online copy isbn publication date guide art networking reveals principle relationship friend influence people carnegie call bfs publication date guide relationship suggestion people business situation book engineering library diversity stem material book delivery book print book cornell university catalog request book record select cornell tech campus delivery location book bloomberg center security book bloomberg center security desk book access delivery email librarytechcornelledu question startup entrepreneurship startup student founder information material search strategy library information time oneonone consultation member team email librarytechcornelledu walkthrough material library zoom question pitchbook pitchbook pitchbook data equity space information thousand equity venture capital deal investor fund source data venture capital association pitchbook benchmark time data deal identify comparables search investor detail cornell email material industry insight indepth market strategy report coverage technology space growth chance technavio niche industry specialty chemical material health care energy user report month market mintel report market variety sector consumer good travel tourism industry internet industry retail food drink account cornell email address ibisworld report snapshot industry china state report industry performance outlook company chain demand structure barrier entry statistic sense size company navigate report industry interest call prep executive insight section question informationals interview competitor industry report information company space profile expense business segment analysis capital screening feature list firm market pull financials firm deal market venture capital pitchbook explore type technology news topic report investor fund market map space market analysis analyst vertical source data venture capital association cornell email address log option note downloads day month whichever account year user account access association industry association source information example participant customer discovery interview sale list competitor association report article topic interest member smarter search tip search google limit site search government institution keywords sitegov siteorg keyword filetypepdf result highquality source whitepapers report tip nonprofit space researcher space google scholar result cornell library google scholar setting link cornell university search link article access cornell access material youre tech campus entrepreneurship list serve link list material library congress business guide entrepreneur book art start guy kawasaki call product service company division show way step art start guy kawasaki call publication date time decade kawasakis guide launching product service idea success startup ries online failure startup approach globe way company product book delivery book print book cornell university catalog request book record select cornell tech campus delivery location book bloomberg center security book bloomberg center security desk book access delivery email librarytechcornelledu question role material role software engineer data engineer data scientistanalyst librarian expertise time information career email librarytechcornelledu core material list material career career planning vault vault guide job series career industry information work environment education requirement day life career outlook job tool career company capital company sheet feature factiva download custom company financials growth product news article industry insight report snapshot industry china state report industry performance outlook company chain demand structure barrier entry statistic indepth market strategy report coverage technology space growth chance technavio niche industry specialty chemical material health care energy user report month mergent intellect navigate report industry interest call prep executive insight section question informationals interview company news article factiva aka thousand newspaper business periodical article company official firm finance interview preparation interview edition laakmann mcdowell call isbn publication date interview question tech company lin call isbn publication date material skill collection ebooks video computer manual business management topic student faculty staff access learning book cornell account choose thousand course book video material topic analyst business skill compliance desktop skill engineering government certification learning linkedin offer course highquality video software business skill people experience level sign signon wwwcornelledu domain learn company interview youre role company youre library information understanding company industry overall time area company website youre company press release news section company startup presence pay attention information public minute company sec report firm pitchbook filing company capital navigation menu left news event filing filing industry space industry profile ibisworld frost sullivan technavio industry profile prep question mergent intellect book career laakmann mcdowell call hch isbn publication date book delivery book print book cornell university catalog request book record select cornell tech campus delivery location book bloomberg center security book bloomberg center security desk book access delivery email librarytechcornelledu question business role product manager material business role product manager work strategy operation business role company librarian expertise time information career email librarytechcornelledu company interview networking session company minute lead job chance company time area company website youre company press release news section company startup presence pay attention information public minute company sec report firm pitchbook filing company capital navigation menu left news event filing filing industry space industry profile ibisworld frost sullivan technavio industry profile prep question mergent intellect interview preparation book interview gayle mcdowell jackie bavaro call isbn publication date decode conquer isbn publication date product manager interview lin teng contribution isbn publication date edition book interview question interview question tech company lin call isbn publication date book delivery book print book cornell university catalog request book record select cornell tech campus delivery location book bloomberg center security book bloomberg center security desk book access delivery email librarytechcornelledu question material skill offer course highquality video software business skill people experience level sign signon wwwcornelledu domain learn student faculty staff access learning book cornell account choose thousand course book video material topic analyst business skill compliance desktop skill engineering government certification core material list material career career planning vault vault guide job series career industry information work environment education requirement day life career outlook job tool career company capital company sheet feature factiva download custom company financials growth product news article industry insight report snapshot industry china state report industry performance outlook company chain demand structure barrier entry statistic indepth market strategy report coverage technology space growth chance technavio niche industry specialty chemical material health care energy user report month mergent intellect navigate report industry interest call prep executive insight section question informationals interview company news article factiva aka thousand newspaper business periodical article company official firm finance growth list company core material list company criterion capital platform data company investment firm transaction people financials company company directory list foundation premium directory information institution leadership leadership leadership connect directory directory criterion job title industry location pitchbook youre information startup company user account cornell email address log log sso cornell email address source information firm world country region state keyword zip code code industry code revenue employee book swipe parth detroja neel mehta agashe call isbn publication date career laakmann mcdowell call publication date project manager elizabeth harrin call publication date book guide project manager project manager field book product management catalog consulting material role consulting job material job search tip interview preparation librarian expertise time information career email librarytechcornelledu company interview networking session company minute lead job chance company time area company website youre company press release news section company startup presence pay attention information public minute company sec report firm pitchbook filing company capital navigation menu left news event filing filing industry space industry profile ibisworld frost sullivan technavio industry profile prep question mergent intellect interview preparation companion point book experience question interview guidance interview point casebook marc cosentino office career service harvard university version question point marc cosentino call hdc publication date ivy system section government point competition marc cosentino kara kravetz cupoli jason rife call publication date interview time graph answer book role graph ivy graph framework graph graph interview secret victor cheng call ilr isbn publication date victor mckinsey management consultant insider interview interview paperback edition brad schiller call hdc isbn interview interview interview interview math lin call hfi experience problem answer job seeker interview question market revenue estimate profitability customer lifetime value analysis alexander chernev call isbn approach business job interview book delivery book print book cornell university catalog request book record select cornell tech campus delivery location book bloomberg center security book bloomberg center security desk book access delivery email librarytechcornelledu question material list material career career planning vault vault guide job series career industry information work environment education requirement day life career outlook job tool career company capital company sheet feature factiva download custom company financials growth product news article industry insight report snapshot industry china state report industry performance outlook company chain demand structure barrier entry statistic indepth market strategy report coverage technology space growth chance technavio niche industry specialty chemical material health care energy user report month mergent intellect navigate report industry interest call prep executive insight section question informationals interview company news article factiva aka thousand newspaper business periodical article company official firm finance growth material skill offer course highquality video software business skill people experience level sign signon wwwcornelledu domain learn student faculty staff access learning book cornell account choose thousand course book video material topic</t>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>welcome welcome cornell technology library career job career cornell technology teach find company industry stand interview list potential company want job find company swot report save locate career support startup explore career resource prepare interview company support consultation write library technology cornell respond business top database pitchbook equity venture finance database find real data deal identify analyze comparables investor detail account cornell address log log sso cornell address finance finance major financial platform find data company investment firm finance transaction include finance company company frost sullivan depth strategy report resume technology transportation industrial energy ibisworld ibisworld industry report resume united state industry wide industry canada china report financial cornell student faculty staff account cornell address apps conjunction account article factiva student contact law library wall article cornell student faculty staff account cornell address apps conjunction account industry library technology cornell additional cornell technology library feedback good submit suggestion feedback exploration networking career exploration librarians expertise save find excellent meet career library technology cornell list employer database finance pitchbook guidestar premium mergent intellect different industry report topic overview resource ibisworld frost sullivan mergent report explore career path life article find reliable library resource trade association report show combine linkedin library resource structured expand network job opening network network skeptical useful want know networking job united state library find networking benefit improve networking skills library show navigate linkedin find professional connection relate interest expand job_search article good start harvard business fall special issue week guide job find great job strength weak tie network culture say reach linkedin love network ask introduction harvard business business complete specific article article top browse entire issue issue article fall special issue library technology cornell connect alumnus cuelinks cuelinks cornell university wide network platform connect cornell alumnus peer faculty staff friend cornell explore achieve academic career personal goal core resource short list core library resource recommend career career planning vault vault guide job ideal career industry job environment education requirement typical life career outlook job hunt tool manage career company resume finance company tear sheet feature factiva custom company report summary finance key product article industry insight ibisworld full report snapshot industry canada china united state report include industry performance outlook major company supply chain demand drivers cost structure barrier entry key statistic frost sullivan depth strategy report european global coverage emerge technology include growth technavio technavio emerge niche industry specialty chemical material health care energy report month mergent intellect navigate report industry interest call prep executive insight section useful prepare informationals interview company article factiva nexis university aka lexisnexis contain full text report business periodical able locate article quote company official discuss firm finance classic career book job_search edition steve dalton call isbn article outline systematic approach secure interview potential employer eat keith ferrazzi tahl raz call isbn article guide art networking reveals fundamental principle take build last beneficial relationship eat keith ferrazzi tahl raz call copy isbn article guide art networking reveals fundamental principle take build last beneficial relationship win friend influence dale carnegie call isbn article sell guide interpersonal relationship suggestion deal social business situation book explore engineering library diversity stem resource book delivery know book deliver print book cornell university library catalog book record cornell technology delivery book arrive pick bloomberg security desk book return bloomberg security desk book delivery library technology cornell startup entrepreneurship startup student founder startups specialize require additional resource strategy library connect save encourage schedule consultation member library technology cornell walk library resource find library support happy meet zoom address pitchbook pitchbook pitchbook data resume equity include equity venture finance deal investor fund lps official data national venture finance association pitchbook establish benchmark find real data deal identify analyze comparables investor detail cornell log sso top library resource industry insight frost sullivan depth strategy report european global coverage emerge technology include growth technavio technavio emerge niche industry specialty chemical material health care energy report month mintel report detailed sector include good travel tourism financial industry internet industry retail food drink account cornell address ibisworld full report snapshot industry canada china united state report include industry performance outlook major company supply chain demand drivers cost structure barrier entry key statistic good sense grow company involve mergent intellect navigate report industry interest call prep executive insight section useful prepare informationals interview competitor lseg workspace industry report company include resume expense business segment swot analysis finance powerful screening chart feature list compete firm potential pull finance firm deal venture finance pitchbook explore fund technology topic report include investor fund screen map emerge analysis analyst curated vertical official data national venture finance association cornell address log sso option note downloads cap month whichever less account purge eligible account regain association professional industry association valuable find participant customer discovery interview build sale list competitor list association publish report article topic interest member free smarter tip advance google limit government non profit organization keywords keyword filetype pdf restrict result pdfs surface high quality whitepapers report combine tip understand association non profit researcher think google scholar result cornell library google scholar setting library add cornell university bring article cornell install connect resource technology entrepreneurship cornell list serve join list eship cornell listserv additional resource library congress small business hub guide entrepreneur book explore art start guy kawasaki call ilr library product company division kawasaki show essential launch dream art start guy kawasaki call isbn article revise expand decade guy kawasaki classic bestselling guide launching product idea success lean startup eric ries call isbn startups fail failure preventable lean startup approach adopt globe change company build product launch book delivery know book deliver print book cornell university library catalog book record cornell technology delivery book arrive pick bloomberg security desk book return bloomberg security desk book delivery library technology cornell technical work technical roles library resource seek technical work software data data scientist analyst librarian expertise save find excellent support career library technology cornell library resource short list library resource recommend career career planning vault vault guide job ideal career industry job environment education requirement typical life career outlook job hunt tool manage career company resume finance company tear sheet feature factiva custom company report summary finance key product article industry insight ibisworld full report snapshot industry canada china united state report include industry performance outlook major company supply chain demand drivers cost structure barrier entry key statistic frost sullivan depth strategy report european global coverage emerge technology include growth technavio technavio emerge niche industry specialty chemical material health care energy report month mergent intellect navigate report industry interest call prep executive insight section useful prepare informationals interview company article factiva nexis university aka lexisnexis contain full text report business periodical able locate article quote company official discuss firm finance interview preparation crack cod interview edition gayle laakmann mcdowell call isbn article interview technology company lewis lin call isbn article resource build technical skill collection book video computer manual business topic skillsoft active student faculty staff skillsoft learning book cornell enterprise account training book video resource stay sharp following topic represent analyst business skill compliance desktop skill engineering government skills certification linkedin learning linkedin detailed training high quality instructional video late software creative business skill experience sign single sign cornell domain prompt company interview aim technical work able articulate want job specific company interview library find good understanding company industry overall recommend tackle area company large trade company take press release section good understand want know company small startup presence pay attention share minute trade company take quarterly sec annual report sec held firm take pitchbook include invest find sec filing company finance navigation left event filing sec filing industry industry resume ibisworld frost sullivan technavio industry resume great call prep find mergent intellect book explore crack technology career gayle laakmann mcdowell call isbn article book delivery know book deliver print book cornell university library catalog book record cornell technology delivery book arrive pick bloomberg security desk book return bloomberg security desk book delivery library technology cornell business work include product manager resource business work want product manager job strategy operation sale marketing business work technology company librarian expertise save find excellent support career library technology cornell company interview attend networking session company know little minute prep lead job_opportunity want check company short area company large trade company take press release section good understand want know company small startup presence pay attention share minute trade company take quarterly sec annual report sec held firm take pitchbook include invest find sec filing company finance navigation left event filing sec filing industry industry resume ibisworld frost sullivan technavio industry resume great call prep find mergent intellect interview preparation book crack interview gayle mcdowell jackie bavaro call isbn article decode conquer lewis lin call isbn article product manager interview lewis lin teng contribution call isbn article edition book title interview interview technology company lewis lin call isbn article book delivery know book deliver print book cornell university library catalog book record cornell technology delivery book arrive pick bloomberg security desk book return bloomberg security desk book delivery library technology cornell resource build skill detailed training high quality instructional video late software creative business skill experience sign single sign cornell domain prompt skillsoft active student faculty staff skillsoft learning book cornell enterprise account training book video resource stay sharp following topic represent analyst business skill compliance desktop skill engineering government skills certification core library resource short list library resource recommend career career planning vault vault guide job ideal career industry job environment education requirement typical life career outlook job hunt tool manage career company resume finance company tear sheet feature factiva custom company report summary finance key product article industry insight ibisworld full report snapshot industry canada china united state report include industry performance outlook major company supply chain demand drivers cost structure barrier entry key statistic frost sullivan depth strategy report european global coverage emerge technology include growth technavio technavio emerge niche industry specialty chemical material health care energy report month mergent intellect navigate report industry interest call prep executive insight section useful prepare informationals interview company article factiva nexis university aka lexisnexis contain full text report business periodical able locate article quote company official discuss firm finance important list company core resource list company match criterion specify finance finance major financial platform find data company investment firm finance transaction include finance company company foundation list foundation guidestar premium searchable detailed nonprofit organization leadership connect leadership library leadership connect allow browse single multiple criterion job title industry geographical pitchbook startup company account cornell address log log sso cornell address uniworld authoritative multinational firm operate country state keyword zip code postal code industry code revenue employee book explore swipe unlock parth detroja neel mehta agashe call isbn article crack technology career gayle laakmann mcdowell call isbn article project manager elizabeth harrin call isbn article book accessible guide project manager project manager job field book product catalog consulting resource consult work aim land top consulting job library resource job_search tip interview preparation librarian expertise save find excellent support career library technology cornell company interview attend networking session company know little minute prep lead job_opportunity want check company short area company large trade company take press release section good understand want know company small startup presence pay attention share minute trade company take quarterly sec annual report sec held firm take pitchbook include invest find sec filing company finance navigation left event filing sec filing industry industry resume ibisworld frost sullivan technavio industry resume great call prep find mergent intellect interview preparation interactive interactive companion book practice interview guidance ideal prepare base interview popular casebook marc cosentino office career_services harvard university version interactive johnson library cornell database interactive marc cosentino call isbn article feature ivy include section government nonprofit competition marc cosentino kara kravetz cupoli jason rife call isbn article interview short complex graph analyze extract important apply answer book design understand work graph consult introduce ivy graph framework allow analyze popular graph include mulitple graph allow unfold interview secret victor cheng call ilr isbn article victor cheng former mckinsey consultant reveal proven insider method ace interview embrace interview paperback edition brad schiller call isbn include interview behavioral interviewing interview interview math lewis lin call practice problem answer job seeker quantitative interview include revenue estimate profitability price customer lifetime value master analysis alexander chernev call isbn systematic approach analyze business give master of business administration job interview book delivery know book deliver print book cornell university library catalog book record cornell technology delivery book arrive pick bloomberg security desk book return bloomberg security desk book delivery library technology cornell core library resource short list library resource recommend career career planning vault vault guide job ideal career industry job environment education requirement typical life career outlook job hunt tool manage career company resume finance company tear sheet feature factiva custom company report summary finance key product article industry insight ibisworld full report snapshot industry canada china united state report include industry performance outlook major company supply chain demand drivers cost structure barrier entry key statistic frost sullivan depth strategy report european global coverage emerge technology include growth technavio technavio emerge niche industry specialty chemical material health care energy report month mergent intellect navigate report industry interest call prep executive insight section useful prepare informationals interview company article factiva nexis university aka lexisnexis contain full text report business periodical able locate article quote company official discuss firm finance important resource build skill detailed training high quality instructional video late software creative business skill experience sign single sign cornell domain prompt skillsoft active student faculty staff skillsoft learning book cornell enterprise account training book video resource stay sharp following topic repr</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>康奈尔大学 针对一般学生1.docx</t>
+        </is>
       </c>
       <c r="B37" t="inlineStr">
-        <is>
-          <t>康奈尔大学 针对一般学生1.docx</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
         <is>
           <t>Home
 Navigation
@@ -5628,22 +5520,19 @@
 The ILR Office of Career Services' guide to Internships. Information about job shadowin...</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>home navigation catherwood kheel center kheel center collection school cornell university cul guide cornell career service career service system information job posting oncampus employer event material career site company human resources experience career guide student job cornell university welcome guide job web school managment library guide career contact martin catherwood ives cornell university ithaca socialfacebook pagetwitter subjectseconomics material labor job career compensation benefit data employee institute ebri ebri understanding furtherance employee benefit policy institution employee benefit program policy regard employee benefit content assistance reference desk platform library access software reference workstation ask reference desk assistance cost information movingcom cost living hundred city state tax table crime index city cost insurance premium mortgage recommendation loan amount move custom timeline information calculator move overview bls statistic pay benefit bureau labor statistic site information benefit bls survey employee compensation site salarycom salarycom compensation information individual business manager material career information compensation survey wizard salarycoms compensation tool addition compensation data editorial content compensation advice negotiation tactic news specific compensation marketplace career information network database worker attribute job characteristic replacement dictionary title onet nation source information outlook outlook guide source career information assistance individual decision future work guide year information job description education earnings job prospect condition career service system information job posting oncampus employer event material career site company subscription business insight reference content gale business collection easytouse company fundamental investment report industry ranking market share data company history business source business source text business journal source text business publication coverage area business database text pdf journal harvard business industry country report euromonitor company industry report datamonitor guidestar directory information institution profile mission program financials leader text pdf charity information revenue expense program activity salary board member database content access content premium content assistance reference desk ibisworld ibisworld industry report profile state industry range industry china business report category industry market industry risk rating company industry data report statistic market characteristic segmentation industry condition competitor industry performance analysis outlook mergent mergent intellect submission collection worldwide business information company business intelligence mergents expertise product reference marketplace company database mergent intellect client chance access business data industry news fact figure information ability access industry profile report database report company key data ranking industry classification people location auditor company citation report company industry date database insight conference board insight business managment database report issue business management economics company business trend leadership decision performance excellence governance human resources productivity crm economics material indicator analysis forecast condition sport market analytics sport market analytics news market sporting good association industry source aspect good sport equipment participation demographic fan profile sport finance sponsorship medium marketing firsthand cornell student access service view company industry vault insider information glimpse culture negotiation interview tip diversity profile advice internship survey message board user account cornell email address access web material company registration statement report form edgar link list filing edgar instruction edgar database filing greenbook index market service provider market outlook outlook guide source career information assistance individual decision future work guide year information job description education earnings job prospect condition valuation material industry information guide industry information analysis industry finance alternative finance tool stock market currency stock price company google list competitor graph pricing yahoo finance industry center trade administration trade administration ita competitiveness industry trade investment trade enforcement trade law agreement business environment institution home industry classification system industry classification system naics nakes standard agency business establishment collection analysis publication data business economy naics auspex office management budget omb classification system classification ilr reference office management budget ntis reference census bureau government business type activity card registration department commerce card database franchise agreement report franchisors minnesota department commerce news database material business news source online service news business information source language country company market coverage street journal ftcom ftcom business finance news web site london newspaper time cornell community account cornell email address nexis database source newspaper journal service newsletter company report filing law government document transcript broadcast reference wsj account cornell community member account street online cornell access partnership student assembly cornell university street journal street journal newspaper dow jones news material access world news access world news information perspective source focus viewpoint world issue date coverage varies newspaper newsstream news content archive news source newspaper newswires news journal television radio transcript podcasts website format collection news europe africa asia latin america abiinform abi inform business management database citation abstract text article publication journal trade magazine labor report signature newsletter labor growth print catherwood bloomberg law discrimination verdictsettlement news link news story job verdict settlement material news news material practitioner bloomberg law safety health reporter growth safety york time business news drug unit resigns drug companythis link windownov signal approach oil productionthis link windownov food stamp cut trump strategy link windownov tariff deal playing field chinathis link windownov builder hardship tariff deportationsthis link windownov family split mamdanithis link windownov trump administration food stamp payment day link windownov atkins againthis link windownov work friend link windownov defends rate cutsthis link windownov websitethis link window feed industry industry classification industry classification system industry classification system naics nakes standard agency business establishment collection analysis publication data business economy naics auspex office management budget omb classification system classification ilr reference office management budget ntis reference census bureau government business type activity industry information industry company company industry industry association material industry question naics code industry census website business source business source text business journal source text business publication coverage area business database text pdf journal harvard business industry country report euromonitor company industry report datamonitor abiinform abiinform business management database citation abstract text article publication journal trade magazine area computer economics engineering management communication finance health care material insurance trend law management administration estate taxation transportation ibisworld ibisworld industry report profile state industry range industry china business report category industry market industry risk rating company industry data report statistic market characteristic segmentation industry condition competitor industry performance analysis outlook gale business insight reference content gale business collection easytouse company fundamental investment report industry ranking market share data company history industry industry industry series range discipline series knowledge scholar investment time market firm institution industry statistic industry industry snapshot data bls survey program data industry classification system naics supersector sector industry level bea industry account industry statistic business economy business economy data survey title topic ceic data manager ceic data contains timeseries database offer coverage country asia europe asia africa america eic concept time series data analyst ground agency data institution country ceic data manager access ceic database excel spreadsheet submission timesseries database excel analysis report president council advisor report president report chairman council advisor nation progress text data appendix year database statistic contains indicator country indicator contains indicator purpose comparability country relies submission data authority term indicator contains data drawn website authority basis data tool site database irs tax statistic range table article data describe measure element tax system data policy bureau labor statistic bureau labor statistic bls department labor agency labor market activity condition price change economy mission analyze information decisionmaking data information survey program census bureau industry company business industry catherwood guide point material community industry faq johnson school management library jgsm library guide material industry job opening labor turnover bureau labor statistic bureau labor statistic jolt collect data job job opening quits layoff discharge separation bls statistic industry place statistic job industry job listing academy management academy management association management institution scholar member professor student business school university academic science field practitioner value knowledge creation submission community today span country search job advertisement country newspaper job posting employer post resume feature profile employer job fair career spotlight tip faq category keyword newspaper location company information benefit employee location registration career stop site job listing job seeker posting employer job keyword menu code post job charge service instruction question section job seeker employer site link job market information internet guide resume internet collegegradcom focus entry level position job listing entry level employer job hunter newsletter internship craigslist community classified place job housing good service activity girlfriend advice community information environment choose location hand side indeedcom search engine job job seeker access million job chance thousand website job listing job board newspaper association company career job source index job state category service leader staffing service job listing state location online career network search job resume advice nationjobcom nationjob network network recruitment service inc company moines site job listing company web site job category newsletter job service job update user qualification interest conduit job market staffing industry nettemps firm candidate contract assignment site job search recruiting talent center email newsletter day job day job blog entrylevel job day contributor employer job college medium information job posting browsing topic geography site keyword wall street journal job job posting salary profile issue advice information article business succeeding work user email alert employer feature information career advice faq career newspaper listing access world news access world news information perspective source focus viewpoint world issue date coverage varies newspaper paperboy link newspaper country interest newspaper online choice language user dispute resolution adrhubcom job job posting board adrhubcom werner institute negotiation dispute resolution creighton university diversity job diversity print publication job board career chance college graduate background industry career woman addition job bank resume service site profile material web woman career advice news diversity minority job search engine career chance material job search engine diversity marketplace diversityworkingcom career expo producer industry event diversity marketplace job fair industry channel career growth job search site database link imdiversity diversity recruiting job search site employer profile growth material news site information link material village group concern woman minority latprocom latpro membership institution link member recruiter career service nonmember job listing select business career book executive recruiter directory event trade show information diversity network community career network job seeker employer diverse workforce need customer base diversity career womens career career pride career ability career job site career company diversity workplace workplace diversitycom source diversity talent career web site recruiter caliber diversity candidate search technology insider company award career content combine site material government job career government career government jig online service individual career government public sector jig forum exchange news information interest job sector occupation access thousand government sector job chance candidate fee usa job government site job job information state office personnel management human resources job hrjobscom job website job seeker employer human resources job society material management shrm world association material management member society need human resources career set material chance human resources job web source human resources job job listing employee benefit career administrator analyst manager attorney compliance officer auditor recordkeepers trustee foundation employee benefit plan job site career benefit compensation material job listing job seeker resumé employer email job posting job site service office learning helpful student cornell expertise mobility elm elm offer service wealth information web site site individual institution topic management difference information job seeker link job seeker federation employer outset human resources career deal workload range jurisdiction result array information education advisory support service core area job law employee relation employee reward cornell career service chance guide cornell career service place job search link visa safety funding chance material work job job vacancy institution court institution nation nation relief agency world bank world health institution vacancy country monster focus job search producer monstercom location destination location job material listing job site region country addition job information work university directory work site directory web site part site site job listing work job place chance career service job information search internship link material internship chance union internship delegation internship college university student graduate chance knowledge union institution activity law statistic relation applicant nationality site washington chance link chance bottom ilr career service office career service information job shadowin</t>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>navigation catherwood library kheel kheel digital collection digitalcollections ilr ilr university cornell university library cul ilr library guide relate cornell ilr career_services handshake cornell career_services career relate job internship posting include recruit employer event resource conduct career find company practice cornell career guide student employment cornell university welcome guide ilr specific job_searching sit recommend johnson university managment library excellent guide career photo flickr photo set contact contact ilrref cornell martin catherwood library ives hall cornell university ithaca social facebook pagetwitter subject economics human_resources labor employment career compensation benefit data employee benefit institute ebri ebri promote understanding furtherance employee benefit national policy neutral organization objective employee benefit policy regard employee benefit additional electronic content ilr library ask assistance ilr desk eri platform library restrict load software ilr library workstation ask ilr desk assistance salary cost live move compare cost living international city state tax table crime city interstate move cost insurance premium estimate mortgage recommendation compute loan amount qualify plan move custom timeline interesting include salary calculator plan move overview bls statistic pay benefit bureau labor statistic recommend find authoritative pay benefit bls various survey report employee compensation describe salary salary compensation business manager human resource professional salary compensation survey salary wizard salary compensation tool addition compensation data editorial content compensation advice negotiation tactic specific compensation career net net occupational network comprehensive database worker attribute job characteristic replacement dictionary occupational title dot net nation primary occupational occupational outlook handbook occupational outlook handbook recognize career design valuable assistance decision future job live handbook revise include job description train education earnings job prospect job handshake cornell career_services career relate job internship posting include recruit employer event resource conduct career company subscription databases gale business insight extensive content gale core business collection easy company fundamental investment report industry ranking resume share data company history business complete business complete full text scholarly business article include full text peer business article coverage include subject area relate business database full text pdf top scholarly article include harvard business include industry country report euromonitor company industry report datamonitor guidestar candid searchable detailed nonprofit organization resume resume mission finance full text pdf charity irs file forward revenue expense activity executive salary board member database contain significant free content free content require registration additional premium content ilr library ask assistance ilr desk ibisworld ibisworld industry report resume united state industry wide industry china business report category industry industry risk rating company global industry economic demographic data report key statistic characteristic segmentation industry lead competitor industry performance analysis future outlook mergent intellect mergent intellect flexible base application feature deep collection worldwide business enable company generate insightful business intelligence couple mergent expertise develop product company database mergent intellect exist client unique international business data industry fact figure executive contact ability industry resume proquest historical annual report database corporate annual report company present key data financial fortune ranking industry classification key geographic auditor related company citation report browse company industry cross searchable historical periodical database insight conference board insight business managment searchable database full text report late issue business global economics proprietary nonbiased include company business trend leadership decision performance excellence corporate governance productivity crm economics material include global economic indicator analysis forecast regional national international economic sport analytics sport analytics searchable national sporting good association industry aspect sport good sport equipment participation demographic fan resume sport finance sponsorship broadcast medium marketing firsthand cornell student unique insider company industry firsthand know vault insider include glimpse company corporate culture salary negotiation interview tip find diversity resume career advice internship salary survey message board personal account cornell address free resource edgar sec company foreign domestic require file registration statement periodic report edgar find complete list filing edgar instruction edgar database filing resume present greenbook provider serve occupational outlook handbook occupational outlook handbook recognize career design valuable assistance decision future job live handbook revise include job description train education earnings job prospect job valuation resource industry free guide industry analysis industry google finance alternative yahoo finance tool analyze stock currency compare stock price company google list top competitor custom graph historical pricing yahoo finance industry biz yahoo ind_index international trade administration international trade administration ita strengthen competitiveness industry promote trade investment ensure fair trade enforcement trade law agreement ita job improve global business environment organization compete north american industry classification north american industry classification naics pronounce nakes develop standard federal statistical agency classify business establishment collection analysis article statistical data relate business economy naics develop auspex office budget omb adopt replace old standard industrial classification sic standard industrial classification manual ilr springfield office budget ntis standardized census bureau federal government classify report business activity card franchise registration minnesota department commerce card searchable database include franchise agreement annual report major franchisors maintain minnesota department commerce database resource top business factiva full text international business resume language country company include factiva include full text coverage wall article international business finance associate london base financial report financial cornell community personalized account cornell mail address nexis interdisciplinary full text database include report article wire newsletter company report sec filing law government report transcript broadcast job lexisnexis academic wsj account cornell community member account wall article line cornell possible partnership student assembly cornell university library wall article wall article business focus english language international daily report publish dow jones resource library newsbank full text perspective international distinctive focus diverse viewpoint local regional issue coverage varies report global newsstream recent global content archive stretch include report newswires article television radio transcript blog podcasts digital websites full text format large collection canada europe africa asia latin america australia abi inform abi inform extensive international business database contain bibliographic citation abstract full text article appear professional article academic article trade magazine publish know proquest daily labor report bna bna signature newsletter resume labor print catherwood library bloomberg law late discrimination verdict settlement bloomberg story describe late employment verdict settlement human_resources human_resources practitioner bloomberg law occupational safety health reporter occupational safety business drug unit chief resigns sue drug companythis windownov opec signal cautious approach oil productionthis windownov food stamp cut expose trump strategy shutdown advance agendathis windownov trump tariff deal playing field china windownov builder find hardship trump tariff deportationsthis windownov chinese american family generational split mamdanithis windownov trump administration food stamp payment judge saysthis windownov paul atkins great windownov job friend townthis windownov feed governor defends call big rate cutsthis windownov websitethis feed industry industry classification north american industry classification north american industry classification naics pronounce nakes develop standard federal statistical agency classify business establishment collection analysis article statistical data relate business economy naics develop auspex office budget omb adopt replace old standard industrial classification sic standard industrial classification manual ilr springfield office budget ntis standardized census bureau federal government classify report business activity industry industry trend affect company analyze company particular industry top industry association resource answer industry find sic naics code industry census business complete business complete full text scholarly business article include full text peer business article coverage include subject area relate business database full text pdf top scholarly article include harvard business include industry country report euromonitor company industry report datamonitor abi inform abi inform extensive international business database contain bibliographic citation abstract full text article appear professional article academic article trade magazine publish abi inform resume area account bank computer economics engineering communication finance health care human_resources insurance international trend law administration real estate taxation transportation ibisworld ibisworld industry report resume united state industry wide industry china business report category industry industry risk rating company global industry economic demographic data report key statistic characteristic segmentation industry lead competitor industry performance analysis future outlook gale business insight extensive content gale core business collection easy company fundamental investment report industry ranking resume share data company history industry association industry job repository industry job bring wide academic discipline publish reflect knowledge scholar significant personal investment firm institution concern industry bls statistic industry industry display snapshot national data obtain different bls survey data show base north american industry classification naics supersector sector industry bea industry economic account industry statistic business economy census business economy data census organize survey title topic ceic data manager ceic data contains economic industrial financial data global database unprecedented coverage country asia europe central asia middle east africa america eic macro economic concept data come analyst ground prime national regional statistical agency major industrial data issue organization country resume ceic data manager entire ceic database microsoft excel spreadsheet application retrieve database import excel quick analysis economic report president council economic advisor economic report president annual report write chairman council economic advisor overviews nation economic progress text extensive data appendix previous ilo database statistic contains indicator resume country economies yearly indicator dataset contains standardized indicator purpose great comparability country relies official submission data national authority short term indicator dataset contains monthly semi annual data drawn official national authority update monthly basis additional data tool database replace laborsta irs tax statistic find wide table article data describe measure element tax data useful scholarly policy bureau labor statistic bureau labor statistic bls department labor principal federal agency responsible measure labor activity job price change economy mission collect analyze disseminate essential economic support decision census economic data survey conduct census bureau pertain industry company business industry company industry catherwood library guide abbreviate guide recommended resource ilr community industry faq johnson graduate_school library recommend jgsm library guide best library material depth industry job opening labor turnover survey jolt bureau labor statistic bureau labor statistic jolt collect data total employment job opening hire quits layoff discharge separation bls statistic industry start statistic employment industry job listing category academy academy preeminent professional association organization scholar member professor doctor of philosophy student business_school university academic related social science field practitioner value knowledge creation application found global community today strong span country careerbuilder updated daily employment advertisement country lead report job posting gather employer sit post resume feature include resume featured employer job fair career spotlight tip faq category keyword report geographic company include resume benefit employee hire free registration necessary career stop job listing job seeker allow posting employer job keyword occupational code post job free charge instruction ask section job seeker employer job_market internet guide prepare resume internet collegegrad focus entry position job_searching resume post listing top entry employer job hunter newsletter internship include craigslist craigslist describe local community classified forums find job housing good social activity girlfriend boyfriend advice community free non commercial environment desire right hand side engine job give job seeker free million employment include job listing major job board report association company career internet job large job organize state category temporary staffing job listing united state international monster monster lead global career network job post resume career advice nationjob network network computerized recruitment nationjob inc independent company base moines iowa include job listing company resume target specific employment category newsletter free confidential job scout job update base qualification interest net temp serve conduit job_market staffing industry net temp staffing firm candidate contract assignment include job_search recruiting talent free weekly newsletter job job blog entry job contributor employer job recent university graduate include offline medium job consult posting tag categorize browsing topic geography keyword wall article job update include job posting salary resume issue job hunt advice job article start business succeeding job sign free alert employer feature include career advice faq career report listing newsbank full text perspective international distinctive focus diverse viewpoint local regional issue coverage varies report paperboy report wide country interest report appear choice language dispute resolution job job posting board host adrhub support werner institute negotiation dispute resolution creighton university diversity job diversity employers print digital article job board career target university graduate diverse background industry black collegian career woman addition job bank free resume post corporate resume resource woman career advice diversity job minority job_search engine career resource job_search engine cultural diversity diversityworking national career expo producer industry specific event diversity produce stand locate job fair targeted industry channel diversity career_development job_search searchable database extensive imdiversity diversity recruiting job_search employer resume career_development resource feature extensive focused resource organize village address specific concern african american hispanic american asian american native american woman minority global latpro latpro membership organization act member corporate executive recruiter bilingual spanish portuguese english professional basic free non member include job listing business career book latin american executive recruiter event trade show professional diversity network diverse community trusted professional network pair job seeker employer serious build diverse workforce meet diverse customer base sub network professional diversity military career womens career ihispano black career asian career pride career ability career saludos job specialize join hispanic bilingual professional company diversity workplace workplace diversity workplacediversity diversity talent career corporate executive recruiter want reach experienced high caliber diversity candidate advance technology insider company award win career content combine long term professional resource government job career government career government jig interactive match qualified career government sector jig forum exchange interest job seek employment sector job government sector job_opportunities prospective candidate fee usa job government official job employment united state office personnel job hrjobs hrjobs local employment job seeker employer shrm job society human resource shrm large association devote human resource represent member society serve professional essential comprehensive set resource find job database lead relate job benefitslink job listing employee benefit professional administrator analyst manager attorney compliance officer auditor recordkeepers trustee international foundation employee benefit plan job listings specialized professional benefit compensation human_resources find job listing job seeker post employer sign daily mail job posting international job cornell international office global learning helpful international student cornell expertise labour mobility elm elm fee base wealth free organize organization include topic cultural difference country specific job seeker international job seeker fedee global call federation european employer fedee global outset international professional deal increase workload widen complex jurisdiction result comprehensive array education advisory support address core area employment law employee relation employee reward cornell career_services international guide cornell career_services good start international job_search left include visa safety funding identify resource include job job find job vacancy organization international criminal court international labour organization united nation united nation relief job agency bank health organization vacancy country monster international focus international job_search producer monster allow customize origin destination international job resource detail listing international job organize country addition helpful job_searching job university michigan job extensive break sit specific sit profession specific international job listing internships cool job find seasonal job adventurous include internship cornell career_services job internships conduct design internship resource list internship european union internship delegation internship intend university university student recent graduate acquire considerable knowledge european union institution activity law statistic relation internship applicant nationality european bottom ilr career_services internships ilr office career_services guide internships job shadowin</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>36</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>康奈尔大学 针对一般学生2.docx</t>
+        </is>
       </c>
       <c r="B38" t="inlineStr">
-        <is>
-          <t>康奈尔大学 针对一般学生2.docx</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
         <is>
           <t>Introduction
 Introduction
@@ -5882,22 +5771,19 @@
 Ithaca, NY 14853</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>introduction introduction note education career collection material library willis room reference olin stack print book serial college graduate school preparation career planning test prep location catalog location print version education career title guide guide link education career material material print migration education career material print publication guide career service career education information cornell career service site starting point information reference reference instruction olin library university olin college directory state education college book volume stack annex holding end edition pre edition annex college guide call stack york college entrance examination board incomplete publication education directory washington education publication year reference year olin annex directory institution possession territory agency department education description district fice identification status carnegie classification code accreditation officer petersons college petersons guide year reference year stack directory profile college university twopage description institution description college official information campus environment student activity information directory profile enrollment statistic expense aid housing career service program directory guide university institution education call association university annex stack publication contains information university level degree institution country territory entry length minimum telephone information description location history structure admission requirement degree year enrollment faculty library holding publication directory directory discipline field publication print form material petersons guide reference volume graduate program association college journey residency official guide school admission school pdf download law school bar association guide school stack dental education association education association subscription association geographer association geographer source information geography profession print title guide geography program america aag guide directory geographer volume stack edition annex program directory member year reference subscription year olin stack annex guide program directory member association association school member school association school state commission directory school state awp official guide program edition annex association writer program program database graduate writing program world program listing information type degree size aid awp guide home directory history department institution historian olin stack directory washington association service program year print version reference graduate psychology field olin stack association washington apa year reference directory information graduate program psychology field questionnaire university department state canada list program type degree index school school art reserve association collegiate school architecture washington acsa edition art reserve edition annex guide department sociology call stack association date year reference guide law school edition heinoline information law school cooperation bar association association law school guide school admission school entry print publication pdf petersons guide volume petersons guide subscription library edition stack survey graduate degree program territory country agency description information field accreditation entrance degree requirement expense aid area faculty submission contact description faculty area expertise institution book overview institution book graduate program humanity science book graduate program science book science mathematics book graduate program engineering science book graduate program business education health information law work rating ranking ranking rating college news world report year reference desk year stack online data httpswwwusnewscombestcolleges report editor reporter news world report college university survey college president dean institution university art college college university art college institution methodology ranking report ranking reputation student admission faculty material graduation rate satisfaction directory college university news article college admission cost profile student graduate school graduate school news world report year reference desk year stack print version publication edition online data httpswwwusnewscombestgraduateschools report graduate school program article discipline varies year year kind college insider art college mcwilliams john seery albany state university york press stack reference guide institution collection essay nature art education college college result education trust contains data college university graduate rate group student comparison graduation rate institution college university share characteristic student populationsare college university law information ranking gale olin stack publication citation thousand source institution education admission selectivity test tuition rate publication salary topic quality education insider degree bloomsbury ebook data writing school interview applicant writing student faculty guide writing school submission field catalog insider college york martin stack publication staff news guide story student college twopage description college university guide inclusion quality size school size edition university department education college scorecard data acceptance rate rate rate college university search compare college field cost admission result test prep test prep test prep guide collection ebooks click connect button search box right enter lsat toefl preparation book test print subscription preparation print edition test prep guide guide sample test convenience example print copy test prep title gmat premium olin stack princeton york random house dat stack princeton york penguin random house edition kaplan book stack volume volume science volume biochemistry volume biology volume chemistry volume chemistry volume physic math volume analysis skill aid aid aid call stack college cost aid guide york college board material college board bigfuture description print version college board guide college contains advice range term planning college expense student parent cost aid information college university state scholarship program directory aid woman barbara service press edition reference edition annex source aid program woman undergraduate school program bibliography aid source state source information aid index sponsor topic location cornell program information material service service career career color parachute bolles berkeley ten edition online ebook print volume reference catherwood ilr reference edition olin publication information job market idea career information table test bibliography outlook department labor washington bureau labor statistic print edition olin stack guide detail hundred occupation information education training earnings job outlook nature work table chart index value publication year encyclopedia career growth call reference jeffrey gerard callanan thousand oak publication online index article title list reader subject premier encyclopedia career career choice bibliography reading article encyclopedia career guidance call stack edition volume fergusons volume overview industry volume job industry support occupation source overview industry curriculum vitae call stack jchicago vgm career edition online ebsco ebook curriculum vitae explanation component curriculum vitae stepbystep instruction career concise sketch asset letter letter selection guide resume letter curriculum vitae call cornell catalog reference reference instruction olin library university olin ithaca</t>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>introduction introduction important note education career collection print resource uris library willis room migrate olin olin stack uris stack collections print book serial university graduate_school assessment resume preparation career planning test prep library catalog verify print version education career title list guide guide include education career resource resource unaffected print migration aware education career resource publish print move article add title guide know cornell career_services career education appear daily cornell career_services excellent starting reliable wendy wilcox contact instruction librarian olin uris library cornell university olin ithaca university united state higher_education directories university blue book multiple volume olin library stack library annex cancel holding end edition pre edition hold library annex university handbook call olin library stack university entrance examination board incomplete cease article higher_education higher_education article late shelve olin library shelve olin stack library annex annual institution possession territory accredit regional national professional agency recognize department education description include county congressional district fice identification irs status carnegie classification code accreditation administrative academic officer peterson guide university princeton peterson guide late shelve olin library shelve olin library stack annual contain resume university university depth description institution latter description write university official include environment student activity comprise basic resume consist enrollment statistic expense financial aid housing career_services special international international handbook university institution higher_education call paris international association university library annex olin library stack cease article contains university degree grant institution country territory entry vary length minimum postal telephone description include history administrative structure admission requirement degree academic enrollment faculty library holding article specific specific discipline field article print supersede resource peterson annual guide graduate comprehensive volume graduate aamc association american medical university journey premed residency official guide medical university admission prepare apply medical university free pdf store aamc official guide medical university admission prepare apply medical university aba approve law_schools american bar association official guide dental university call uris library stack american dental education association american dental education association subscription cancel american association geographer american association geographer geography profession print title guide geography america aag handbook geographer print volume shelve olin library stack edition shelve library annex member late shelve olin library subscription cancel early begin shelve olin stack library annex guide member american anthropological association association theological university member university pittsburgh association theological university united state canada commission accredit searchable theological university united state canada awp official guide academic write print edition library annex oversize association writer write awp awp guide academic write free searchable database graduate undergraduate writing academic listing contain degree average cohort financial aid awp guide history department historical organization historian call olin stack searchable american historical association institutional late print version shelve olin library graduate psychology associate field call olin stack american psychological association apa late shelve olin library graduate psychology related field obtain questionnaire send university department organize state canada include include list degree alphabetical university guide architecture university call fine art library permanent reserve association collegiate university architecture acsa late edition shelve fine art library permanent reserve edition library annex guide graduate department sociology call olin library stack american sociological association late shelve olin library official guide aba approved law_school edition heinoline aba approve law_schools entry produce cooperation american bar association association american law_school official guide medical university admission prepare apply medical university aamc entry print article free downloadable pdf peterson annual guide graduate volume princeton peterson guide subscription cancel library edition olin library stack oversize comprehensive annual survey graduate professional degree united state territory foreign country accredit accredit agency brief description contain complete field accreditation entrance degree requirement expense financial aid area faculty application contact supplementary full description include faculty area expertise institution book contain overview institution book graduate humanity social science book graduate biological agricultural science book physical science mathematics book graduate engineering applied science book graduate business education health law social job rating ranking ranking rating america best university report late shelve olin desk early shelve olin library stack limited data usnews best university report editor reporter report rank university university accord survey complete university president dean rat similar institution national university national liberal art university regional university university regional liberal art university specialized institution methodology ranking include report ranking base reputation student admission faculty financial resource graduation rate alumni satisfaction include university university article resume university admission cost resume student best graduate_school best graduate_school report late shelve olin desk early shelve olin library stack oversize print version cease article edition limited data usnews best graduate_schools annual report rank major graduate_school additional article highlight specific discipline varies best kind university insider guide america small liberal art university edit susan mcwilliams john seery albany state university press library stack guide institution thoughtful collection essay nature liberal art education university university result education trust contains comparative institutional data university university graduate rate overall diverse student comparison graduation rate similar institution university university share characteristic serve similar student population university university require law collect educational ranking annual detroit gale olin library stack cease article annotated citation rank institution higher_education accord admission selectivity alumni achievement test score tuition rate faculty article salary topic regard potential quality education insider guide graduate degree creative write bloomsbury academic ebook bring data creative writing university interview mfa applicant creative writing student faculty complete practical guide creative writing university put successful application summary field catalog insider guide university martin olin library stack cease article compiled edit staff yale daily guide inside story student university coast coast subjective narrative description university university dominate guide inclusion base academic quality university emphasize recent edition large university department education university scorecard downloadable data acceptance rate retention rate graduation rate university university compare university field cost admission result test prep test prep best late test prep guide overdrive collection ebooks locate overdrive connect overdrive upper right enter gre lsat toefl find preparation book test library maintain print subscription test preparation recommend purchase late print edition test prep guide mark guide take sample test convenience print copy test prep title crack gmat premium olin library stack oversize princeton random house crack dat uris library stack oversize princeton penguin random house edition kaplan mcat complete book subject uris library stack oversize volume volume behavioral science volume biochemistry volume biology volume chemistry volume organic chemistry volume physic math volume critical analysis reason skill financial aid financial aid financial aid call olin library stack oversize continue university cost financial aid handbook university board replace resource university board bigfuture description print version university board annual guide pay university contains advice long short term planning university expense student parent list cost financial aid university university include state federal scholarship financial aid woman santa barbara press edition olin library edition shelve library annex comprehensive biennial financial aid woman include secondary undergraduate graduate_school include annotated bibliography financial aid state financial aid sponsor topic cornell library material cornell library career plan career plan color parachute bolles nelson berkeley ten speed press edition ebook late print volume shelve olin library catherwood ilr previous edition shelve olin stack annual article job_market break useful idea various career pack useful table chart test bibliography occupational outlook handbook department labor bureau labor statistic annual previous print edition shelve olin stack handbook describe detail job give education training require earnings job outlook nature job photographs table statistical chart enhance value article update encyclopedia career_development call ilr library edit jeffrey gerard callanan oak sage article browseable article title list guide major subject resume premier academic encyclopedia career career choice bibliography reading article encyclopedia career vocational guidance call olin library stack oversize edition volume fergusons volume overview major industry volume resume specific job industry managerial administrative professional clerical support emerge technician job good overview major industry prepare curriculum vitae call olin library stack jchicago vgm career revise edition ebsco ebook pdfs prepare curriculum vitae depth explanation component curriculum vitae instruction condense career concise biographical sketch underscore asset resume resume resume resume resume resume browse selection guide prepare resume resume resume curriculum vitae call cornell library catalog wendy wilcox contact instruction librarian olin uris library cornell university olin ithaca</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>37</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>德克萨斯大学奥斯汀分校   商业学科职业选择.docx</t>
+        </is>
       </c>
       <c r="B39" t="inlineStr">
-        <is>
-          <t>德克萨斯大学奥斯汀分校   商业学科职业选择.docx</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
         <is>
           <t>Research Career Options
 Occupational information
@@ -5931,22 +5817,19 @@
 https://texasrealitycheck.com/</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>career option information onet onet program nation source information project database information hundred descriptor outlook outlook guide source career information assistance individual decision future work guide year job career accelerator internship account address search job internship job career link open window user info section registration information material jobseekers stage career exploration jobapplication user interest occupation profile job internship jobapplication material material content track module store resume cover letter account library job career accelerator reality check labor market career information department texas workforce commission texas reality check calculator lifestyle future planning reality check living expense amount money calculator expense month need occupation youll need occupation calculator occupation expense salary view calculator tour expense cost occupation</t>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>career option occupational net net nation primary occupational central project net database contain standardized job specific descriptor occupational outlook handbook occupational outlook handbook recognize career design valuable assistance decision future job live handbook revise job career accelerator internship account issue address utexas job internship job career unlimited additional section registration update resource job seeker career exploration job application assess job relate interest explore job resume job internship prepare job application material resource personalize content track train module complete store individualize resume resume resume note account learningexpress library job career accelerator interchangeable texas reality check bring labor career department texas workforce commission texas reality check lifestyle calculator able afford lifestyle want difficult predict future early start planning texas reality check show living expense cost amount money earn pay lifestyle calculator walk expense incur month decide spend lifestyle determine minimum salary explore job earn salary job calculator job expense salary support lifestyle quick calculator skip guided tour expense compare cost different job texasrealitycheck</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>38</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>德克萨斯大学奥斯汀分校  护理学职业选择.docx</t>
+        </is>
       </c>
       <c r="B40" t="inlineStr">
-        <is>
-          <t>德克萨斯大学奥斯汀分校  护理学职业选择.docx</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
         <is>
           <t>Nursing——Career Information
 eBooks
@@ -6029,22 +5912,19 @@
 BoardVitals has question banks for NAPLEX, NCLEX RN, and USMLE tests</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>information career handoff healthcare leader transfer generation nurse etiquette nursing career experience nursing profession dissertation nurse technology career concept nursing hrcareer title intelligence emotion impact life career character temperament intelligence color job hunter companion jobhunting book world artist way path creativity people print book nursing concept challenge today perspective success career guide advancement recognition nurse disability issue job retention nursing job leadership nursing experience landscape healthcare man guide men leadership challenge future nursing solution lifestyle nurse transition experience introduction health profession nurse advantage grantwriting nursing career nursing leadership management nurse communication advantage communication skill nursing career nursing profession growth chance growth growth leader year nurse transition novice career nursing hrcareer title career secret personality hour escape website job career link open window user info section registration information material jobseekers stage career exploration jobapplication user interest occupation profile job internship jobapplication material material content track module store resume cover letter account library job career accelerator librarythis link window user info section registration information range online test course ebooks school child adult college admission prep placement test school admission test workplace softskills training preparation licensing material content track module online scoring analysis strength weakness recommendation account library job career accelerator measurement link open window user text information englishlanguage test skill personality aptitude psychology area corresponds part print measurement link window user data thousand institution source access data market opinion institution business institution government agency data topic source percent data statista source online world bank census data source industry marketing trade group data government industry information scope time series data focus statista metadata table information table source information abstract statesthis link window user abstract state compilation statistic focus data table region state city statistic table source data table pdf format section population health nutrition education commerce aid price database result source geography time period breakdown petersons prepthis link window user offer college graduate entrance exam college school information aid source requirement user test experience exam college graduate school military school test preparation service officer service dsst emt firefighter gre law enforcement flight aptitude officer candidate state trooper toefl career career nursing career service series nurse min video essential career july reflection student program career male specie profile men nursing pathway doctor of philosophy dnp piece nursing growth practitioner april career march nursing profession image selfconcept identity discussion certification stepbystep guide boardvitals boardvitals question bank test</t>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>nurse career ebooks career handoff healthcare guide wisdom knowledge transfer generation nurse etiquette advantage professional etiquette advance nursing career lived experience nursing profession dissertation nerdy nurse guide technology advance career concept professional nursing career title emotional intelligence manage emotion positive impact life career understand character temperament intelligence color parachute job hunter workbook companion best selling job hunt book spiritual path high creativity win successful successful print book professional nursing concept challenge mentor today nurse global perspective success accelerate career nurse guide professional advancement recognition nurse disability professional issue job retention land perfect nursing job leadership nursing practice change landscape healthcare man practical guide men nurse leadership challenge future nurse night shift nursing savvy solution healthy lifestyle registered nurse transition practice introduction health profession nurse grant write advantage grantwriting advance nursing career nursing leadership nurse communication advantage business savvy communication skill advance nursing career nursing profession challenge growth nurse nurse transition total novice successful professional career nurse geriatric nursing career title discover perfect career secret personality workweek escape live join rich databases job career unlimited additional section registration update resource job seeker career exploration job application assess job relate interest explore job resume job internship prepare job application material resource personalize content track train module complete store individualize resume resume resume note account learningexpress library job career accelerator interchangeable learningexpress librarythis unlimited additional section registration wide test skill training book elementary university child adult include university admission prep placement test graduate_school admission exams ged test workplace soft skill training preparation occupational licensing resource personalize content track train module complete instant scoring customized analysis strength weakness personalized recommendation note account learningexpress library job career accelerator interchangeable mental measurement yearbookthis update contain full text english language standardize test resume educational skill personality vocational aptitude psychology related area corresponds print mental measurement yearbook statistathis unlimited statista statistical data institution data opinion institution business organization government agency statista include data topic percent total data statista come free bank census data include numerous exclusive include industry marketing trade data relate demographic government industry international scope historical data focus statista metadata table necessary table historical statistical abstract united statesthis unlimited statistical abstract united state compilation social political economic statistic focus national data table resume state city comparative international statistic table identify data table pdf format divide broad section population health nutrition education foreign commerce aid price database browse retrieve result narrow geography period subject breakdown peterson test prepthis unlimited update regularly late university graduate entrance exam university vocational university financial aid requirement prepare specialized test practice exam university graduate_school military trade university include test preparation act american foreign officer civil clep clerical dsst emt firefighter ged gmat gre law enforcement lsat mcat military flight aptitude nclex officer candidate postal sit state trooper toefl career nurse rntobsn career tool nursing career_services article video tell career nurse min video essential build career nurse july nurse reflection second student july innovative promote career nurse male specie resume men nursing pathway doctor of philosophy dnp august essential piece nurse future continue nurse practitioner expert clinician scientist april pursue career nurse march nursing profession image self concept professional identity discussion february continue certification guide boardvitals boardvitals bank naplex nclex usmle test</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>德克萨斯大学奥斯汀分校 （信息科学与图书馆学）.docx</t>
+        </is>
       </c>
       <c r="B41" t="inlineStr">
-        <is>
-          <t>德克萨斯大学奥斯汀分校 （信息科学与图书馆学）.docx</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
         <is>
           <t>Jobs and Internships in Library &amp; Information Science
 Library &amp; Information Science Job &amp; Internship Sites
@@ -6086,22 +5966,19 @@
 #libjobs</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>job internship information science information science job internship residency interest group association college library library association association law library job chance law library country career job internship world archive record management arl job residency internship association library library society internship roster grain job bank career chance country news library publisher book jobber subscription agent gig blog job posting job job information science position knowledge manager state canada job link state job listing type job posting role job zone job company profile post job listing allows job seeker site library congress offer chance job internship fellowship volunteer position job job announcement material society archivist career center resume service job listing job agent career member library association job association public school position experience design job experience career listservs listservs range information group conference announcement job chance question area youre listserv way event field library congress list list library information literacy discussion list part library association ala section loex loex institution instruction information literacy information metadata listserv metadata librarian librarian architect information architect career heritage institution information science federation association institution twitter job libraryjobs lisjobs</t>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>job internship library science library science job internship sit acrl residency interest association university library ala joblist american library association american association law library career include job_opportunities law library country archive gig career job internship archive record arl job residency internship listings association library art library society north american internship roster grain job bank find professional career country include library publisher book jobber subscription agent archive gig updated blog archive related job posting higheredjobs academic job library job library science position include knowledge manager include united state canada international job include state job listing libgig librarian job posting include non traditional librarian work library article job zone enable locate apply job manage company resume post edit job listing allows job seeker apply library congress seek employment internship fellowship volunteer position nasig job serial related job announcement resource society american archivist career resume post job listing job agent keep updated sla career member special library association job texas library association academic university library position experience design job experience professional association library listservs listservs contain specific particular conference announcement job write particular area interested subscribe listserv great familiarize event field library congress listserv list short list generate library congress literacy discussion list american library association ala listservs various section ala loex loex organization devote library instruction literacy metadata librarians listserv listserv intend metadata librarian digital librarian metadata architect architect professional job cultural heritage institution science libjobs moderate ifla international federation library association institution twitter job follow libraryjobs lisjobs libjobs</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>德州农工大学 就业指南.doc</t>
+        </is>
       </c>
       <c r="B42" t="inlineStr">
-        <is>
-          <t>德州农工大学 就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
         <is>
           <t>Career Research Guide
 Explore resources and recommendations from Syracuse University Career Services and Syracuse University Libraries to support your career search efforts
@@ -6206,22 +6083,19 @@
 If you would like to schedule an online meeting, or you simply want to email a question, please do email me.</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>career guide material recommendation syracuse university career service university library career search effort material syracuse university career service career service material undergraduate graduate student university career service website syracuse university career service event material list syracuse university school college career center career support handshake handshake career management tool student alumnus job growth chance syracuse university partner career appointment growth event connect employer interview interview syracuse university career service interview skill platform interview syracuse university career service industry insight growth content event mentor matching chance syracuse university career service student connect community discover job internship state world work authorization type employer record sponsorship linkedin syracuse university career service networking visibility job chance vmock syracuse university career service platform offer resume labor market insight labor market insight syracuse university career service data onet department labor job training administration database career projection estimate occupation industry state county level career service material graduate student university graduate school career exploration planning material career material syracuse university graduate school career growth office master student student material graduate student school career growth platform module master student education career professoriate doctor of philosophy career growth platform stage program student transition career start graduate school career skill value interest confidential tool humanity science student website business management move contemplate question living career keywords career industry question career interest online complement move search option data report career outlook guide information work environment education training qualification job outlook hundred occupation job search site job resume glassdoorcom job search site employee salary interview question thousand company job volunteer search site sector dice job search site tech job database business management entrepreneurship addition material tip syracuse university career service website company industry article database syracuse university library list employer industry trend industry association company interview industry industry trend company outlook ibisworld industry company report industry outlook risk rating report market share business environment profile keyword naics code business insight company financials analysis association market share report business publication search keyword naics code industry industry report industry industry information industry database industry company list company industry code naics code geography criterion company interview information company company news business ratio company person industry content dollar database industry profile demographic consumer lifestyle directory axle reference solution profile state company company business business database consumer criterion income level area interesthobbies directory resident company company database company tip business article information company industry career business article collection index abstract publication business management news report text business source elite coverage hundred business publication economics journal publication text world management marketing journal harvard business database business article article business article industry association industry association industry statistic data industry report industry news industry association member listservs job industry industry information nonmember association library business insight ibisworld industry association yearbook institution association industry association ibisworld industry association material assistance section industry report ibisworld industry association business insight business insight search association directory industry association directory edition business insight instruction keyword business insight industry energy note naics search association directory association result result option publication title encyclopedia association state institution publication date note limiter countryterritory state publication search search edition association directory edition industry association directory business insight instruction publication menu publication search box keyword association search edition industry association directory encyclopedia association institution encyclopedia association institution encyclopedia association state institution list click publication title publication year publication description publication edition publication publication directory publication title encyclopedia association state institution list association association result search term industry energy note naics search association directory limiter countryterritory andor state result industry association yearbook institution yearbook institution institution igos institution business management entrepreneurship meeting question</t>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>career guide explore resource recommendation syracuse university career_services syracuse university library support career effort recommend resource syracuse university career_services career_services resource undergraduate graduate student syracuse university career_services main syracuse university career_services event resource include list syracuse university university university career specialized career support handshake handshake syracuse university centralize career tool student alumnus find internships professional employment professional syracuse university internal external partner schedule career advise appointment career fair professional event connect employer big interview big interview syracuse university career_services strengthen interview skill platform practice virtual person interview firsthand syracuse university career_services include industry insight professional content event mentor matching networking interstride syracuse university career_services student connect international community discover job internship united state job authorization employer historical record sponsorship linkedin linkedin recommend syracuse university career_services professional networking visibility employment vmock vmock syracuse university career_services resume platform offering personalized resume labor insight labor insight syracuse university career_services draw data net department labor employment training administration database show career projection salary estimate job industry national state county career_services resource graduate student syracuse university graduate_school career exploration planning resource career resource recommend syracuse university graduate_school professional career_development office master student doctor of philosophy student postdocs highlighted resource graduate student graduate_school career training platform professional platform feature module master student leverage education build meaningful career professoriate doctor of philosophy career train platform professional platform feature student postdocs transition academic nonacademic career imaginephd start plan graduate_school career assess skill value interest free confidential tool design humanity social science student recommend librarian business entrepreneurship next move contemplate want living career keywords browse career industry answer discover career align interest net complement next move additional option data report career occupational outlook handbook job environment education training qualification salary job outlook job job_search find employment post resume glassdoor job_search include employee salary interview company idealist job volunteer focus non profit sector dice job_search focus technology job database recommend librarian business entrepreneurship addition resource tip syracuse university career_services recommended company industry article database syracuse university library list prospective employer discover industry trend industry association company interview industry industry job trend top company future outlook ibisworld industry company report industry outlook risk rating report share business environment resume searchable keyword naics code business insight include company resume finance swot analysis association share report business article keyword naics code industry discover relevant industry report additional recommend industry databases industry industry database industry tip company targeted list company job industry code naics code geography criterion certain company interview mergent intellect international company company key business ratio searchable company person industry include content dollar database firstresearch industry resume nielsen demographic residential lifestyle data axle solution include resume united state canadian company include small company business business add lifestyles database identify criterion income area interest hobby canadian resident additional recommend company databases company database find additional company tip business article databases find company industry career business article databases abi inform collection abstract article business report job include full text business elite coverage business article economics article include peer article contain full text top marketing article include harvard business additional recommended database business article find article explore additional business article databases find industry association industry association gather industry statistic data industry report publish industry article industry association include member listservs job industry post valuable industry non member association library databases business insight ibisworld databases useful locate industry association yearbook international organization include industry professional association industry association ibisworld ibisworld industry association find additional resource assistance section industry report ibisworld industry association business insight business insight association industry association edition business insight follow instruction enter keyword business insight relevant industry energy note naics code job association association show result filter result option certain article title encyclopedia association regional state local organization article note specific limiter country territory state article describe edition specific association edition specific industry association business insight follow instruction browse article dropdown article enter keyword association multiple edition following industry association list encyclopedia association international organization encyclopedia association national organization encyclopedia association regional state local organization list article title find article article description article publish edition article article article title encyclopedia association regional state local organization bring list association association filter result enter term relevant industry interested energy note naics code job association limiter country territory state filter result industry association yearbook international organization yearbook international organization include intergovernmental organization igos international nongovernmental organization ingos librarian business entrepreneurship schedule meeting want</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>斯坦福大学-通用资源列表.docx</t>
+        </is>
       </c>
       <c r="B43" t="inlineStr">
-        <is>
-          <t>斯坦福大学-通用资源列表.docx</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
         <is>
           <t>Career Research Guide	2
 Research Industries	2
@@ -6608,22 +6482,19 @@
 Older copies are available in the stacks for longer check-out.</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>career guide industry industry report tech report non material stanford gsb company company profile startup firm firm company news create target list company interview cmc material interview book prep job location area cost venture capital startup question material link database industry analysis report statistic industry association material management book book gsb career management book company industry book interview prep book guide guide material student alumnus job hunting career chance industry material job search career chance material material lot information niche segment industry report tech report technology marketing communication career market report analysis issue trend analysis product market contentfeatures stanford subscription stanford faculty staff student stanford access uit idc consumer tech market subscription data product report stanford faculty staff student market report industry material device engineering material industry report industry source material industry report cover industry performance driver industry wizard list industry search hoover downloads option thousand record platform information million company financials swot report strategy industry analyst report datasets gsb alumnus access hoover hoover report country risk rating analysis forecast market information market report country region solution stanford faculty staff student search business market information market report country region stanford faculty staff student material mygsb material student gsb career material mygsb material recommendation biotechnology industry education industry energy industry enterprise technology industry entertainment medium industry health care wellness industry device industry industry estate industry restaurant hospitality tourism ecommerce industry sport industry material telemedicine telehealth industry venture capital equity stanford gsb material day graduation access range material partnership stanford gsb alumnus association gsb database list database gsb alumnus database guide student alumnus alumnus link description alumnus database login gsb alumnus job search material section tip guidance material way company company profile startup company fund investor investment lifecycle venture capital venture capital startup stanford faculty staff student access pitchbook search insight track venture capital venture capital company investor company ipo activity intelligence report institution stanford faculty staff student insight account insight search startup company financials news pevc data stanford gsb faculty staff student msx doctor of philosophy account search firm material company list company financials report hoover downloads option thousand record platform information million company financials swot report strategy industry analyst report datasets gsb alumnus access hoover hoover capital data company statement deal executive board worldwide intelligence module note access analyst report capital connect capital stanford faculty staff student capital access instruction capital search firm subscription recommendation company data family equity venture company startup stanford faculty staff student access instruction public company company industry lookup coverage orbis variable product moody dijk largescale data stanford faculty staff student access instruction business market information market report country region stanford faculty staff student analyst report equity search business news trade article company news business news website subscription link online newspaper magazine stanford wsj washington post economist search business news trade way industry market product news industry medium outlet information create target list company faq detail target list company list company list startup industry prepare interview cmc material cmc interview material search interview prep tool student rocketblocks interview street prep alumnus interview material interview book interview preparation book interview gayle mcdowell jackie bavaro publication date product manager program manager role varies company experience experience translate resume cover letter interview estimation question question question product question question pitch interview secret victor cheng publication date interview secret instruction job interview worldthe interview point marc cosentino publication date cosentino interview interview type question share ivy system confidence copy stack checkout call prep addition company industry material interview analyst report equity analyst reportsequity report overview companyindustry performance outlook estimate iexpert report variety question industry job location area material location fit online map zipcodes tapestry segmentation soccer mom laptop way sense population makeup neighborhood datausa gather data source overview location focus city quality life cost salary city house lifehacker article alan henry cost cost varies world material salary wallet cost calculator cost area variable calculator cnn cost calculator cost area bureau labor statistic consumer price index change time price consumer consumer good service cost living allows cost living city world teleport focus city quality life cost salary venture capital question material recommendation information startup deal fund firm recommendation startup company information source deal funding round data source fund fund performance data source investor manager data source list startup industry link database company fund investor investment lifecycle venture capital venture capital startup stanford faculty staff student access pitchbook search insight track venture capital venture capital company investor company ipo activity intelligence report institution stanford faculty staff student insight account insight search startup company financials news pevc data stanford gsb faculty staff student msx doctor of philosophy account search data information asset market data cover capital hedge fund fund fund manager investor information marketwide benchmark access subscription recommendation company data family equity venture company startup stanford faculty staff student access instruction terminal london stock exchange group reuters refinitiv access pricing data stock bond company fundamental estimate data deal table analyst report eikon stanford faculty staff student access information video tutorial analystequity report vcpe industry analysis report statistic group report statistic venture capital landscape industry association section website material publication material member example venture capital association nvca edition print copy stanford europe report statistic venture capital activity investment council information investment trend performance investment equity return pension fund industry association material place report statistic venture capital industry venture capital equity country attractiveness index index business school university pitchbook pitchbook access report analysis vcpe industry panel center note access insight insight access report analysis vcpe industry venture capital funding industry keyword search search box brief intelligence report subscription statista statistic topic industry market source tab chart data consumer insight consumer behavior brand preference data career management book book gsb collection careermanagement book print ground floor gsb library online audiobooks selection book searchworks career management book guide career harvard business publication date hbr guide career self skill industry implication change youre role job career path role hbr guide growth harvard business staff publication date matter career guide skill feedback goal time play strength challenge life bill burnett evans publication date life walk reader satisfying life challenge way designer iteration move matter blake publication date book answer question whats youve plateau job youre role job company industry thing career success career playbook james publication date survey thousand graduate career hundred interview world business leader career playbook graduate career advice hbr guide balance harvard business peter bregman friedman grace saunders publication date hbr guide balance priority expectation time budget plansand backup plan tradeoff selfcare identity christopher gobet publication date book nature expertise individual transition course career business sport music role motivation flexibility intelligence thinking intelligence identity change adapts career transition concept course career thomas lys ebook version publication date ebook people time option ebook version people time audiobook copy print book availability world work russell beck publication date book megatrends world today series lens business individual range market world examination future work challenge charge career harvard business isbn publication date part woman work series collection hbr article woman workplace rule secret career right isbn publication date identity strategy career herminia ibarra isbn publication date intelligence series power impact selfawareness confidence leadership presence people meaning passion leadership joel peterson publication date impact initiative approach fromthetrenches executive mentor entrepreneur leadership expert joel peterson bos harry dent publication date harry dent author entrepreneur trend forecaster business way clark publication date blueprint independence insight advice brand expertise reach impact online superstar kahan publication date superstar insider guidance career tech startup revolution entrepreneur voice career staff isbn publication date book entrepreneur career expert life veil rank company side gig business success company industry book interview guide investment banking paul pignataro publication date statement valuation merger acquisition buyout discussion answer question understanding core analysis core model way rasiel publication date technique world business consultancy experience business role tactic consultant project book businessmen woman technique strategy basis business dna amazon apple facebook google scott galloway publication date galloway strategy need speed scope match investment bank fund equity david stowell publication date investment bank fund equity firm life stowells introduction way reshaped business plan wake meltdown book reveals function compensation system role wealth creation risk management epic battle investor fund influence fire scott mautz isbn publication date fire malaise dial motivation youre wrestling fear disconnectedness boredom lack outlet issue insight story checklist force inspiration audiobooks memoir creator nike phil publication date founder ceo phil share story company day startup evolution world brand publication date leadership status power people leader people people idea potential book brené strategy example couragebuilding program scott galloway publication date amazon apple facebook google company planet book galloway strategy need sheryl sandberg publication date sheryl sandberg woman change life effect scale experience world business answer problem woman workplace life bill burnett evans publication date life walk reader satisfying life challenge way designer iteration rescue work jon acuff publication date day ice cream restock shelf chance element career relationship skill character degree time way career saving difference voss tahl raz publication date hostage negotiator fbi approach boardroom home interview book interview preparation book interview gayle mcdowell jackie bavaro publication date product manager program manager role varies company experience experience translate resume cover letter interview estimation question question question product question question pitch interview secret victor cheng publication date interview secret instruction job interview worldthe interview point marc cosentino publication date cosentino interview interview type question share ivy system confidence copy stack checkout</t>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>career guide industry introduction industry report technology focus report global regional non report additional resource stanford gsb company company finance resume startup large firm firm non company target list company prepare interview cmc resource interview prep book call prep job area overviews cost live startup ask top resource faqs quick database industry analysis report statistic industry association additional resource career book career book gsb library ebooks career book entrepreneurship company industry specific book audiobooks interview prep book career guide guide list library resource gsb student alumnus job hunting explore career industry introduction following resource job_search career resource relevant resource particular find lot niche segment ask industry report technology focus gartner report relevant technology marketing communication professional include report depth analysis issue trend analysis product worldwide content feature include stanford subscription stanford faculty staff student stanford gartner uit uhr idc global telecom technology report subscription include data product report stanford faculty staff student bcc global report industry include material medical device engineering report popular resource industry report industry guide additional resource ibisworld global china industry report resume industry performance driver include industry wizard list industry ibisworld hoover limit downloads option record platform million company worldwide include finance swot report strategy industry analyst report historical datasets stanford gsb alumnus hoover hoover global regional non report bmi country risk rating macroeconomic analysis forecast global emerge report country worldwide fitch solution stanford faculty staff student bmi emis next business global emerge report country worldwide stanford faculty staff student additional resource cmc mygsb career resource student find additional gsb career resource mygsb industry specific resource recommendation biotechnology industry education industry energy industry enterprise technology industry entertainment medium industry health care wellness industry medical device industry pharmaceutical industry real estate industry restaurant hospitality tourism retail ecommerce industry sport industry resource telemedicine telehealth industry venture finance equity stanford gsb alumni library resource alumni start graduation able remote resource partnership stanford gsb alumnus association gsb alumni library database list database stanford gsb alumnus database guide student alumnus alumnus description take alumnus database gsb job_search resource section find tools tip guidance resource company company finance resume startup pitchbook company deal fund investor investment lifecycle worldwide great venture finance startup stanford faculty staff student pitchbook pitchbook insight track venture finance back company investor company ipo activity worldwide expert intelligence report academic institution stanford faculty staff student insight account insight tracxn global startup company resume finance data stanford gsb faculty staff full student master of business administration msx doctor of philosophy tracxn account tracxn large firm follow popular resource company list depth company finance report hoover limit downloads option record platform million company worldwide include finance swot report strategy industry analyst report historical datasets stanford gsb alumnus hoover hoover finance data company financial statement deal executive board worldwide contain snl intelligence module global note analyst report finance pro connect legacy finance stanford faculty staff student academic finance pro instruction capiq pro add finance firm privco subscription end november alternative recommendation company data include family equity venture back company startup stanford faculty staff student privco instruction non orbis global company resume small company industry ups broad coverage orbis tend include variable regional product moody bureau van dijk large scale data orbis historical stanford faculty staff student orbis instruction emis next business global emerge report country worldwide stanford faculty staff student analyst report equity business trade article company business subscription quick popular report magazine stanford include wsj post economist business trade article great industry product scour industry medium outlet target list company faq detail target list company list company list startup industry prepare interview cmc resource cmc interview prep resource mygsb interview prep tool gsb student include rocketblocks exponent interview prep wall prep gsb alumnus interview resource interview prep book popular interview preparation book crack interview gayle mcdowell jackie bavaro article product manager manager work varies company experience exist experience translate great resume resume resume master interview estimation behavioral product technical super important pitch interview secret victor cheng article interview secret discover instruction dominate consider complex difficult intimidating corporate job interview infamous interview marc cosentino article cosentino demystify consult interview take typical interview explore various share acclaim ivy give confidence answer sophisticated old copy stack long check call prep addition company industry following resource helpful prepare interview analyst report equity analyst report equity report overview company industry performance expert outlook estimate ibisworld iexpert report call prep organize industry job area overviews following resource determine potential good fit tapestry segmentation map allow zip code associated tapestry segmentation soccer mom laptop lattes quick sense overall population makeup specific neighborhood datausa gather various data quick visual overview geographic teleport global focus compare city quality life cost live salary city leave house lifehacker article alan henry publish relevant cost live cost live varies resource compare salary nerd wallet cost live calculator allow compare cost live metro area variable cnn calculator cnn cost live calculator allow compare cost live metro area bureau labor statistic price average change price pay urban good salaryexpert cost living allows compare cost living major city teleport global focus compare city quality life cost live salary ask top resource top recommendation startup deal fund firm list ask specific recommendation startup back company deal funding round data fund fund performance data investor fund manager data list startup industry quick database pitchbook company deal fund investor investment lifecycle worldwide great venture finance startup stanford faculty staff student pitchbook pitchbook insight track venture finance back company investor company ipo activity worldwide expert intelligence report academic institution stanford faculty staff student insight account insight tracxn global startup company resume finance data stanford gsb faculty staff full student master of business administration msx doctor of philosophy tracxn account tracxn preqin financial data alternative asset data resume finance hedge fund include fund fund manager investor deal wide benchmark preqin privco subscription end november alternative recommendation company data include family equity venture back company startup stanford faculty staff student privco instruction lseg workspace financial terminal london stock exchange thomson reuters refinitiv global pricing data stock bond company fundamentals estimate esg data deal league table analyst report replaced eikon stanford faculty staff student lseg workspace video tutorial analyst equity report industry analysis report statistic report gather statistic landscape industry association section title resource article data material restrict member national venture finance association nvca yearbook late edition pdf format print copy stanford libraries europe report statistic venture finance activity europe american investment council investment trend fund performance sector specific investment equity return pension fund find industry association additional resource report statistic industry include global venture finance equity country attractiveness annual iese business_school university navarra pitchbook pitchbook find report analysis industry left panel library note content insight insight find report analysis industry focus funding industry keyword main brief note expert intelligence report include subscription statista statistic topic industry chart track data insights insight country behavior brand preference data career book career book gsb library curated collection career relate book print ground gsb library ebooks audiobooks large selection book searchworks career book hbr guide change career harvard business article hbr guide change career imagine professional self identify skill possess transfer industry financial implication change consider try work endanger job explain winding career path pitch work hbr guide professional growth harvard business staff article matter career guide assess skill acquire elicit feedback set meaningful achievable goal play strength identify next challenge design life bill burnett dave evans article design life walk build satisfying meaningful life approach challenge designer experimentation wayfinding prototyping constant iteration pivot move matter next jenny blake article book answer next hit plateau perfect job consider take work job want move company industry remain clear career success depend pivot plan career playbook james citrin article base depth survey graduate young professional interview top business nonprofit career playbook recent graduate aspire young professional actionable advice excel hbr guide job life balance harvard business peter bregman daisy wademan dowling stewart friedman elizabeth grace saunders article hbr guide job life balance evaluate adjust priority manage expectation set spend budget plan backup plan understand trade offs prioritize care discover job transition identity christopher fernand gobet article book examine nature expertise enable repeated successful transition training career focus business sport music examine work motivation cognitive flexibility personal intelligence generative thinking contextual intelligence show identity change adapts career transition self concept evolve training career want margaret neale thomas lys ebook version article ebook option ebook version audiobook copy check print book availability job russell beck article book consider megatrends play today lens explain business future proof illustrate broad apply smart examination future job overcome challenge take charge career harvard business isbn article woman job collection hbr article woman workplace unspoken rule secret start career right gorick isbn article job identity unconventional strategy reinvent career herminia ibarra isbn article hbr emotional intelligence include ebooks power impact self awareness mindful listen confidence leadership presence deal difficult purpose meaning passion entrepreneurship entrepreneurial leadership joel peterson article lasting impact launch initiative inspire champion innovative approach trench guide trusted executive mentor entrepreneur leadership expert joel peterson bos harry dent article harry dent bestselling author entrepreneur trend forecaster encourage start business best suit entrepreneurial dorie clark article entrepreneurial dorie clark blueprint professional independence insight advice build brand monetize expertise extend reach impact startup superstar steven kahan isbn article startup superstar expert insider guidance ignite career join technology startup revolution entrepreneur voice career inc staff isbn article book successful entrepreneur career expert life veil take rise rank company build successful side gig set business success company industry specific book technical interview guide investment banking paul pignataro article resume financial statement valuation merger acquisition leveraged buyout discussion answer common technical refresh understanding core technical analysis core model analyse mckinsey ethan rasiel article discover translate technique lead business consultancy meaningful practice employ business work highlight tactic mckinsey consultant project book inform businessmen woman technique strategy daily basis successful business roles hidden dna amazon apple facebook google scott galloway article galloway deconstruct strategy show manipulate fundamental emotional drive speed scope match investment bank hedge fund equity david stowell article investment bank hedge fund equity firm come life david stowell introduction challenge sustain capture reshaped business plan wake global meltdown book reveals key function compensation unique work wealth creation risk epic battle investor fund corporate influence find fire scott mautz isbn article find fire discover shake malaise dial motivation wrestle fear disconnectedness boredom lack creative outlet overwhelm issue find applicable insight exercise inspire story checklist force drain inspiration audiobooks shoe dog memoir creator nike phil knight article founder ceo phil knight share inside story company early intrepid start evolution iconic profitable brand dare lead brown article leadership status power hold accountable recognize potential idea develop potential book actionable strategy real base courage build scott galloway article amazon apple facebook google influential company planet book galloway deconstruct strategy explain manipulate fundamental emotional lean sheryl sandberg article sheryl sandberg woman small change life effect change universal scale draw experience job successful business academic find practical answer problem face woman workplace design life bill burnett dave evans article design life walk build satisfying meaningful life approach challenge designer experimentation wayfinding prototyping constant iteration rescue monday reinvent job stick jon acuff article start pay scoop ice cream restock shelf chance develop element great career common relationship skill character hustle degree amplify apply career saving account amazon split difference chris voss tahl raz article former international hostage negotiator fbi field test approach high stake negotiation boardroom interview prep book popular interview preparation book crack interview gayle mcdowell jackie bavaro article product manager manager work varies company experience exist experience translate great resume resume resume master interview estimation behavioral product technical super important pitch interview secret victor cheng article interview secret discover instruction dominate consider complex difficult intimidating corporate job interview infamous interview marc cosentino article cosentino demystify consult interview take typical interview explore various share acclaim ivy give confidence answer sophisticated old copy stack long check</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>斯坦福大学-音乐职业资源.docx</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
-        <is>
-          <t>斯坦福大学-音乐职业资源.docx</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
         <is>
           <t>Music careers, internships, graduate programs	1
 Getting Started	1
@@ -6808,22 +6679,19 @@
 The Enterprising Musician's Legal Toolkit i...</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>music career graduate program graduate program music competition internship grant music business book music business career career music business entrepreneur matter matter music career graduate program guide source music career graduate program music business area interest place america listing variety chance growth tab job listing contest chance scholarship grant graduate program music directory music faculty college university music degree program type degree location graduate program music nichecom society composer guidance school composition competition performing art yearbook information competition description contact information eligibility volume europe north america pacific rest world print volume music reference room call print edition gramophone magazine list competition year music library internship america company institution opera internship jazz internship sony music warner music group grant endowment art grant foundation center california art council music business book music business business song scott brickell robert noland told publication date youre artist college grad scott business song guide world music industry year experience manager artist band brickell detail artist manager promotor booking agent share industry secret formula song tip show matter goalwhether thats stage microphone scene showsthe business song industry insider terminology goal path career journey music business exciting career music industry scott brickells guide screen scott hallgren editor isbn publication date book collection essay interview composer film television video game business side lack career growth business responsibility composer music business guide career guide baskerville baskerville call item reference call status isbn publication date edition powerhouse tradition uptodate guide music industry diversity reader music business career baskerville tim baskervilles goto source regardless specialty music field create bruenger isbn publication date create cycle experience musician career entrepreneur music industry building concept book money music david bruenger reader framework relationship artist audience producer consumer method creationproductionreception creationconsumptioncompensation chapter perspective structure listener experience interact music artist taylor swift music spotify rise artist site patreon bruenger realworld example industry experience encounter music create produce consume tool reader agile knowledge music industry graph table reading question discussion illustrate concept material instructor student list reading music business essential mark cabaniss mike curb foreword publication date today music business music availability consumption force offer chance desire music business essential guide career musician business student journey nut bolt knowledge wisdom industry music industry mark cabanisss concise approach reveals principle reader career music band dynamic promotion record label revenue stream music machine talent tax music business essential introduction guide reference time college student school student career music lesson road pasternack michael item stack status isbn publication date success language music language business examination influence impact creativity improvisation collaboration institution interview business people musician thoughtleader todd pasternack reader throughlessons road business leader realworld story road today business leader idea institution product solution team dot way interview avery scala health bass player boysetsfire jimmy chamberlin ceo strategy drummer smashing genauer cmo magisto guitar vocal assembly dust anurag gulati facebook studio owner cat insurance guitar vocal michael bass clarinet margolin armada vocalist sam moore mark band glenn rosenstein group record label president record producer guitarist guitar vocal moe music business weissman isbn publication date today music industry career music need aspect business control career music business student concise overview music industry realworld experience wealth career profile edition growth advent streaming shift diy side reader opinion issue music business introduction talent living music business herstand derek sivers item stack status publication date decade industry upheaval turmoil music industry diy business guide success water music business tutorial negotiating contract play licensing musicbut manifesto musician path indie rock richard turgeon isbn publication date indie rock concise allinone primer musician fundamental band basic year book magazine part band topic band people experience part cover preproduction consideration basic timeless fundamental technique mixing part iii cover fan base design press kit sharing music video youre primer music level indie rock book photo qas birdmonster cdbaby founder derek sivers vanderslice karate mark kozelek art music publishing helen gammon publication date career area music art music publishing inspiration hand perspective side highreward music business prepare career music publishing complex part music business author gammon role publisher right income stream contract income area business industry income stream business model website interview podcasts music business gammon doesnt music publishing level music publishing book composer aint body rufus chaka khan song youre music publisher book mass information idea opinion interview music biz thought business plenty anecdote bellnbsp manager yardbrids george michael marc bolan idiot music business michael miller isbn publication date idiot guider music businessis musician business music businesspeople music industry author miller business topic wealth job chance music industry business perspective negotiating contract song royalty promotion strategy cover industry career management concert promotion music production radio feature information frontier music savvy musician cutler call publication date youre music marketplace musician chance aspect life career living difference concept strategy vignette musician career book element misunderstood musician control career brand capitalize internet tool network money dream savvy musician material performer composer educator student administrator industry employee future demo delivery rus hepworthsawyer editor isbn publication date demo delivery production discusses stage music production start creation growth composition song production book mixing mastering stage marketing distribution book technique music start information signpost source information end chapter demo delivery map musician producer engineer music career music idea studio demo hand market check book httpdemodeliverycom business music james walker call isbn publication date reference book business advice area music industry record deal label publishing music marketing information today musician example quote anecdote dozen artist executive business music author james walker entertainment lawyer client jamie foxx dmx year expertise litigation business property law business music price musician career career music business career music library misti shaw editor susannah cleveland editor isbn publication date reflection art management paola isbn publication date singersongwriter guide justin williams editor williams editor call isbn publication date singersongwriter music everpresent figure music singersongwriter guide material student songwriter musician fan scholar entertainment larry wacholtz isbn publication date entertainment insider career entertainment music industry thorough exploration state industry emphasis trend streaming advice career artist technician industry executive book variety topic entertainment music industry business model property right destruction return hustle sheinkop isbn publication date movie way life series finale television show heart video game perception reality youre consumer question music film show game role response experience fact music medium purpose audience level access music strategy success television film brand video game expectation content animation celebrity cameo consumer way audience music experience song partnership music band bond product experience music way word return hustle music marketing industry insider diverse audio touchpoints key industry marketer storyteller advertiser music audience customer journey consumer brand advocate hustle reader blueprint music strategy career level industry consumer content relationship brand end credit interview return reader playbook marketing power music business result business brain jennifer rosenfeld julia torgovitskaya call publication date artist businessperson time musician age world interconnectivity answer jennifer rosenfeld julia torgovitskaya founder icadenza cadenza artist share lesson music career coaching business talent agency business brain artist lot misconception business side art growth sacrifice contract way musician artist businessperson jennifer julia essential survival today music world career guidance wisdom business brain music career dedication jennifer julia music business compassionate book mustread artist management music business paul allen isbn publication date evolution music business influence record artist manager center artist artist manager abreast music industry artist management career industry insight guidance management tool strategy career artist management music tool artist manager analysis dozen lesson contract example author paul allen artist career followup edition chapter entrepreneurship information artist management enterprise business coverage risk challenge money management chapter section medium web promotion material book wwwartistmanagementonlinecom music business richard weissman call item stack status isbn publication date music business student overview music business music business text offer approach question today music student living music business basic part text section deal fundamental industry music publishing agent manager radio television union internet technology music market half text ground career path artist industry growth need skill way individual career industry artist aaron isbn publication date artist lesson creatives dworkin offer guide fulfillment accomplishment mozart creatives lesson matter medium dworkin book actor jeff daniel bill jones grammy wynton marsalis pulitzer winner miranda story twelve individual lesson love loss despair perseverance artistentrepreneur takeaway book peer patron sponsor diversity focus work student artist search tool career reinvention artist offer kind muse isbn publication date muse career music principle entrepreneurship music student career educator perspective understanding complexand landscape music career author career journey narrative view career possibility reader tool view possiblecareer path skill value stcentury marketplace goal entrepreneurship endeavor reader artisticintegrity muse explains approach career music music career growth muse reader imagination tool career fulfilling art onstage studio jennifer hamady call publication date book singer talent technique song audience skill training technology stage studio people matter voice money performing technology youre ride singer business figure studio headphone stage monitor need producer engineer singer art stage studio book issue easytoread style discussion evolution technology voice culture root cause performance issue singer performer producer engineer book origin field tool trade clearer communicate savvy music teacher cutler call publication date music career savvy music teacher dollarfordollar blueprint income music teacher impact income material reveals lesson cutler guidance reader thriving studio curriculum innovation strategy aspect business art powerhouse marketing time management skill literacy independence career outlook mustread music student studio owner career instructor savvy music teacher advice language reallife experience teacherentrepreneurs piano success gordon isbn publication date pianist career face barrage question choice challenge book stewart gordon way reader secure career ground decade gordon pianist detail college year career livelihood guide career gordon wisdom decade body information pianist goal advice work motivation security aspiration reality inspiration institution gordon blueprint dream achievement point example life musician book matter keyboard technique reading skill repertoire demand musician life volume material pianist parent matter guitar program bill isbn publication date guitar program guide music educator task music program interest guitar mariachi rock band music technology music educator music author bill swick book educator music program ground floor year experience music educator guitar book willassist music educator classroom management scheduling structure institution fund festival travel subject guitar classroom principle music educator program standsout school district state attracting student parent educator administrator money music bruenger isbn publication date money music offer entrepreneurship music business classroom workplace reader principle context understanding thing work music business concept variety situation reader capacity problem music money culture marketplace matter enterprising musician toolkit williams isbn publication date enterprising musician toolkit</t>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>music career internships graduate start start graduate music competition internship grant music_business book music_business career career music_business entrepreneur teach legal matter teach legal matter music career internships graduate guide gather music career internships graduate music_business related area interest start start good start musical america worldwide listing professional growth take job listing contest award educational include scholarship grant graduate music music faculty university university music degree degree graduate music niche list society composer guidance grad university composition competition performing art yearbook list competition worldwide include description contact eligibility prize volume europe asia north america pacific aka rest print volume music library room call print edition gramophone magazine issue january list competition come find music library internship musical america worldwide mention specific company organization metropolitan opera internship jazz internship spotify sirius sony music warner music grant national endowment art grant foundation art council music_business book music_business business song scott brickell robert noland told isbn article aspiring university grad seasoned professional scott brickell business song handbook navigate confusing unapproachable music_industry draw experience manager numerous record breaking band scott brickell explain nitty gritty detail take manager promotor booking agent share industry secret formula successful song give invaluable tip put successful show tour matter goal microphone scene promote show business song understand industry start insider terminology identify goal set clear path future career start journey music_business break exciting fulfil career music_industry scott brickell guide show compose screen scott hallgren editor isbn article book collection essay write interview job composer film television video game explore business side compose address lack understand career_development business responsibility relate composer music_business handbook career guide david baskerville timothy baskerville call item call status isbn article twelfth edition powerhouse best sell text maintain tradition comprehensive guide music_industry diversity music_business seasoned professional find david baskerville tim baskerville handbook regardless specialty music field produce consume david bruenger isbn article produce consume explore cycle musical experience musician professional bud entrepreneur break music_industry concept previous book money music david bruenger basic framework understand relationship audience producer examine method underlying creation production reception creation consumption compensation chapter different perspective structure lead listener discover experience interact music musical taylor swift refusal allow music stream spotify rise support patreon bruenger relevant real industry practice shape encounter music produce consume critical tool give agile knowledge necessary adapt change music_industry graphs table list additional reading discussion illustrate key concept resource instructor student include sample syllabi list expanded reading music_business essential mark cabaniss mike curb foreword isbn article today music_business challenge music availability consumption powerful force unprecedented desire succeed music_business essential guide aspire professional take musician begin business student journey full vital nut bolt knowledge practical wisdom veteran industry professional dynamic music_industry change mark cabaniss concise encouraging realistic approach reveals unchanging principle guide successful fulfil career music band dynamic tour songwriting publish brand promotion record label revenue stream cabaniss resume entire music machine talent tax return music_business essential easy introduction prove invaluable handbook ideal university student high university student interested career music lesson road todd pasternack michael lowenstern call item stack call status isbn article tough measure success exist language music meet language business unorthodox examination influence impact creativity improvisation collaboration organization interview successful business professional musician musician technology think todd pasternack take throughlessons road musicians business real story road today business find fresh idea bring organization innovative product solution build strong connect dot unexpected valuable feature interview rob avery scala digitas health bass player boysetsfire jimmy chamberlin ceo blue strategy drummer smashing pumpkins reid genauer cmo magisto guitar vocal assembly dust anurag gulati uber facebook studio owner cat progressive insurance guitar vocal job michael lowenstern bass clarinet naomi margolin armada global vocalist sam moore mark newman band glenn rosenstein wealthpoint financial record label president record producer derek richmond prettybird guitarist schnier guitar vocal moe understand music_business dick weissman isbn article today move music_industry take build life long career job music aware aspect business take control career understand music_business student concise comprehensive overview evolve music_industry root real experience anchor wealth career resume second edition update include important contemporary include advent streaming shift diy paradigm side feature understand differ opinion key issue readable understand music_business perfect introduction seek understand musical talent connect living music_business ari herstand derek sivers call item stack call status isbn article last decade industry upheaval turmoil music_industry democratic diy business guide success water tell survive ari music_business compile tutorial accomplish specific task rout tour negotiating contract pay streamed play license music manifesto encourage musician pave path indie rock richard turgeon isbn article indie rock clear concise primer begin mid musician essential fundamental run record promote band basic take collate specialized technical book magazine write real independent musician run band resume topic relevant run band practice songwriting record resume pre production consideration gear basic timeless fundamental technique record mixing master iii promote resume know establish grow fan base include graphic design press kit sharing sell music play video start degree primer take music next indie rock book resume feature photo birdmonster cdbaby founder derek sivers juliana hatfield john vanderslice karate mark kozelek art music publishing helen gammon isbn article want pursue career succeed lucrative area music publish art music publishing real inspiration tangible hand perspective exciting side high risk high reward music_business prepare career music publishing understand complex profitable music_business author gammon walk know understand work publisher copyright manage right income stream contract income generate area business explore industry income stream business model develop support include video interview podcasts music_business legend helen gammon know music publishing worth know want take next music publishing book know refer david hawk composer aint body rufus chaka khan covered song alreadynbsp music publisher book give mass useful fresh idea legal opinion video interview music biz legends provocative thought business head plenty good anecdote simon napier bellnbsp manager yardbrids george michael wham marc bolan japan complete idiot guide music_business michael miller isbn article complete idiot guide music_businessis write musician business music businesspeople enter music_industry author michael miller resume key business topic reveal wealth job_opportunities music_industry business perspective resume find agent negotiating contract publish song collect royalty promotion strategy resume nonmusician industry career concert promotion music production radio feature essential frontier electronic music savvy musician david cutler call isbn article talented trained passionate music professional flood outstanding musician force compete shrinking traditional savvy musician balance override aspect professional musical life build career earn living difference fill articulate concept detailed strategy vignette actual musician job meaningful prosperous career book examine critical element overlook misunderstood musician take control career discover build recognizable brand capitalize technology internet tool record paradigm expand network raise money fund dream savvy musician invaluable resource performer composer educator student administrator industry employee interested thriving musical future demo delivery rus hepworth sawyer editor isbn article demo delivery production discusses typical music production start finish begin creation composition song production book trace record mixing mastering marketing distribution book want pro technique involve music start finish pack essential include signpost end chapter demo delivery map musician semi pro aspire producer music professional interested music idea studio demo hand check book demo delivery business urban music james walker call isbn article book sound business legal advice tailor area music_industry secure record deal start label publishing music marketing promote today musician insightful quote anecdote dozen top executive business urban music entertain informative author james walker leading entertainment lawyer represent known client cole jamie foxx dmx bring professional expertise litigation business intellectual property corporate law business urban music price aspire musician afford career career music_business career music library misti shaw editor susannah cleveland editor isbn article reshape critical reflection art trevisan paola isbn article singer songwriter handbook justin williams editor katherine williams editor call isbn article singer songwriter write perform music present complex figure popular music worlds singer songwriter handbook useful resource student songwriter active musician fan scholar monetize entertainment larry wacholtz isbn article monetize entertainment insider handbook career entertainment music_industry thorough guide exploration state industry emphasis trend copyright digital streaming practical advice develop career technician industry executive book investigate topic entertainment music_industry traditional emerge business model intellectual property right creative destruction happen return hustle eric sheinkop isbn article commercial bring tear movie inspire change life finale television show break heart video game alter perception reality answer least remember music film show game play big work influence emotional response experience fact music include medium purpose connect audience deep visuals strong music strategy fundamental success television film brand video game high expectation audiovisual content take clever animation celebrity cameo connect authentic organic audience genuine music experience exclusive song partnership feature music emerge band build bond extend product experience music touch word feel remember return hustle leading music marketing industry insider discuss diverse audio touchpoints key industry show marketer storyteller advertiser music guide audience customer journey passive brand advocate return hustle blueprint music strategy professional industry attract immerse content extend relationship brand commercial end credit roll detailed exhaustive interview thorough return hustle give playbook marketing power music drive business result awaken business brain jennifer rosenfeld julia torgovitskaya call isbn article businessperson aspire musician ask age interconnectivity answer jennifer rosenfeld julia torgovitskaya founder icadenza cadenza share lesson music career coaching business talent agency awaken business brain receive lot misconception business side art focus self marketing detrimental artistic growth sacrifice big contract sell musician teach businessperson jennifer julia say possible essential survival today music career guidance personal wisdom awaken business brain show foster successful music career sacrifice dedication artistry jennifer julia demystify music_business compassionate encouraging book aspiring musician music_business paul allen isbn article evolution music_business shift influence large record label manager career manager task keep abreast music_industry support manage career include key industry insight exclusive plan guidance tool strategy successful career music_businesshas tool support experienced manager analysis dozen lesson contract author paul allen focused manage career follow best selling second edition feature chapter entrepreneurship include detailed run enterprise business include coverage anticipate risk react challenge basic money chapter contain additional section effective social medium handle promotion additional resource visit book artistmanagementonline understand music_business richard weissman call item stack call status isbn article understand music_business student overview music_business music_business text weismann deliver contemporary approach address unanswered today music student possible living musician understand music_business resume basic text section deal fundamental industry include record music publishing agent manager radio television union internet technology regional international music second half text break ground resume career path industry entrepreneurial skill forge career industry entrepreneurs entrepreneurial aaron isbn article entrepreneurial lesson successful creatives aaron dworkin engage practical guide achieve artistic fulfillment base accomplishment shakespeare mozart several contemporary creatives lesson realize goal matter medium dworkin interview book emmy win actor jeff daniel tony win choreographer bill jones grammy win musician wynton marsalis pulitzer prize winner lin manuel miranda story twelve remarkable come alive lesson love loss despair sacrifice perseverance triumph entrepreneur takeaway explore book include build partnership peer patron sponsor embrace diversity expand focus allow job mature aspiring student practical tool build sustainable career veteran seek reinvention entrepreneurial insight test unusual innovative meaningful kind creative entrepreneurial muse jeffrey nytch isbn article entrepreneurial muse inspire career classical music explore principle entrepreneurship classical music set inspiring student emerge professional educator gain broad perspective strategic understanding require negotiate complexand change landscape professional music career author career journey additional narrative intend inspire broad creative career possibility acquire strategic observational tool design expand possiblecareer path stimulate creative think unique skill find value century realize goal entrepreneurial entrepreneurship creative endeavor entrepreneurship artisticintegrity coexist nurture inspire entrepreneurial muse explains illustrate approach develop maintain career classical music supplement replace traditional music career_development entrepreneurial muse inspire creative imagination give practical tool tohelp realize authentic career sustainable fulfilling impactful art sing onstage studio jennifer hamady call isbn article book great singer talent technique important excellent song able move audience include critical skill address vocal training manage technology studio interact run matter fantastic voice money know job performing record technology tough ride countless phenomenal singer stagnate leave business figure deliver studio headphone monitor communicate producer capable singer art sing studio book address critical issue easy accessible style start discussion evolution technology voice culture explore root cause anxiety related performance issue overcome singer performer producer come book knowledgeable origin field empower tool trade clearer best communicate savvy music teacher david cutler call isbn article possible music teach career meaningful fulfil self support savvy music teacher unveil clear realistic dollar dollar blueprint earn steady income music teacher increase impact income comprehensive resource reveals entrepreneurial lesson find arm cutler expert guidance develop thriving studio transformative curriculum multiple income impact streams innovation strategy aspect business art powerhouse marketing skill financial literacy independence inspired career outlook music student aspire studio owner career instructor establish gurus savvy music teacher pack actionable advice write accessible language real life experience successful teacher entrepreneur feature plan piano success stewart gordon isbn article young pianist pursue professional career face barrage choice challenge book experience teacher performer stewart gordon practical approach plan build secure successful career ground decade gordon guide young pianist detail prepare navigate university forge career livelihood guide begin musical career gordon assemble wisdom decade teach fundamental body emerge pianist rely job goal advice focus mental practical job enhance motivation security balance aspiration reality inspiration organization gordon blueprint transform dream achievement illustrate draw life famous musician book address practical matter develop keyboard technique acquire reading memorize skill build repertoire balance demand musician live full life volume valuable resource young pianist parent teach legal matter teach build award win guitar bill swick isbn article build award win guitar practical guide assist secondary post secondary music educator task involve establish successful music rise interest guitar mariachi rock band handbells bluegrass music technology music educator ask teach innovative music training author bill swick craft book educator build innovative music ground base experience music educator specialize guitar book willassist music educator classroom scheduling structure organization fund raise festival travel subject relate teach guitar classroom principle relevant music educator hop unique standsout university district state attracting student parent educator administrator money music david bruenger isbn article money music tool encourage creative adaptive entrepreneurship music_business write classroom workplace introduce core principle show apply context facilitate deep understanding job music_business apply essential concept real life situation improve capacity analyze solve problem predict music money converge evolving culture legal matter enterprising musician legal toolkit david williams call isbn article enterprising musician legal toolkit</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>普林斯顿大学 职业指南.doc</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
-        <is>
-          <t>普林斯顿大学 职业指南.doc</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
         <is>
           <t>Career Guidance
 Guides
@@ -6878,22 +6746,19 @@
 Call (609) 258-4820 to speak to a reference librarian during most open hours of the Libraries.</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>career guidance guide career career guide profile company industry location guide profession user account outlook bureau labor statistic guide hundred occupation forecast information source vault guide internship pay internship resume connection job experience berger speed press nation economy perlin verso call company source source career librarythis link window career guide profile industry company internship information career advice data axle reference link window information business consumer health care provider business source elitethis link window swot analysis company access company toplevel menu nonprofit link window subscription princeton university library subscription december access date institution information information data directory librarythis link directory institution part directory library source nonprofit criterion asset income type activity blood bank order community group etc etc master list type activity record layout description code institution master revenue service industry source link open window report state industry digit naics code report china market access china section start link china site report internship source guide internship pay internship resume connection job experience berger speed press firestone nation economy perlin verso call source catalog institution graduate student association institution graduate student institution association material graduate student institution student membership rate institution network connection field growth chance access post job chance discipline career path publishing presenting guide association discipline explore association fit career plan growth career material grad future growth website update question guide contact jen hunter jenhunterprincetonedu offline question appointment specialist call call reference hour library</t>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>career guidance guide vault career library career guide resume company industry guide devote profession account occupational outlook handbook bureau labor statistic annual guide job forecast internship vault guide top internship job pay find internship build resume connection gain job experience lauren berger ten speed press call intern nation earn little brave economy ross perlin verso call company firsthand vault career library career guide resume industry company internship career advice data axle detail business health care provider business elitethis swot analysis large company company resume top nonprofit guidestar prothis subscription note princeton university library subscription end december renew non profit organization detailed nccs data archive gale librarythis national nonprofit organization gale library find nonprofit base specific criterion total asset income activity blood bank religious order community theatrical wildlife sanctuary refuge master list activity record layout description code exempt organization master list internal revenue industry ibisworldthis detailed report united state industry digit naics code include report china global china section start global china archival report include internship vault guide top internship job pay find internship build resume connection gain job experience lauren berger ten speed press firestone intern nation earn little brave economy ross perlin verso call additional catalog professional organization graduate student professional association organization graduate student professional organization association key resource graduate student organization reduce student membership rate join organization network connection field discover professional listservs post exclusive job_opportunities feel connect discipline career path start publishing presenting guide mean start explore professional association academic discipline explore association best fit career plan find professional career resource grad future professional update guide contact jen hunter jenhunter princeton chat librarian offline librarian appointment subject specialist call librarian call speak librarian library</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>普渡大学  就业指南.doc</t>
+        </is>
       </c>
       <c r="B46" t="inlineStr">
-        <is>
-          <t>普渡大学  就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
         <is>
           <t>DO THE RESEARCH, LAND THE JOB
 Explore   Start by exploring the possibilities
@@ -7026,22 +6891,19 @@
 The Ultimate Guide to Negotiating Your Salary</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>job start possibility material discipline discipline material information education section career planning guide material career path education choice career field atlas job career accelerator myfuture outlook guide onet online vault career material school guidebook planning tool future material investment basic library literacy guide rating career growth material skill communication skill information literacy growth career learningexpress sage campus sage skill business sage skill student success workplace information literacy search material job internship career field industry chance job board industry website job industry material category search internship experience job field internship way cco calendar discovery internship fund program internship material cco mycco office experience assistance program student service internship work cco calendar discovery internship fund program internship material cco mycco office experience assistance program student service internship work job country material job experience job field internship way cco calendar discovery internship fund program internship material cco mycco office experience assistance program student service internship work indiana youre try job board ascend indiana search option job country material job vista japan goinglobal career account job posting india trabajoscom zhaopin student material visa option culture career account student material center myvisajobscom career account job offer company employer today job market news site market report analysis company profile view company step company material guide database company consult database decision matrix google company news company contact search database abiinform company news check profit database pitchbook hoover company report learn industry ibisworld swot business insight article company applying standout resume cover letter interview skill question experience elevator pitch interview careerspotscom cover letter interview skill interview question answer job career accelerator jobnow cco resume cco resume owl resume resume template industry salary discussion compensation bureau labor statistic job projection job offer cco job seeker calculator overview bureau labor statistic pay wage paycheckcity calculator guide salary</t>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>land job start explore possibility resource discipline discipline specific resource include continue education outline section career planning guide resource explore potential career path determine education right choice bigfuture explore career cco handbook field atlas career guide job career accelerator jobnow myfuture occupational outlook handbook net vault career resource graduate_school guidebook financial planning tool plan financial future include budget resource investment basic library financial literacy guide weiss financial rating professional following resource useful improve certain professional skill communication interpersonal skill literacy personal apply career learningexpress library sage sage skill business sage skill student success workplace literacy resource job internship specific career field industry include job board industry list job specific industry explore resource category keep broad internship want gain experience job field internship fantastic achieve cco calendar discovery undergraduate interdisciplinary internship duiri fund american tfas internship base academic internship internship resource purdue cco mycco purdue office professional practice purdue technical assistance tap virtual student federal internship job indiana cco calendar discovery undergraduate interdisciplinary internship duiri fund american tfas internship base academic internship internship resource purdue cco mycco purdue office professional practice purdue technical assistance tap virtual student federal internship job indiana employment interested job country resource find employment internships want gain experience job field internship fantastic achieve cco calendar discovery undergraduate interdisciplinary internship duiri fund american tfas internship base academic internship internship resource purdue cco mycco purdue office professional practice purdue technical assistance tap virtual student federal internship job indiana find try job board ascend indiana include option internships employment interested job country resource find employment canadajobs cultural vista daijob japan eurojobs gaapweb goinglobal require purdue career account fish job job posting canada naukri india trabajos canada zhaopin china international student check resource settle job live find visa option workplace culture goinglobal require purdue career account international student resource myvisajobs uniworld require purdue career account land job prepare secure company potential employer stand today job_market report swot analysis company resume broad company check company resource guide database started company consult database decision matrix decide start apply google company recent company check linkedin contact interview database abi inform company check recent profit database pitchbook hoover company annual report accept industry check ibisworld swot find business insight global article company comparisons applying interview standout resume resume resume improve interview skill common practice elevator pitch big interview careerspots resume resume interview skill interview answer job career accelerator jobnow myperfectresume network purdue cco resume purdue cco resume purdue owl resume guide resume template vault salary negotiation industry salary prepare salary discussion negotiate ensure receive fair compensation bureau labor statistic bls employment projection job negotiate purdue cco job seeker salary calculator overview bureau labor statistic bls pay wage paycheckcity calculator salary ultimate guide negotiate salary</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>普渡大学  教育学就业指南.doc</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
-        <is>
-          <t>普渡大学  教育学就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
         <is>
           <t>EDPS 105: Academic &amp; Career Planning
 Get Started
@@ -7114,22 +6976,19 @@
 Career Anchors Reimagined</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>career planning welcome career material edp menu access kind information planning strength purdues center career chance major career interest major major theme investigative idea variety career option job sector employer strategy job variety major site major career material learn career option personality interest inventory assessment major admission webpage information major list major collegeschool career interest characteristic list advisor collegeschool info career onet onet program nation source information department laboremployment training administration outlook guide search browse occupation pay education level job growth rate profile people type job family background type job bureau labor statistic career portal material job discipline internship cco library nation road trip story confidence tool career podcasts college student work employer student center career chance center career chance informs empowers student graduate career service career difference student chance state careeronestop flagship career training job search website department labor serf job seeker business student career advisor variety online tool information material buzzfiles engine filter user business compile prospect list cornerstone center cornerstone center corporation material career path science technology engineering mathematics site explores field offer education requirement job data precollege idea career planning material state myers personality test test insight personality type behavior link window aggregate industry report company profile jobseeker material internship job internship cco internship material internship cco website material internship link search engine chance work indiana program institute workforce excellence subsidiary chamber commerce program employer learner school college university job internship career portal material job discipline internship cco library job site world visitor month search employer youll rating people employer employer information tip interview question job seeker linkedin world network internet job internship connect relationship skill career ziprecruiter employer technology million data point match role talent jobsinstead careeronestop flagship career training job search website department labor serf job seeker business student career advisor variety online tool information material cco job search material job career resume salary tip cco job seeker material letter resume interview career success information grad salary grad report calculator state region occupation tip ebooks anchor</t>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>edps academic career planning start welcome welcome career resource edp different kind relate career planning strength purdue career explore major career take major match interest purdue specific major display purdue major holland occupational theme realistic artistic investigative major major idea career option include job sector potential employer strategy land job wide major exploratory expl explore major career include resource major different career option take personality interest inventory assessment purdue major visit undergraduate admission purdue major include list major university university career interest personal characteristic list advisor university university include contact find advise career net net nation primary occupational maintain department labor employment training administration occupational outlook handbook browse job pay education project job growth rate include resume job family gain background job maintain bureau labor statistic purdue career portal resource consider job discipline internship maintain purdue cco purdue library roadtrip nation take road trip capture empower story give confidence tool find career matter videos podcasts university student seek find meaningful job interview employer student purdue career cco career informs empowers student graduate transformative career_services career coach embrace difference connect student professional indiana united state careeronestop careeronestop flagship career training job_search department labor serf job seeker business student career advisor free tool resource buzzfile buzzfile interactive screening engine smart filter empower business compile targeted prospect list career cornerstone career cornerstone corporation manage resource explore career path science technology engineering mathematics medicine extensive explores degree field detail education requirement salary employment data precollege idea career planning resource ball state myers briggs personality test test base insight categorize personality possible identify common behavior plunkett aggregate industry report company resume job seeker resource find internship job find internship purdue cco internship resource internship cco include resource internship start internship engine job indiana job indiana institute workforce excellence subsidiary indiana chamber commerce employer learner high university university university find job include internship purdue career portal resource consider job discipline internship maintain purdue cco purdue library job unique visitor month glassdoor potential employer find rating job employer depend employer find salary tip interview ask job seeker linkedin linkedin large professional network internet linkedin find right job internship connect strengthen professional relationship skill succeed career ziprecruiter rat employer powerful matching technology analyze million data find best match work invite top talent apply job wait careeronestop careeronestop flagship career training job_search department labor serf job seeker business student career advisor free tool resource purdue cco global job_search resource job career tip resume interviews salary pro tip purdue cco job seeker resource resume resume resume cvs interview career success handbook salary recent purdue grad salary purdue grad major report earn graduate salary calculator calculate project salary state job tip career ebooks career anchor reimagined</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>杜克大学 就业指南.docx</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
-        <is>
-          <t>杜克大学 就业指南.docx</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
         <is>
           <t>Career Tools: Print, E-Book, &amp; Audiobook
 Links to continually updated lists of e-books, print books, and audiobooks that you can browse or search -- all focused on helping you with your job and career search.
@@ -7153,22 +7012,19 @@
 ORBIS covers over 400 million companies worldwide, with an emphasis on private company information, integrating information held across BvDEP's company information product range. ORBIS provides global standard report formats as well as descriptive information, and company financials, along with news, market research, ratings and country reports, scanned reports, ownership and M&amp;A data.</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>career tool ebook audiobook link list ebooks book job career search title youd book ebooks database career company job advice guidance career intelligence vaultcom material vault guide ranking article career strategy job posting vaultcom student onestopshop student alumnus job information career chance visa immigration support screen company capital contains company analysis pitchbook search thousand equity venture capital deal hundred criterion pitchbook benchmark time data deal identify comparables search investor detail data reference usa information address phone business resident health care provider consumer orbis company emphasis company information information bvdeps company information product range report format information company financials news market rating country report report ownership data</t>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>career tool print book audiobook updated list book print book audiobooks browse focus job career know title add know book print book audiobooks overdrive database career company job advice guidance vault career intelligence vault primary resource vault guide vault ranking article career job seek strategy job posting due cost vault fuqua student interstride stop shop empowers duke student alumnus seek international employment career network mentorship visa immigration support screen company finance contains comprehensive fundamental quantitative company analysis pitchbook equity venture finance deal criterion pitchbook establish benchmark find real data deal identify analyze comparables investor detail data fka usa contain detailed include address phone business resident health care provider orbis orbis resume company worldwide emphasis company integrate hold bvdep company product orbis global standard report format descriptive company finance rating country report scan report ownership data</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>波士顿大学 就业指南.doc</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
-        <is>
-          <t>波士顿大学 就业指南.doc</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
         <is>
           <t>Career Research @ Pardee Library - OLD
 Assistant Head, Information Services
@@ -7290,22 +7146,19 @@
 Publication Date: 2021</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>career pardee head information service contact subjectsbusiness management guide guide material company industry information career internship job search tab side guide database part project book jobcareer job search guide top source company information company create company list tab list company industry area revenue text access newspaper publication business newswires press release medium transcript news photo investment analyst market report country profile company market data data axle solution directory business consumer business company area business type code revenue location employee job listing directory business contact information headquarters subsidiary branch firm office country country industry directory firm country firm state pardee source company industry information information industry company profession list job prospect listing company industry geography prepare interview company industry interview career exploration industry career guide access boston university career center registration time user step account click register bottom box email address registration create account click link firsthand email address minute note firsthand email profile material industry company profession vault guide ranking vault guide select tab side youll link guide navigation bar vault ranking career career side ranking field career firsthand industry profession industry profile profession profile industry report industry report career focus sale finance regulation issue material statistic industry industry business challenge chance preparation question ratio outlook guide industry guide department labor description myriad job nature work job outlook earnings target company list company company dossier university company dossier box click create company list list company industry area revenue company sale data axle solution directory business consumer business company area business type code revenue location employee job listing business data axle reference solution click screener toolbar company industry geography keyword business description affiliation online directory business contact information headquarters subsidiary branch firm office country country industry directory firm country firm state directory insight insight track venture capital investment activity company search company hand column list company industry geography access campus connect guidestar database institution list institution type area search keyword city state type income range directory advertising agency client brand medium expenditure list company contact email job search book website job book job career growth management career pivot exploration diversity workplace relationship experience website website company information employee career builder dice tech job career jobscom nationjob network job service zip recruiter preinterview database company news competition structure subsidiary history mission management team product service analysis company information company information source company hoover company link window hoover company record database contains information company record overview year job data list product competitor officer address phone fax company link window marketline datamonitor company profile company profile business description company history key employee productsservices competitor profile weakness chance threat analysis company profile browse list company profile company browse search box click button business source company news factiva link window text access newspaper publication business newswires press release medium transcript news photo investment analyst market report country profile company market data business link window business combine business information accounting tax amp banking entrepreneurship document database journal magazine news source thousand ebooks video company industry country report link window nexis university source newspaper magazine trade journal service transcript source state statute court decision information company executive company insight company overview employee perspective information company vault answer hour phone call reference contact person appointment tech internship search internship career library school business major minor alum access vault industry information range industry guide tab industry company registration detail instruction career guide career exploration internship httpswwwcheggcomappinternship internjobs httpwwwinternjobscom internweb httpwwwinternwebcom star internship httpwwwsumerjobscom company target company list cover employability search work experience stewart book phenomenon internship policy issue time internship internship way education work contribution scholar range discipline book benefit regulation arrangement country world challenge work intern need form regulation exploitation intern background standard data analysis internship extent bridge education job internship employability search work experience material policymakers academic law relation economics material management education location online publication date</t>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>career pardee library old assistant head contact pardee library subject business start guide guide design best library resource relate company industry pertain career internship job_search left hand side guide relevant database project book find job career right guide top company nexis university international company company list list international company industry geographic area revenue factiva worldwide full text local regional report trade article business newswires press release wire medium transcript photo business rich websites investment analyst report report country regional resume company resume historical data data axle solution historical business business company geographic area business sic code revenue employee include job internship listing uniworld business contact headquarters subsidiary branch multinational firm office country resume country industry release separate uniworld label american firm operate foreign country foreign firm operate united state career pardee library company industry industry company profession list job prospect listing company industry geography prepare interview company industry walk interview career exploration industry career guide firsthand vault boston university career registration require follow account firsthand start bottom enter address next complete registration account start firsthand mail confirm address take several minute note firsthand send follow complete resume require optional excellent resource job industry company profession find vault guide ranking vault guide library library left side guide top navigation bar vault ranking career career left side ranking various field career include firsthand industry profession include industry resume profession resume industry report industry report career focus include sale finance regulation regional international issue human_resources statistic industry contain quarterly industry update business challenge trend call preparation ratio occupational outlook handbook industry guide department labor include description myriad job include nature job require train job outlook earnings target company list company directories company dossier nexis university company dossier company list list international company industry geographic area revenue rank company sale data axle solution historical business business company geographic area business sic code revenue employee include job internship listing tutorial list business tutorial data axle solution netadvantage quick screener screen top toolbar company industry geography keyword business description corporate affiliation international uniworld business contact headquarters subsidiary branch multinational firm office country resume country industry release separate uniworld label american firm operate foreign country foreign firm operate united state specialized insight insight track global venture finance investment activity relate company advanced company left hand column list company industry geography connect vpn guidestar national database nonprofit organization list nonprofit organization geographical area keyword city state nonprofit income winmo advertising agency key client brand include medium expenditure sample good list company contact include job_search book websites job_search book job_search career_development career pivot exploration diversity workplace network relationship build international experience websites glassdoor useful company salary employee linkedin bostonjobs career builder dice high technology job financial career job nationjob network net temp job post zip recruiter pre interview following database find late company competition corporate structure subsidiary finance history mission product swot analysis company company company overviews hoover company record hoover company record database nexis university contains major company worldwide depth record include overview histories key financial employment data list product key competitor key officer address phone fax marketline company resume marketline datamonitor company resume resume company resume include business description company history key employee major product competitor resume contain strengths weakness threat swot analysis locate company resume browse alphabetical list company resume company browse browse business complete company factiva full text local regional report trade article business newswires press release wire medium transcript photo business rich websites investment analyst report report country regional resume company resume historical data proquest business proquest business combine multiple proquest business databases include abi inform accounting tax amp banking entrepreneurship contain report content database resume article magazine several ebooks video company industry country report university nexis university report magazine trade article wire transcript legal federal state statute include supreme court decision international company executive company insight glassdoor company overviews employee perspective include salary job company firsthand vault ask answer pardstf phone call contact person library appointment technology internship websites internship firsthand vault career library questrom university business major minor alum firsthand vault industry broad industry guide premium industry company guide registration detail complete instruction career guide career exploration internship websites chegg chegg app internship internjobs internjobs internweb internweb rise star internship rsinternships summerjobs sumerjobs company directories target company list resume artinternships employability decent job experience andrew stewart groundbreaking book examine grow phenomenon internship policy issue raise internship traineeship important transition education pay job feature contribution establish emerge scholar discipline book present important benefit regulation arrangement consider various country meet challenge ensure decent job intern realise objective regulation minimise prevent exploitation intern explore background possible international labour standard present data analysis internship extent effective bridge education employment internship employability decent job experience key resource policy maker academic labour law industrial relation labour economics human resource education article</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>波士顿大学 就业服务介绍.doc</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
-        <is>
-          <t>波士顿大学 就业服务介绍.doc</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
         <is>
           <t>Kickstart Your Career Research at Pardee Library
 As you start looking for internships or begin your entry into the job market, we’re here to remind you that Pardee Library is your go-to resource for career research. Our Career Research @ Pardee Library guide is an excellent tool to jumpstart your career exploration. It’s designed to help you delve into industry research, create target company lists using our extensive company directory databases, and access a wide range of job search literature covering topics from career development and pivots, to networking, diversity in the workplace, and more.
@@ -7313,22 +7166,19 @@
 If you need any help navigating these resources, don’t hesitate to reach out to our friendly staff at pardstf@bu.edu or visit us in person. We’re here and ready to help you succeed in your career endeavors!</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>career library internship entry job market goto material career career pardee guide tool career exploration industry create target company company directory database access range job search literature topic career growth pivot diversity workplace guide section preinterview internship material hesitate staff pardstfbuedu person career endeavor</t>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>kickstart career pardee library start internship begin entry job_market remind pardee library resource career career pardee library guide excellent tool jumpstart career exploration design delve industry target company list extensive company database wide job_search literature resume topic career_development pivot network diversity workplace guide include specific section pre interview find internship navigate resource hesitate reach friendly staff pardstf visit person ready succeed career endeavor</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>纽约大学-职业导航.docx</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
-        <is>
-          <t>纽约大学-职业导航.docx</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
         <is>
           <t>Job Search, Interviewing, and Compensation
 Home
@@ -7683,22 +7533,19 @@
 A: While Firsthand's ca...</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>job search interview compensation home welcome guide job hunt youre campus killer internship corner office layoff midcareer pivot event job database training date job internship search country city guide business etiquette advice countryspecific regulation job applicationinterview advice training nav highimpact document recruiter briefing moment document analyst report workspace online swot database marketline globaldata report industry report question firstresearch analyst question earnings conference call transcript workspace streetevents report direction interview job hunt meet career coach overarching strategy career plan doc target company list need strength aspiration step networking hurdle company industry interview compensation data offer circle career coach job search work life work life bill burnett evans thinking life regardless living book career service step hour job hour job search technology job dalton detail approach job efficiency strategy dalton program director career consultant school business ebook copy ebook copy job job technique resume interview negotiation dalton advice dream job resume cover letter interview offer ebook time restriction job search interview min video recording learn highimpact highpayoff material strategy job search interview material presentation advice strategy career coach workshop request instructor student group lead time log zoom sso career center job search coaching mentoring accompaniment career job material dont hesitate career centerdepartment office career growth ocd career center career master of business administration graduate student wasserman center career growth student college art science center wasserman service school student career service support student school engineering brooklyn wagner office career service career growth nyu abu dhabi career growth stern career management center cmc stern master of business administration career guide career material shanghai henry huang sep view year target company target company list datarich approach chance company interest work need life situation job hunt chance campus careersindustries list material allow list company data point result excel analysis manipulation company link window link window link window data company statement madeals lbos executive board screening feature list firm task investment analysis coursework job search information capital guide password cooky web browser capital incognito window mergent intellectthis link window click search list lseg workspace link window account creation account request business day period user account interface workspace access data company merger acquisition market data quote analyst report equity venture capital screening capability product thomson eikon workspace user andor download analyst report hour period faculty access availability business library team form user web platform mac software startup link window click company deal list note result pitchbook user pitchbook interface duo push step screen york university sign sign sso email netidnyuedu user library download print limit row maximum row capture bulk data access wrds wrds refer wrds guide information nonprofit foundation directory onlinethis link window search search feature database institution access section guidestar account user record month registration link product dive company information interview ranking firsthand firsthandthis link window user account email address access database employer list ranking insider information employee intern year survey thousand career intern result survey employer internship program industry diversity quality life company click career lefthand nav ranking category advertising marketing banking consumer service consumer product energy internship law technology material interview time document utility employer sphere analyst report workspace link window account creation account request business day period user account interface workspace access data company merger acquisition market data quote analyst report equity venture capital screening capability product thomson eikon workspace user andor download analyst report hour period faculty access availability business library team form user web platform mac software difference analyst report online workspace swot workspace interface globaldata report search swot keyword user andor download analyst report hour period faculty access availability business library team form user web platform mac software business source industry report prep question link open window click submit search browse report industry click profile report ibisworldthis link window ibis world collection industry market password earnings call transcript link window company search company blue arrow search transcript blue arrow word earnings call date range sort login campus lseg workspace search company ticker navigation bar contributor field search streetevents thomson reuters streetevents date range result user andor download analyst report hour period faculty access availability business library team form user web platform mac software data source material step position market value mind salary factor job seniority industry location locate source order consensus data source compensation calculator job search site employee compensation company survey project site data stop outlook guide range profession government data bureau labor statistic department labor survey trade industry association survey compensation survey membership layer paywall relocating calculating change cost cer data toolkitthis link window cer cost index coli cost area manhattan brooklyn queen insight tax income cost expenditure grocery housing utility transportation healthcare expenditure household type consumer price good service home price energy bill gasoline doctor visit prescription drug negotiation compensation package linkedin video minute aries linkedin video overview negotiation beginner advice pay job offer hour minute deepak malhotra lecture harvard business school professor deepak malhotra insight job book negotiation agreement roger fisher ury book negotiation strategy edge ask woman negotiation linda babcock sara guide woman author negotiation woman negotiation gender divide linda babcock sara laschever babcock force woman industry insight industry career guide link open window vault guide jobseekers industryspecific advice job search database click vault guide navigation category user account email address access database accounting banking finance energy hospitality insurance engineering investment management law medium entertainment industry estate industry profile link open window sale personnel industry overview industry trend chance business challenge link news link window collection industry market overview industry target market driver projection material netid password password standard poor link window industry survey range industry survey company click industry survey access industry information browser cooky access material globaldata disruptorthis link window disruptor track chance industry information startup innovation technology influencers consumer insight venture capital portfolio investment click access disruptor access database news date recruiter interviewer company industry news tool employer topic uptodate knowledge company press release business news source interview executive business newspaper nyu business library list database access article magazine newspaper business source completethis link window text business database database keyword company company entity menu right search box factiva link window link window search newspaper news transcript trade journal news business information factiva press material information company companiesmarkets support report company login campus nexis link window access newspaper news wire transcript trade journal company info template company information news browser cooky access material bloomberg brief brief brie newsletter date field job search topic economics economics economics market oil oil europe oil asia credit regulation equity hedge fund report visa company work visa job recruiter tool company work visa myvisajobs job title company visa approval goinglobals database million submission listing employer talent state department labor record search engine position job location range company occupation industry job title visa submission record date identify employer career skill website employer record work visa card salary withdrawn tip visa company role asset candidacy example company operation india career goal rule possibility company office possibility transfer location america offer sponsorship state neighbor canada speaking country pas chance place netherlands business life premba gmat master of business administration submission strategy montauk gordon submission book bschool admission officer submission consultant master of business administration program richard montauk table content master of business administration type master of business administration program school ranking admission submission timetable credential principle essay topic essay recommendation interview rejection disappointment business school example essay admission strategy gordon table content admission fundamental admission value element admission master of business administration program hand submission profile recognition growth profiling project profile analysis profile analysis positioning essay interview management master of business administration question archetype approach content interview writing tool method reader structure outline expression word sentence strategy tip interview admission officer program insight submission school submission admission team cover letter job search customization admission success example podcast interview executive director admission business school ranking time business school asiapac diversity index list master of business administration candidate industry consumer healthcare energy estate mediaentertainment nonprofit transportation government hospitality business school quants news business school time bloomberg businessweek business school asiapac diversity index time master of business administration list executive master of business administration finance management business school year master of business administration program year master of business administration program time master of business administration list executive master of business administration finance management business school executive master of business administration program news executive master of business administration program fortune part time master of business administration program news parttime master of business administration program fortune online master of business administration news world report master of business administration undergraduate business program quants business program news world report business program admission consultant service admission consultant program poet quants article consultant master of business administration admission consultant master of business administration admission consultant master of business administration admission consultant admission consulting firm preparation company company variety forfee class product service person online gmat executive assessment note nyu company service option curve prep manhattan princeton varsity tutor material business alumnus material access nyu business team learning alumnus selection subscription material enrichment career advancement access database charge world alumnus netid thats dan head nyu business library business database alumnus business source alumnus edition topic trade publication magazine journal newspaper market report industry profile country report abiinform feature thousand journal dissertation newspaper time country report data company hoover hoover company executive profile industry coverage company fact sheet mergent intellect directory company information financials personnel building list company industry industry coverage prep question interviewer career job seeker traveler location country city guide business etiquette advice countryspecific regulation listing employer visa job applicationinterview advice firsthand insight employer culture pro con firm etc series employer list industry function guide information career work environment education requirement day life career outlook alumnus access career material career developmentsternlife archive archive access collection industry document mergents collection manual equity report report industry report collection mergent bondviewer mergent bond viewer access bond data issuer bond level term condition data bond bond note sport market analytics market industry trend statistic sport sport business library access periodical reference search mix journal trade publication magazine discipline jstor highquality content scholarship jstor journal humanity science science monograph material work project muse version journal booklength scholarship humanity art science press society collection scientist volume year discipline physical science health management collection material field health administration journal dissertation newspaper indexing user news information issue newspaper researcher access news story information section cover information company people product law journal heinonline law periodical coverage issue periodical issue contract publisher article title author state country text date material discipline alumnus portal home alumnus material purchase access business library alumnus subscription access material vendor subscription thank option bobst access benefit gift business andor alumnus material thank dan head business generosity need student scholar business metropolitan area business library community standout example city standalone business facility department library list business database york yoseloff business center stavros foundation library snfl avenue floor york brooklyn library business career center army plaza floor brooklyn email business library angeles library business economics department library philadelphia business material innovation center library business science technology center library kirstein business innovation center library pittsburgh business spokane public county district library business forfee business service firm industry excellence expertise askstatista information service advantage society freelance career intelligence career association information career question job search time program guidance career office timeline recruiting summer internship program career center advisor timeline program course job search month part time time master of business administration assist student material career part time program career coach experience industry role advice</t>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>job_search interviewing compensation welcome guide design connect tool useful job hunt recruit secure killer internship corner office bounce layoff mid career pivot event goinglobal job internship database training multiple goingglobal improve job internship include country city guide business etiquette advice country specific visa regulation include job application interview advice training top nav high impact report meet recruiter attend corporate briefing moment prepare impactful report analyst report lseg workspace mergent swot analyse database marketline globaldata report industry report call prep firstresearch ibisworld analyst quarterly earnings conference call transcript lseg workspace streetevents report factiva find direction interviewing job hunt roadmap meet career coach develop overarching strategy timeline career plan worksheet google doc target company list customize strength aspiration identify next networking hurdle address company industry prepare interview salary compensation data best circle career coach librarian job_search evolve design job life design job life bill burnett dave evans burnett evans show design thinking life meaningful fulfil regardless living young old book recommend stern career_services job_search job_search technology right job steve dalton detail holistic approach job_searching focus efficiency proven strategy dalton director senior career consultant duke university fuqua university business ebook hard copy ebook archive hard copy job closer job close save technique ace resume interview negotiation steve dalton advice land dream job write perfect resume resume resume nail interview negotiate ebook limit due publisher restriction training record optimize job_search interview library min video recording high impact high payoff resource strategy systematize job_search prepare corporate interview resource presentation design complement advice strategy career coach training stern instructor student allow sufficient lead schedule log nyu zoom sso nyu career job_search coach mentoring critical accompaniment career employment resource library hesitate reach career department stern office career_development ocd career job professional ccwp serve stern master of business administration graduate student alumni wasserman career_development serf nyu nyc student include university art science sps wasserman wasserman exclusive university professional sps student tandon career_services career support student enrol nyu tandon university engineering brooklyn wagner office career_services nyu shanghai career_development nyu abu dhabi career_development stern nyuad career cmc serve stern nyuad master of business administration alumni career guide career resource nyu shanghai henry huang last updated sep target company list build target company list data rich data approach find prioritize surface company interest come mind job unique life situation job hunt recruit change career industry build list resource allow build list company base data important result export excel analysis manipulation company finance data company financial statement deal lbos executive board worldwide screening chart feature list firm task investment analysis coursework job_search finance guide require netid password important third party cooky enable browser set finance incognito recommended mergent intellectthis advance begin build list lseg workspace account creation require account require mandatory business period exist account log interface lseg workspace fundamental financial data company merger acquisition financial data quote analyst report equity venture finance feature powerful screening chart capability product know thomson eikon refinitiv workspace permit analyst report content amr period faculty expand amr pending availability business library log lseg platform lseg mac software startup pitchbook company deal begin build list note result pitchbook limited direct pitchbook interface duo push follow base screen prompt sign university prompt sign pitchbook sign sso enter nyu netid nyu nyu library log daily print limit restrict row monthly maximum row screen capture prohibit bulk data pitchbook wrds wrds account refer wrds guide profit foundation onlinethis advanced feature guidestar national database nonprofit organization premium section guidestar account nyu permit record month registration product deep dive foundational company prepare interview find employer ranking firsthand firsthandthis account nyu address database best employer list firsthand vault ranking base exclusive insider verify employee intern firsthand survey full professional intern result survey rank top employer internship various industry prestige diversity quality life overall company job career left hand nav browse ranking top category account advertising marketing banking consult product energy internship law technology interview interviewing resource schedule interview limit prepare report high practical utility come understand potential employer sphere compete analyst report lseg workspace account creation require account require mandatory business period exist account log interface lseg workspace fundamental financial data company merger acquisition financial data quote analyst report equity venture finance feature powerful screening chart capability product know thomson eikon refinitiv workspace permit analyst report content amr period faculty expand amr pending availability business library log lseg platform lseg mac software faq difference analyst report mergent lseg workspace swot analyse lseg workspace interface describe globaldata marketline report advanced include swot keyword permit analyst report content amr period faculty expand amr pending availability business library log lseg platform lseg mac software business complete industry report call prep researchthis submit browse find report industry full resume complete report ibisworldthis ibis comprehensive collection industry require netid password quarterly earnings call transcript factiva company add company blue arrow subject add transcript blue arrow word earnings call adjust sort recent necessary require netid lseg workspace company ticker navigation bar contributor field streetevents thomson reuters streetevents adjust result permit analyst report content amr period faculty expand amr pending availability business library log lseg platform lseg mac software salaries negotiation salary data resource understand position value keep mind salary structure influence factor include job title seniority industry geographic locate salary possible order determine consensus data compensation salary salary calculator glassdoor job_search employee post compensation large company payscale salary survey tool salary project submit salary data career stop occupational outlook handbook salary_ranges profession government data bureau labor statistic department labor salary survey professional trade industry association produce salary survey critical understand salary compensation salary survey membership layer paywall relocating calculating change cost live regional economic data toolkitthis cost live coli compare cost live metro area include manhattan brooklyn queen coli include insight tax income overall cost key expenditure grocery housing utility transportation healthcare anticipate monthly expenditure household average local price common good include rent price energy bill gasoline doctor visit prescription drug negotiation negotiate compensation package linkedin video minute emilie aries linkedin video basic overview negotiation beginner include advice ask pay negotiate job youtube minute deepak malhotra lecture harvard business_school professor deepak malhotra conceptual practical insight negotiate job seminal book negotiation negotiating agreement give roger fisher william ury famous book negotiation foundational strategy give edge negotiate ask woman negotiation want linda babcock sara laschever guide negotiate woman inform author negotiation gender woman ask negotiation gender divide linda babcock sara laschever babcock examine social force dissuade woman negotiate industry insight vault industry career guide firsthandthis firsthand know vault career guide arm job seeker foundational industry specific advice approach job_search enter database vault guide top navigation overarch category find account nyu address database accounting advertising marketing banking finance consult energy hospitality insurance engineering investment law medium entertainment industry pharma healthcare real estate industry resume researchthis design enable sale personnel speed industry overview industry trend business challenge recent article ibisworldthis comprehensive collection industry include great overview industry target important driver projection resource sign netid password require netid password standard poor netadvantage industry survey international industry relevant survey company industry survey industry clear browser cache cooky attempt resource globaldata disruptorthis disruptor track emerge technology enable industry start ups technology lead innovation late technology trend influencers insight venture finance portfolio investment disruptor database recruiter interviewer want knowledgeable company industry tool prep meet potential employer avoid controversial topic demonstrate knowledge start company include press release business outline interview relevant suite executive business report nyu business library complete list database article magazine report major list business completethis full text business database database keyword limit company company entity dropdown right factiva international report transcript trade article business factiva include corporate press release good resource small company company tabs support generate report company require netid nexis full text report international wire transcript trade article company template company clear browser cache cooky attempt resource bloomberg brief bloomberg brief brie weekly newsletter useful keep certain field job_search topic include economics economics europe economics asia municipal oil americas oil europe oil asia credit regulation etfs equity hedge fund dine quicktake special report visa visa determine company sponsor job visa difficult disclose job post recruiter tool determine successful company sponsor job visa myvisajobs job title company receive visa approval hire goinglobal goinglobal goinglobal database million visa application listing american employer seek international talent united state department labor record engine allow identify position job salary_ranges base company job industry job title certified visa application record identify employer hire international professional skill set free understand employer track record come sponsor job visa green card include salary certify deny withdrawn tip visa prove elusive wish prioritize apply company work bilingual asset strengthen candidacy speak hindi english target base company significant operation india match career goal rule possibility job large company international office explore possibility internal transfer preferred interested job north america luck secure include visa sponsorship united state forget neighbor north canada english speaking country pas netherlands singapore english business life pre master of business administration gmat master of business administration application strategy montauk gordon recommend master of business administration application book bschool admission officer master of business administration application consultant top master of business administration richard montauk table content master of business administration master of business administration right university ranking admission application timetable credential principle understand key essay topic write persuasive essay recommendation interview respond wait listing rejection disappointment accepted business_school finance master of business administration essay master of business administration admission strategy gordon table content admission fundamental talk adcom master of business administration admission value element admission master of business administration hand application resume recognition profiling project personal resume analysis professional resume analysis positioning message essay interview master of business administration archetype essay approach content map interview writing tool method serve structure outline improve expression word sentence strategy tip find interview admission officer intend apply insight successful application university tailor application admission resume resume job_search customization critical admission success accept nyu stern podcast interview lindsay loyd executive director master of business administration admission stern business_school ranking full master of business administration bloomberg businessweek best business_school include europe canada asia pac diversity include top list master of business administration candidate hire specific industry include consult financial technology healthcare manufacture energy real estate retail medium entertainment nonprofit transportation government hospitality forbes best business_school poets quants top master of business administration composite rank best business_school full master of business administration international bloomberg businessweek best business_school include europe canada asia pac diversity financial global master of business administration rank include list master of business administration executive master of business administration finance european business_school best international master of business administration forbes best international master of business administration executive master of business administration financial global master of business administration rank include list master of business administration executive master of business administration finance european business_school executive master of business administration executive master of business administration master of business administration fortune best master of business administration best master of business administration master of business administration fortune best master of business administration report best master of business administration undergraduate business poets quants undergrad business report undergrad business master of business administration admission consultant secure admission consultant useful determine competitive find several poet quants article determine hire consultant right master of business administration admission consultant cost hire master of business administration admission consultant top master of business administration admission consultant master of business administration admission consulting firm gmat preparation company profit company fee training tutor product person prepare take gmat executive assessment note nyu endorse recommend particular company include option bell curve gmat manhattan prep manhattan princeton varsity tutor nyu alumni resource business library alumnus resource welcome nyu business library believe support lifelong learning alumnus selection subscription resource personal enrichment career advancement database provided free charge active alumnus netid require log dan hickey head nyu business library business database nyu alumnus start business alumnus edition resume business related topic present include trade article magazine academic article report report industry resume swot analysis country report proquest abi inform complete feature full text article dissertation job key report financial country industry focus report data company hoover hoover contain company resume include key executive resume industry coverage detailed company fact sheet mergent intellect mergent intellect company worldwide include contact finance key personnel mergent intellect list company easy industry industry resume include international coverage include call prep prepare meet interviewer career goinglobal goinglobal job seeker traveler job live include country city guide business etiquette advice country specific visa regulation include listing employer sponsor visa job application interview advice firsthand vault insight potential employer include organizational culture pro con job firm best employer list different industry function ebook guide career include job environment education requirement life career outlook stern alumnus additional career resource stern career_development sternlife focus mergent archive mergent archive indexed collection corporate industry related report include mergent full collection digitized manual ford equity report annual report industry report collection mergent bondviewer mergent bond viewer bond data include issuer bond term data taxable bond municipal bond retail note sport analytics industry trend statistic relate sport sport business useful proquest library stop periodical broad inclusive databases respect diversified mix scholarly article trade article magazine resume academic discipline jstor high quality interdisciplinary content support scholarship teach jstor digital archive include lead academic article humanity social science science monograph material valuable academic job project muse complete full text version scholarly article book length scholarship humanity art social science university press scholarly society annual comprehensive timely collection critical write lead scientist annual volume publish focused discipline biomedical physical social science proquest health collection reliable relevant resource field health administration include article dissertation proquest report database detail indexing find issue report indexed researcher top story contain various section resume complete bibliographic company product law article library heinonline contain law law relate periodical coverage issue publish periodical publish issue allow base contract publisher article title author subject state country publish full text narrow alumni resource discipline alumnus library portal nyu alumnus resource faqs purchase great business library alumnus subscription resell resource job vendor pursue personal subscription thank understanding visit bobst library option bobst library benefit gift support business library alumni resource contact thank contact dan hickey head business library generosity best meet nyu student scholar leverage local business library major metropolitan area business library dedicate serve local community find standout city standalone business facility department library maintain list business database library yoseloff business stavros niarchos foundation library snfl fifth avenue brooklyn library business career central library grand army plaza brooklyn business library los angeles library business economics department free library philadelphia business resource innovation san francisco library business science technology boston library kirstein business library innovation kblic carnegie library pittsburgh downtown business library spokane county district library spokane business library fee business firm know industry excellence expertise askstatista bat bizologie librarian advantage professional society useful locate freelance professional strategic competitive intelligence professional scip association independent professional aiip ask start job_search full master of business administration receive guidance career office timeline recruiting summer internship master of business administration career advisor timeline base training begin job_search less month intend graduate master of business administration full master of business administration library assist nyu student wish resource advance career include non stern assigned career coach limit experience industry work seek targeted advice firsthand</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>耶鲁大学 职业指南.doc</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
-        <is>
-          <t>耶鲁大学 职业指南.doc</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
         <is>
           <t>Business &amp; Management Research Guide: Career Resources
 A guide to business and management resources at Yale Library.
@@ -7802,22 +7649,19 @@
 The National Compensation Survey (NCS) is an establishment-based survey that provides comprehensive measures of (1) employer costs for employee compensation, including wages and salaries, and benefits, (2) compensation trends, and (3) the incidence of employer-sponsored benefits among workers. The NCS also collects data and produces estimates on the provisions of selected employer-sponsored benefit plans. Freely available site.</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>business management guide career material guide business management material career job search material career material job search source regulation database job trend range advice vault firsthand career insider feature industry vault career guide ranking article company interview advice student faculty staff company target list strategy company strategy custom company list way company industry trait example ranking list knight company startup employer list business employee criterion reputation employee satisfaction growth impact data dataset impact data corporation dataworld lab user account culture index mit culture company world company charity charity amount support period data company asset investment fund company interbrand brand world brand management consulting firm forbes area filter innovation consulting firm board innovation yale material firsthand feature access vault list company range industry function list banking consulting accounting firm information firm culture compensation balance student register account sign yale block data analysis asset landscape ecosystem view space example stablecoins gaming blockchain ecosystem ecosystem bridge knowledge gap user yale email address impact alpha news insight trend impact investing impact market data tool section tool target company fund list finance tracker space competitor list company profile company competitor reason source search company industry location size criterion database capital realtime information company market transaction people account email address individual account netadvantage functionality mergent directory business information access business data executive contact information industry data hoover database bureau van dijk information company feature coverage company ownership startup company database insight insight information startup company investor user account email address pitchbook feature time data analyze company deal fund investor service provider investment lifecycle user email address user yale signin log sso account search institution location program guidestar directory institution information analyst report search equity fund firm database source data equity investment list firm fund manager industry industry survey capital access industry survey cfra hover market navigation bar top industry survey market list industry industry trend data question feature report industry overview statistic analysis market characteristic condition performance industry participant subscription report state report archive canada mexico china report find industry market material search contact capital capital realtime information company market transaction people account email address individual account netadvantage functionality leadership leadership find background contact information leader business government nonprofit state export function subscription mergent directory business information access business data executive contact information industry data hoover news information service access newspaper magazine transcript business information information company contact information question science science yale university library street level team allison gallaspy wachowicz schedule appointment website subjectsbusiness management economics workshop handout building target list company career service support yale career growth office student alumnus career material alumnus yale college office career strategy compensation data angelco startup salary equity role location skill market site comparison tool insider business insider database year disclosure website range company reporter registration account instruction database capital compensation job edition collaboration compensation specialist ferguson partner trend statistic capital firm world insight section preqin instruction report compensation survey bureau labor statistic compensation survey survey measure employer cost employee compensation wage salary benefit compensation trend incidence benefit worker data estimate provision benefit plan site</t>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>business guide career resource guide business resource yale library career job_search resource goinglobal global career resource feature job_search job permit visa regulation include searchable database employment trend salary_ranges cultural interview advice vault career call firsthand career insider feature industry function focus vault career guide vault ranking article company interview advice student faculty staff log vault netid company target list strategy exist company list strategy custom company list exist list quick easy identify company specific industry specific trait ranking list global corporate knight sustainable company america best startup employer forbes list compile evaluate business least employee base criterion employer reputation employee satisfaction growth corp impact data dataset contain impact data certified corporation publish data lab require free account culture interactive mit measure compare culture company forbes global large company forbes top charity large charity iin america measure amount support receive late fiscal period data large company impact asset impact investment fund inc fast grow company america interbrand best global brand rank valuable brand best consulting firm annual rank forbes section functional area filter top innovation consulting firm board innovation yale resource vault call firsthand feature vault list top ranked company resume industry function include list best banking consulting accounting firm rankings include firm culture compensation job life balance student account sign yale block feature data depth analysis digital asset landscape ecosystem map foot entire stablecoins blockchain gaming nyc blockchain ecosystem speed ecosystem bridge potential knowledge gap sign valid yale address impact alpha feature insight global trend impact investing social impact financial data tool section include tool identify target company include fund list climate finance tracker impact competitor list company resume company databases note competitor identify various reason depend company industry criterion following database finance finance real historical company transaction worldwide require account yale address want account netadvantage similar functionality mergent intellect global business feature international business data executive contact industry data hoover orbis database bureau van dijk company notable feature include extensive coverage company corporate ownership structure identify start backed company database insight insight real global start company investor require sign account yale address pitchbook feature real data analyze company deal fund investor provider entire investment lifecycle require sign yale address direct yale sign log sso account commercial prohibit nonprofit organization guidestar searchable nonprofit organization feature operational financial analyst report equity hedge fund firm following database preqin historical data equity alternative investment generate list firm fund manager industry cfra industry survey finance industry survey cfra hover locate navigation bar top industry survey locate list industry report mergent intellect industry resume include trend benchmark data call prep ibisworld feature report industry overview key statistic analysis characteristic operate project performance major industry participant subscription include report include state report historical archive canada mexico china global report find industry additional resource contact finance finance real historical company transaction worldwide require account yale address want account netadvantage similar functionality leadership connect leadership library find background contact business government nonprofit united state note export function subscription mergent intellect global business feature international business data executive contact industry data hoover pitchbook nexis university know lexisnexis academic include full text report magazine transcript business legal company executive contact ask contact marx science social science library yale university library prospect concourse allison gallaspy erin wachowicz schedule appointment subject business economics som training handout target list company career_services support yale career_development office limit som student som alumnus career resource som alumnus yale university office career strategy compensation data startup salary equity work skill salary comparison tool insider business insider searchable database last salary disclosure collect uscis curated company insider reporter resume registration account require instruction locate database preqin finance compensation employment late edition produce collaboration lead compensation specialist ferguson partner feature late trend statistic finance firm insight section preqin instruction locate preqin report national compensation survey bureau labor statistic national compensation survey establishment base survey comprehensive measure employer cost employee compensation include wage salary benefit compensation trend incidence employer sponsor benefit worker collect data produce estimate provision employer sponsor benefit plan</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>芝加哥大学 毕业生职业资源集.docx</t>
+        </is>
       </c>
       <c r="B53" t="inlineStr">
-        <is>
-          <t>芝加哥大学 毕业生职业资源集.docx</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
         <is>
           <t>New Graduate Career Development Resources Collection
 The Library is pleased to announce the opening of the new Graduate Career Development Resources Collection.  This new collection is a collaboration between UChicagoGRAD and the Library and is made possible through the generous support of Danette (Dani) Gentile Kauffman, who works with UChicagoGRAD to provide career workshops, and Diane Adams, a member of the Visiting Committee to the Library.
@@ -7826,22 +7670,19 @@
 For more on career resources available, see our Career Research guide.</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>graduate career growth material library opening graduate career growth material collection collection collaboration library support danette dani kauffman career workshop diane adam member committee twissbrooks question graduate career growth material collection career material career guide</t>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>graduate career_development resource collection library announce opening graduate career_development resource collection collection collaboration uchicagograd library possible generous support danette dani gentile kauffman job uchicagograd career training diane adam member visit committee library contact andrea twiss brook graduate career_development resource collection career resource career guide</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>芝加哥大学 资源指南.docx</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
-        <is>
-          <t>芝加哥大学 资源指南.docx</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
         <is>
           <t>Career Research
 Home
@@ -7946,22 +7787,19 @@
 Most public libraries offer some company databases, such as Hoovers or ReferenceUSA. Check with your local library to identify what's available to you.</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>career home material career subscribes source information company industry tool company interview industry graduate career growth material graduate career growth material collection collaboration library support danette dani gentile kauffman diane adam collection floor reading room regenstein library periodical newspaper sign collection collection catalog material career grad career exploration material graduate student university chicago career success career material college student job internship network alumnus online course technology software business skill résumé graduate science material school job employer dangelo law librarian specialist room socialfacebook pageinstagram economics industry industry library source overview industry level detail industry ibisworldthis link window scope material subscription state industry report netadvantagethis link window industry macro level material guide industry material guide industry industry business economics librarian company company basic company company web medium site report press release source information article trade journal newspaper source analysis picture situation key material link open window news database source search company executive news trade publication business source completethis link window profile company article trade journal source businessthis link window trade journal newspaper press release netadvantagethis link window coverage company material material company company information guide company information business economics librarian analyst report investment analyst report company information article company downside database refinitiv workspace guide workspace information report career book collection guide information duty education training pay outlook hundred occupation heading guidance occupation state catalog material book professor karen hfk publication date career guide student postdoc tenure doctor of philosophy job rule secret career right call isbn publication date book guide career career background schooltowork transition ascend position leadership interview career geography industry job type job job job skill job guide advice skill interview book job subject catalog job book killer job interview mcwhir call isbn publication date job dream cover letter winning interview job book collection tool technique strategy success punchy chapter youve graduation material guide subscription database wont graduation material article database site point finance yahoo finance offer access information company combine job listing company employee company registration material alumnus database material alumnus sep library library company hoover check library whats</t>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>career library resource career library subscribes company industry useful tool company invite interview industry interested job graduate career_development resource collection graduate career_development resource collection collaboration uchicagograd library possible generous support danette dani gentile kauffman diane adam collection locate second reading room regenstein library periodical report sign identify collection browse collection catalog uchicago resource career uchicago grad career exploration resource graduate student university chicago career success career advancement resource uchicago university student find employment internship network alumnus linkedin take free training add technology software business creative skill graduate library science resource find library university library job library researching legal employer angelo law librarian update subject specialist contact greg fleming treptow regenstein library room social facebook pageinstagram subject business economics industry industry overviews library give broad overview specific industry detail vary depend industry ibisworldthis broad scope resource subscription resume state specific industry report global netadvantagethis resume industry macro resource guide industry resource include guide specific industry conduct industry business economics librarian update aug company company basic company say company social medium annual report press release good say article trade article report excellent analysis picture company situation key secondary resource factivathis database company key executive find resume trade article business completethis include resume company worldwide article trade article proquest businessthis include trade article report press release global netadvantagethis international coverage company resource find resource company company guide company business economics librarian update oct deep dive analyst report investment analyst produce detailed report trade company hard dig article company report downside difficult specialized database call refinitiv workspace guide refinitiv workspace include report career book library collection career guide find career duty education training pay outlook job subject heading vocational guidance job united state library catalog find resource book list professor karen kelsky call isbn article definitive career guide grad student adjuncts post doc eager tenure turn ideal job unspoken rule secret start career right gorick call full text isbn article book guide early career professional underrepresented background navigate university job transition ascend position leadership base interview professional geography industry job job hunt find job land job skill develop academia job hunt guide advice communicate skill succeed interview hire book similar job hunt subject library catalog ultimate job hunt book write killer hide job succeed interview david mcwhir call full text isbn article craft perfect find job dream write great resume resume winning interview ultimate job hunt book dynamic collection tool technique strategy success short punchy chapter mean start apply uchicago graduation resource highlight guide subscription database win graduation free resource helpful article database alumni free useful start yahoo finance yahoo finance free trade company glassdoor glassdoor combine job listing company former employee give insight company sure consider free registration require library resource alumnus database alumnus electronic resource alumnus ask librarian update sep library library company databases hoover referenceusa check local library identify</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>麻省理工  httpslibguides.mit.edumajor.doc</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
-        <is>
-          <t>麻省理工  httpslibguides.mit.edumajor.doc</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
         <is>
           <t>Choosing a Major: Home
 Self-assessment tools
@@ -7994,9 +7832,9 @@
 barbaraw@mit.edu</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>home selfassessment tool myplan assessment tool personality test career interest inventory career skill profiler career assessment major material career assessment vice versa access myplan log careerbridge account orange bar top mouse material myplan register myplan account direction screen material occupation outlook guide welcome nation source career information profile hundred occupation environment pay profile job projection decade description guide home online description occupation skill ability work activity department departmental activity department faculty etc way link faculty example web faculty department guide subject taught mit guide database journal article subject background material manual contact information subject librarian department mit news mit news mit news site faculty question literature theater art szarkomitedu barbara aeronautics astronautics barbarawmitedu</t>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>major self assessment tool myplan several assessment tool include personality test career interest inventory career skill profiler career value assessment major include resource callsed major match career assessment potential major vice versa myplan log careerbridge account orange bar top mouse additional resource myplan myplan account follow direction screen internet resource job occupational outlook handbook welcome nation premier career resume feature resume job describe job environment pay resume include bls employment projection decade description handbook net detail description job include skill ability typical job activity potential department check departmental webpages highlight activity department faculty great potential major faculty find departmental guide faculty potential department write guide subject taught mit guide find database article article subject background material manual encyclopedias contact subject librarian department mit mit mit spotlight faculty mark szarko literature theater art write humanistic librarian szarko mit barbara williams aeronautics astronautics librarian barbaraw mit</t>
         </is>
       </c>
     </row>

</xml_diff>